<commit_message>
Gia tri thang du
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="91" customWidth="1" min="1" max="1"/>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>in-draft</t>
+          <t>done</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1189,12 +1189,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>19-08-2026</t>
+          <t>09-09-2026</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>- [ ] Nhân bản hoạt động - [ ]</t>
+          <t>Chắc hẳn anh em đã được nghe đâu đó đại loại rằng một nền kinh tế thực sự phát triển là một nền kinh tế tạo ra thật nhiều giá trị và phân phối chúng đi khắp nơi. Anh em nghe điều đó bất kể là anh em đang học ở đâu - Đông hay Tây, xưa hay na...</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1205,21 +1205,74 @@
       <c r="K9" t="inlineStr">
         <is>
           <t># Giá trị thặng dư
-## 2 cách đạt được thặng dư
-## 
-- [ ] Nhân bản hoạt động
-- [ ]</t>
+Chắc hẳn anh em đã được nghe đâu đó đại loại rằng một nền kinh tế thực sự phát triển là một nền kinh tế tạo ra thật nhiều giá trị và phân phối chúng đi khắp nơi. Anh em nghe điều đó bất kể là anh em đang học ở đâu - Đông hay Tây, xưa hay nay. Mức sống của một quốc gia phụ thuộc vào năng lực sản xuất hàng hóa và dịch vụ của quốc gia đó.[^1] Sản xuất vật chất là cơ sở của sự tồn tại và phát triển xã hội.[^2] Và rồi sau mỗi giai đoạn, mỗi thời kỳ, mỗi một sự đổi mới được hình thành, anh em bắt đầu nhìn lại và coi lại cách chúng áp dụng trong thời đại hiện tại. Và đây cũng là chủ đề mà Hải được nghe nhiều nhất từ thời đi học. 
+## Giá trị thặng dư là gì?
+Được rồi, trước khi đến với cách để đạt được thặng dư, hãy cùng làm rõ một số thứ. Đầu tiên là giá trị của hàng hóa:[^3]
+&gt; Lao động xã hội của người sản xuất hàng hóa kết tinh trong hàng hóa. 
+Trước hết, đó là do lao động tạo ra, và nó phải được xã hội chấp nhận. Nghĩa là bạn không thể tự ý đưa ra một con số cho nó, giá trị của nó là bao nhiêu và đổi được những gì phải là do xã hội thừa nhận. Bởi vì người sản xuất cũng cần phải trao đổi với người khác, nếu không, chúng sẽ không được gọi là hàng hóa.
+Tiếp đến là phần thặng dư. Trước hết hãy nhìn theo công thức lưu thông trong tư bản $T-H-T'$, thặng dư được gọi là:
+&gt; Phần dôi ra vượt sức lao động do người lao động tạo ra mà không được các nhà tư bản trả công. 
+Phần dôi ra đó được ký hiệu là $\Delta m = T - T'$ và được hình thành bằng việc biến hàng hóa (bao gồm sức lao động) thành trung gian để tạo ra tư bản lớn hơn thay cho việc coi tiền là trung gian để trao đổi hàng hóa như công thức lưu thông giản đơn $H-T-H$. Tất nhiên phần này có một chút sự khác biệt với cách nhìn kiểu của Mankiw: 
+&gt; Phần lợi ích mà người tham gia giao dịch nhận được từ chênh lệch giữa mức giá thực tế và mức giá 2 bên chấp nhận. 
+Phần thặng dư đó gồm sản xuất và tiêu dùng. Thặng dư tiêu dùng đến từ việc người mua sẵn sàng mua hàng với giá cao hơn nhưng lại được mua hàng với giá rẻ hơn họ nghĩ. Thặng dư sản xuất đến từ việc người bán sẵn sàng bán giá thấp hơn nhưng họ vẫn bán được với giá cao. Nếu họ không cảm thấy hời từ giao dịch, họ có quyền từ chối bán hoặc từ chối mua - không ai ép. Và vì có kha khá cách nhìn về thặng dư, trong bài viết này Hải sẽ dùng cách nhìn mà được nhiều bên chấp nhận nhất:
+&gt; Phần giá trị nhận được sau khi trừ đi cái giá để có được nó
+hay nói cách khác: Thặng dư = Giá trị nhận được - Chi phí bỏ ra 
+## 2 cách để đạt được thặng dư
+Cách thứ nhất đó chính là nhân bản hoạt động lên. Bạn làm tốt cái gì thì hãy làm cái đó nhiều hơn. Nếu 1 tiếng của bạn gấp được 10 origami, thì cách để tăng số lượng origami là tăng số giờ gấp chúng lên. Nếu sức của bạn 1 ngày chỉ cung cấp được 50 suất ăn, thì cách để tăng số lượng suất ăn phục vụ mỗi ngày là tuyển người về và chỉ họ cách làm. Cao tay hơn bạn cho mỗi người đúng ở mỗi khâu trong quy trình và truyển kết quả của mình cho người kế tiếp, bạn sẽ thấy số lượng origami và suất ăn đều tăng khủng khiếp. Từ một vài nếp gấp giấy, từ dọn bàn tới rửa bát, từ xới cơm cho tới múc canh - tốc độ của chúng đã nhanh hơn rất nhiều. Miễn là bạn thấy xứng đáng, hãy làm việc đó nhiều hơn hoặc tìm cách thuyết phục người khác làm việc đó với bạn. 
+Nhưng cách làm này có gì không ổn không? Bạn biết rằng quán ăn của bạn chỉ có tối đa 100 khách đến mỗi ngày. Vì vậy nếu bạn tuyển thêm nhiều người để phục vụ 200 suất ăn mỗi ngày, 100 phần ăn sẽ không có đầu ra - và chúng sẽ không được gọi là thặng dư theo bất cứ cách hiểu nào. Lúc này bạn hiểu rằng đó đã là giới hạn của cách nhân bản - nó đã không còn quan trọng như trước đây nữa. Bạn biết mình sẽ phải tìm cách để tăng lượt khách tới quán mỗi ngày nếu muốn tăng giá trị của bản thân. Có thể là đổi công thức, có thể là xây dựng thương hiệu để nhiều người biết đến hơn. 
+Nhìn chung nó là sự thay đổi, hoặc sự cải tổ. Đó là những phát minh, đó là những ý tưởng mới. Chúng được dùng để thay đổi hành vi hoặc thói quen giúp tăng giá trị chất lượng cuộc sống. Lúc này, việc tăng thặng dư không chỉ giới hạn ở việc cung cấp thêm suất ăn hay gấp origami; không chỉ giới hạn ở việc sản xuất thêm laptop hay điện thoại hay xe máy; hay tăng các nhu yếu phẩm, dụng cụ học tập và y tế hằng ngày. Bất kỳ thứ gì tạo ra giá trị cho xã hội hoặc làm giảm chi phí để giải quyết vấn đề đều làm tăng thặng dư. Và vì thế bạn cũng biết rằng việc làm giảm tắc đường cũng làm tăng thặng dư, việc giảm tải áp lực cho bệnh viện công giúp giảm thời gian khám bệnh cũng làm tăng giá trị thặng dư, việc làm giảm thời gian đi làm thủ tục hành chính cũng làm tăng thặng dư. Vì bạn biết thời gian cũng vừa là giá trị vừa là chi phí, việc cải tiến công nghệ giúp tăng trải nghiệm, giảm lag, giảm thời gian phản hồi, tăng băng thông kết nối dữ liệu cũng làm tăng thặng dư.   
+## Thặng dư trong thời kỳ bùng nổ thông tin
+Dữ liệu cũng là một loại hàng hóa đặc biệt. Nó là hàng hóa vì nó thỏa mãn 2 thuộc tính cơ bản của hàng hóa là giá trị (có thể đem ra trao đổi) và giá trị sử dụng nhằm phục vụ cho nhu cầu nào đó của con người. Nó đặc biệt ở chỗ chi phí để nhân bản chúng gần như bằng 0, bạn chỉ cần copy-paste là đủ. Và nó còn đặc biệt ở chỗ trong một số trường hợp, bạn không được phép nhân bản. Bạn có thể copy mã nguồn của Office và phân phối chúng cho nhiều người nhưng làm vậy sẽ gây thiệt hại cho Microsoft. Bạn cũng có thể lấy luồng truyền hình bóng đá và phát trực tiếp cho mọi người, nhưng làm vậy sẽ gây thiệt hại cho bên tổ chức giải đấu và bên mua bản quyền. Tại sao họ không cho phép mọi người copy-paste? Bởi vì họ cũng cần ăn cơm và uống nước như những người khác, bạn sẽ bị hạn chế hoặc dính tới pháp luật nếu tự ý nhân bản và phân phối chúng.    
+Để tăng thặng dư trong thời kỳ này, cách bạn có thể làm là đem công nghệ đi phục vụ cho tất cả ngành nghề. Bạn biết rằng dữ liệu giao thông trong một thời gian dài có thể giúp bạn làm giảm tắc đường theo cách này hoặc theo cách khác. Bạn biết rằng hình ảnh công trường được gửi đi và tạo báo cáo nhanh có thể giúp bạn quản lý dự án một cách hiệu quả. Bạn biết rằng thông tin ngày nay có thể nhanh chóng chảy tới bất kỳ đâu. Vì thế chúng có thể được dùng như những kênh môi giới, những trang niêm yết sản phẩm, những "mặt bằng" để giới thiệu và quảng bá thương hiệu. Và bạn cũng có thể làm SaaS để giải quyết các công việc lặp lại - và sự nhân bản cách giải quyết vấn đề này là hoàn toàn hợp pháp. 
+[^1]: Principles of Economics - N. Mankiw
+[^2]: Triết học Mác – Lênin
+[^3]: Kinh tế chính trị Mác - Lênin</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>&lt;h1 id="gia-tri-thang-du"&gt;Giá trị thặng dư&lt;/h1&gt;
-&lt;h2 id="2-cach-at-uoc-thang-du"&gt;2 cách đạt được thặng dư&lt;/h2&gt;
-&lt;h2 id="_1"&gt;&lt;/h2&gt;
-&lt;ul class="task-list"&gt;
-&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Nhân bản hoạt động&lt;/li&gt;
-&lt;li&gt;[ ]&lt;/li&gt;
-&lt;/ul&gt;</t>
+&lt;p&gt;Chắc hẳn anh em đã được nghe đâu đó đại loại rằng một nền kinh tế thực sự phát triển là một nền kinh tế tạo ra thật nhiều giá trị và phân phối chúng đi khắp nơi. Anh em nghe điều đó bất kể là anh em đang học ở đâu - Đông hay Tây, xưa hay nay. Mức sống của một quốc gia phụ thuộc vào năng lực sản xuất hàng hóa và dịch vụ của quốc gia đó.&lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt; Sản xuất vật chất là cơ sở của sự tồn tại và phát triển xã hội.&lt;sup id="fnref:2"&gt;&lt;a class="footnote-ref" href="#fn:2"&gt;2&lt;/a&gt;&lt;/sup&gt; Và rồi sau mỗi giai đoạn, mỗi thời kỳ, mỗi một sự đổi mới được hình thành, anh em bắt đầu nhìn lại và coi lại cách chúng áp dụng trong thời đại hiện tại. Và đây cũng là chủ đề mà Hải được nghe nhiều nhất từ thời đi học. &lt;/p&gt;
+&lt;h2 id="gia-tri-thang-du-la-gi"&gt;Giá trị thặng dư là gì?&lt;/h2&gt;
+&lt;p&gt;Được rồi, trước khi đến với cách để đạt được thặng dư, hãy cùng làm rõ một số thứ. Đầu tiên là giá trị của hàng hóa:&lt;sup id="fnref:3"&gt;&lt;a class="footnote-ref" href="#fn:3"&gt;3&lt;/a&gt;&lt;/sup&gt;&lt;/p&gt;
+&lt;blockquote&gt;
+&lt;p&gt;Lao động xã hội của người sản xuất hàng hóa kết tinh trong hàng hóa. &lt;/p&gt;
+&lt;/blockquote&gt;
+&lt;p&gt;Trước hết, đó là do lao động tạo ra, và nó phải được xã hội chấp nhận. Nghĩa là bạn không thể tự ý đưa ra một con số cho nó, giá trị của nó là bao nhiêu và đổi được những gì phải là do xã hội thừa nhận. Bởi vì người sản xuất cũng cần phải trao đổi với người khác, nếu không, chúng sẽ không được gọi là hàng hóa.&lt;/p&gt;
+&lt;p&gt;Tiếp đến là phần thặng dư. Trước hết hãy nhìn theo công thức lưu thông trong tư bản &lt;span class="arithmatex"&gt;\(T-H-T'\)&lt;/span&gt;, thặng dư được gọi là:&lt;/p&gt;
+&lt;blockquote&gt;
+&lt;p&gt;Phần dôi ra vượt sức lao động do người lao động tạo ra mà không được các nhà tư bản trả công. &lt;/p&gt;
+&lt;/blockquote&gt;
+&lt;p&gt;Phần dôi ra đó được ký hiệu là &lt;span class="arithmatex"&gt;\(\Delta m = T - T'\)&lt;/span&gt; và được hình thành bằng việc biến hàng hóa (bao gồm sức lao động) thành trung gian để tạo ra tư bản lớn hơn thay cho việc coi tiền là trung gian để trao đổi hàng hóa như công thức lưu thông giản đơn &lt;span class="arithmatex"&gt;\(H-T-H\)&lt;/span&gt;. Tất nhiên phần này có một chút sự khác biệt với cách nhìn kiểu của Mankiw: &lt;/p&gt;
+&lt;blockquote&gt;
+&lt;p&gt;Phần lợi ích mà người tham gia giao dịch nhận được từ chênh lệch giữa mức giá thực tế và mức giá 2 bên chấp nhận. &lt;/p&gt;
+&lt;/blockquote&gt;
+&lt;p&gt;Phần thặng dư đó gồm sản xuất và tiêu dùng. Thặng dư tiêu dùng đến từ việc người mua sẵn sàng mua hàng với giá cao hơn nhưng lại được mua hàng với giá rẻ hơn họ nghĩ. Thặng dư sản xuất đến từ việc người bán sẵn sàng bán giá thấp hơn nhưng họ vẫn bán được với giá cao. Nếu họ không cảm thấy hời từ giao dịch, họ có quyền từ chối bán hoặc từ chối mua - không ai ép. Và vì có kha khá cách nhìn về thặng dư, trong bài viết này Hải sẽ dùng cách nhìn mà được nhiều bên chấp nhận nhất:&lt;/p&gt;
+&lt;blockquote&gt;
+&lt;p&gt;Phần giá trị nhận được sau khi trừ đi cái giá để có được nó&lt;/p&gt;
+&lt;/blockquote&gt;
+&lt;p&gt;hay nói cách khác: Thặng dư = Giá trị nhận được - Chi phí bỏ ra &lt;/p&gt;
+&lt;h2 id="2-cach-e-at-uoc-thang-du"&gt;2 cách để đạt được thặng dư&lt;/h2&gt;
+&lt;p&gt;Cách thứ nhất đó chính là nhân bản hoạt động lên. Bạn làm tốt cái gì thì hãy làm cái đó nhiều hơn. Nếu 1 tiếng của bạn gấp được 10 origami, thì cách để tăng số lượng origami là tăng số giờ gấp chúng lên. Nếu sức của bạn 1 ngày chỉ cung cấp được 50 suất ăn, thì cách để tăng số lượng suất ăn phục vụ mỗi ngày là tuyển người về và chỉ họ cách làm. Cao tay hơn bạn cho mỗi người đúng ở mỗi khâu trong quy trình và truyển kết quả của mình cho người kế tiếp, bạn sẽ thấy số lượng origami và suất ăn đều tăng khủng khiếp. Từ một vài nếp gấp giấy, từ dọn bàn tới rửa bát, từ xới cơm cho tới múc canh - tốc độ của chúng đã nhanh hơn rất nhiều. Miễn là bạn thấy xứng đáng, hãy làm việc đó nhiều hơn hoặc tìm cách thuyết phục người khác làm việc đó với bạn. &lt;/p&gt;
+&lt;p&gt;Nhưng cách làm này có gì không ổn không? Bạn biết rằng quán ăn của bạn chỉ có tối đa 100 khách đến mỗi ngày. Vì vậy nếu bạn tuyển thêm nhiều người để phục vụ 200 suất ăn mỗi ngày, 100 phần ăn sẽ không có đầu ra - và chúng sẽ không được gọi là thặng dư theo bất cứ cách hiểu nào. Lúc này bạn hiểu rằng đó đã là giới hạn của cách nhân bản - nó đã không còn quan trọng như trước đây nữa. Bạn biết mình sẽ phải tìm cách để tăng lượt khách tới quán mỗi ngày nếu muốn tăng giá trị của bản thân. Có thể là đổi công thức, có thể là xây dựng thương hiệu để nhiều người biết đến hơn. &lt;/p&gt;
+&lt;p&gt;Nhìn chung nó là sự thay đổi, hoặc sự cải tổ. Đó là những phát minh, đó là những ý tưởng mới. Chúng được dùng để thay đổi hành vi hoặc thói quen giúp tăng giá trị chất lượng cuộc sống. Lúc này, việc tăng thặng dư không chỉ giới hạn ở việc cung cấp thêm suất ăn hay gấp origami; không chỉ giới hạn ở việc sản xuất thêm laptop hay điện thoại hay xe máy; hay tăng các nhu yếu phẩm, dụng cụ học tập và y tế hằng ngày. Bất kỳ thứ gì tạo ra giá trị cho xã hội hoặc làm giảm chi phí để giải quyết vấn đề đều làm tăng thặng dư. Và vì thế bạn cũng biết rằng việc làm giảm tắc đường cũng làm tăng thặng dư, việc giảm tải áp lực cho bệnh viện công giúp giảm thời gian khám bệnh cũng làm tăng giá trị thặng dư, việc làm giảm thời gian đi làm thủ tục hành chính cũng làm tăng thặng dư. Vì bạn biết thời gian cũng vừa là giá trị vừa là chi phí, việc cải tiến công nghệ giúp tăng trải nghiệm, giảm lag, giảm thời gian phản hồi, tăng băng thông kết nối dữ liệu cũng làm tăng thặng dư.   &lt;/p&gt;
+&lt;h2 id="thang-du-trong-thoi-ky-bung-no-thong-tin"&gt;Thặng dư trong thời kỳ bùng nổ thông tin&lt;/h2&gt;
+&lt;p&gt;Dữ liệu cũng là một loại hàng hóa đặc biệt. Nó là hàng hóa vì nó thỏa mãn 2 thuộc tính cơ bản của hàng hóa là giá trị (có thể đem ra trao đổi) và giá trị sử dụng nhằm phục vụ cho nhu cầu nào đó của con người. Nó đặc biệt ở chỗ chi phí để nhân bản chúng gần như bằng 0, bạn chỉ cần copy-paste là đủ. Và nó còn đặc biệt ở chỗ trong một số trường hợp, bạn không được phép nhân bản. Bạn có thể copy mã nguồn của Office và phân phối chúng cho nhiều người nhưng làm vậy sẽ gây thiệt hại cho Microsoft. Bạn cũng có thể lấy luồng truyền hình bóng đá và phát trực tiếp cho mọi người, nhưng làm vậy sẽ gây thiệt hại cho bên tổ chức giải đấu và bên mua bản quyền. Tại sao họ không cho phép mọi người copy-paste? Bởi vì họ cũng cần ăn cơm và uống nước như những người khác, bạn sẽ bị hạn chế hoặc dính tới pháp luật nếu tự ý nhân bản và phân phối chúng.    &lt;/p&gt;
+&lt;p&gt;Để tăng thặng dư trong thời kỳ này, cách bạn có thể làm là đem công nghệ đi phục vụ cho tất cả ngành nghề. Bạn biết rằng dữ liệu giao thông trong một thời gian dài có thể giúp bạn làm giảm tắc đường theo cách này hoặc theo cách khác. Bạn biết rằng hình ảnh công trường được gửi đi và tạo báo cáo nhanh có thể giúp bạn quản lý dự án một cách hiệu quả. Bạn biết rằng thông tin ngày nay có thể nhanh chóng chảy tới bất kỳ đâu. Vì thế chúng có thể được dùng như những kênh môi giới, những trang niêm yết sản phẩm, những "mặt bằng" để giới thiệu và quảng bá thương hiệu. Và bạn cũng có thể làm SaaS để giải quyết các công việc lặp lại - và sự nhân bản cách giải quyết vấn đề này là hoàn toàn hợp pháp. &lt;/p&gt;
+&lt;div class="footnote"&gt;
+&lt;hr /&gt;
+&lt;ol&gt;
+&lt;li id="fn:1"&gt;
+&lt;p&gt;Principles of Economics - N. Mankiw&amp;#160;&lt;a class="footnote-backref" href="#fnref:1" title="Jump back to footnote 1 in the text"&gt;&amp;#8617;&lt;/a&gt;&lt;/p&gt;
+&lt;/li&gt;
+&lt;li id="fn:2"&gt;
+&lt;p&gt;Triết học Mác – Lênin&amp;#160;&lt;a class="footnote-backref" href="#fnref:2" title="Jump back to footnote 2 in the text"&gt;&amp;#8617;&lt;/a&gt;&lt;/p&gt;
+&lt;/li&gt;
+&lt;li id="fn:3"&gt;
+&lt;p&gt;Kinh tế chính trị Mác - Lênin&amp;#160;&lt;a class="footnote-backref" href="#fnref:3" title="Jump back to footnote 3 in the text"&gt;&amp;#8617;&lt;/a&gt;&lt;/p&gt;
+&lt;/li&gt;
+&lt;/ol&gt;
+&lt;/div&gt;</t>
         </is>
       </c>
     </row>
@@ -1500,47 +1553,131 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người</t>
+          <t>Gửi Hải tuổi 35</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ky-nang-cot-loi-de-thanh-cong---danh-cho-tat-ca-moi-nguoi</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
+          <t>gui-hai-tuoi-35</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Quý Hải Ng</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
+          <t>06-09-2026</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>06-09-2026</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>data\blogs\Gửi Hải tuổi 35.md</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Học cách kể chuyện</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>hoc-cach-ke-chuyen</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>04-09-2026</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>04-09-2026</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>data\blogs\Học cách kể chuyện.md</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t># Học cách kể chuyện</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>&lt;h1 id="hoc-cach-ke-chuyen"&gt;Học cách kể chuyện&lt;/h1&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ky-nang-cot-loi-de-thanh-cong---danh-cho-tat-ca-moi-nguoi</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
           <t>23-07-2026</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Khi đọc sách self-help hay tham gia bất kỳ hội thảo khóa học nào, anh em có thể đã nghe que hàng trăm đức tính để trở nên thành công, thành đạt, thịnh vượng. Nào là cần cù, chịu thương, chịu khó. Nào là thông minh, sáng tạo, tư duy mở. Nào...</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>data\blogs\Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người.md</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t># Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người
 Khi đọc sách self-help hay tham gia bất kỳ hội thảo khóa học nào, anh em có thể đã nghe que hàng trăm đức tính để trở nên thành công, thành đạt, thịnh vượng. Nào là cần cù, chịu thương, chịu khó. Nào là thông minh, sáng tạo, tư duy mở. Nào là hình thành thói quen tốt, kỹ năng tự học, tính kỷ luật. Và hàng loạt yếu tố khác như tinh thần cầu tiến, sự tập trung, quản lý thời gian, dám chấp nhận rủi ro,...
@@ -1570,7 +1707,7 @@
 Là một người viết, thành công đối với Hải là thuyết phục được người khác đọc hết bài viết của mình. Vì thế Hải sẵn sàng đón nhận mọi ý kiến, bất kể là khen hay chê. Khi ai đó khen Hải, Hải sẽ kiểu: "Ok, cảm ơn bạn nhé, tầm ngày này tuần sau Hải sẽ lại ra bài mới, nhớ đón đọc nha!". Còn khi ai đó chê bai, Hải sẽ biết rằng : "Được rồi, có điều gì đó cần thay đổi!".</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>&lt;h1 id="ky-nang-cot-loi-e-thanh-cong-danh-cho-tat-ca-moi-nguoi"&gt;Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người&lt;/h1&gt;
 &lt;p&gt;Khi đọc sách self-help hay tham gia bất kỳ hội thảo khóa học nào, anh em có thể đã nghe que hàng trăm đức tính để trở nên thành công, thành đạt, thịnh vượng. Nào là cần cù, chịu thương, chịu khó. Nào là thông minh, sáng tạo, tư duy mở. Nào là hình thành thói quen tốt, kỹ năng tự học, tính kỷ luật. Và hàng loạt yếu tố khác như tinh thần cầu tiến, sự tập trung, quản lý thời gian, dám chấp nhận rủi ro,...&lt;/p&gt;
@@ -1605,54 +1742,54 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Tạm biệt Wordpress - Vì sao mình chuyển sang content engine thay vì hệ thống back-end CMS</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>tam-biet-wordpress---vi-sao-minh-chuyen-sang-content-engine-thay-vi-he-thong-back-end-cms</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Công nghệ</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
         <is>
           <t>web, tech, wp</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>24-05-2026</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>Từng nghiên cứu Wordpress 5 năm và thực chiến 2 năm, cũng xuất bản được kha khá blog. Bản thân Hải thấy Wordpress đem lại rất nhiều trải nghiệm thú vị nơi blogger chỉ cần quan tâm tới tuyến nội dung và quản trị thay vì đầu tư nhiều thời gia...</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>data\blogs\Lựa chọn content engine thay vì hệ thống back-end.md</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t># Tạm biệt Wordpress - Vì sao mình chuyển sang content engine thay vì hệ thống back-end CMS
 Từng nghiên cứu Wordpress 5 năm và thực chiến 2 năm, cũng xuất bản được kha khá blog. Bản thân Hải thấy Wordpress đem lại rất nhiều trải nghiệm thú vị nơi blogger chỉ cần quan tâm tới tuyến nội dung và quản trị thay vì đầu tư nhiều thời gian cho code, web, database, ...  Wordpress mang lại rất nhiều giá trị cho Hải. Với những anh em đã từng đau đầu hoặc đã trả giá vì hệ thống quản lý phân quyền, quản lý media, danh mục, bình luận,... thì sẽ hiểu rõ Wordpress có thể giúp anh em tiết kiệm cả tỷ đồng. Và trên hết nó là mã nguồn mở, miễn phí.
@@ -1705,7 +1842,7 @@
 Với 1 blogger, thay vì phải duy trì một CMS phức tạp với hàng loạt plugin, tài khoản quản trị, cơ sở dữ liệu và các bản vá bảo mật định kỳ, việc thuần tập trung vào sản xuất nội dung mới là ưu tiền hàng đầu. Toàn bộ quá trình còn lại được tự động hóa thông qua content engine để chuyển đổi cắt văn bản và nhúng vào các tập tin định dạng.</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-biet-wordpress-vi-sao-minh-chuyen-sang-content-engine-thay-vi-he-thong-back-end-cms"&gt;Tạm biệt Wordpress - Vì sao mình chuyển sang content engine thay vì hệ thống back-end CMS&lt;/h1&gt;
 &lt;p&gt;Từng nghiên cứu Wordpress 5 năm và thực chiến 2 năm, cũng xuất bản được kha khá blog. Bản thân Hải thấy Wordpress đem lại rất nhiều trải nghiệm thú vị nơi blogger chỉ cần quan tâm tới tuyến nội dung và quản trị thay vì đầu tư nhiều thời gian cho code, web, database, ...  Wordpress mang lại rất nhiều giá trị cho Hải. Với những anh em đã từng đau đầu hoặc đã trả giá vì hệ thống quản lý phân quyền, quản lý media, danh mục, bình luận,... thì sẽ hiểu rõ Wordpress có thể giúp anh em tiết kiệm cả tỷ đồng. Và trên hết nó là mã nguồn mở, miễn phí.&lt;/p&gt;
@@ -1759,42 +1896,42 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Markdown_Example</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>markdownexample</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>21-07-2026</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>Example paragraph</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>data\blogs\Markdown_Example.md</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t># This is heading 1 for title
 Example paragraph
@@ -1843,7 +1980,7 @@
 [^1]: This is the footnote.</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>&lt;h1 id="this-is-heading-1-for-title"&gt;This is heading 1 for title&lt;/h1&gt;
 &lt;p&gt;Example paragraph&lt;/p&gt;
@@ -1902,50 +2039,50 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Một cách kiếm tiền không mới nhưng luôn mới mẻ</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>mot-cach-kiem-tien-khong-moi-nhung-luon-moi-me</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>22-07-2026</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>Năm 1889, vào thời điểm chưa có Google Map và thị trường xe hơi ở Pháp chưa có tới 3000 chiếc, 2 anh em Andre và Edouard đã nhận thấy tiềm năng từ việc giúp cho tài xế có được hành trình thú vị nhằm thúc đẩy doanh thu từ việc bán xe và lốp....</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>data\blogs\Một cách kiếm tiền không mới nhưng luôn mới mẻ.md</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t># Một cách kiếm tiền không mới nhưng luôn mới mẻ
 Năm 1889, vào thời điểm chưa có Google Map và thị trường xe hơi ở Pháp chưa có tới 3000 chiếc, 2 anh em Andre và Edouard đã nhận thấy tiềm năng từ việc giúp cho tài xế có được hành trình thú vị nhằm thúc đẩy doanh thu từ việc bán xe và lốp. Vì thế họ tạo ra cẩm nang hướng dẫn cho khách du lịch. Từ việc đổ xăng ở đâu, thay lốp ở đâu, ăn uống ở đâu, nghỉ ngơi ở đâu. Trong hơn 2 thập kỷ đầu, cuốn cẩm nang có chứa danh sách khách sạn, nhà hàng ở Paris được chia theo danh mục cụ thể hoàn toàn miễn phí. Tới năm 1920, cuốn cẩm nang đó được bán với giá 7 franc. Nếu quy đổi theo lạm phát, cuốn cẩm nang đó có giá khoảng 32.000 VND vào năm 2026. Và đó là khởi đầu của giải thưởng Sao Michelin ngày nay. [^1]
@@ -1989,7 +2126,7 @@
 [^3]: [Content Engine - Vì sao các cá nhân và doanh nghiệp nên quan tâm?](https://haicogihay.com/blog/content-engine---vi-sao-cac-ca-nhan-va-doanh-nghiep-nen-quan-tam)</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>&lt;h1 id="mot-cach-kiem-tien-khong-moi-nhung-luon-moi-me"&gt;Một cách kiếm tiền không mới nhưng luôn mới mẻ&lt;/h1&gt;
 &lt;p&gt;Năm 1889, vào thời điểm chưa có Google Map và thị trường xe hơi ở Pháp chưa có tới 3000 chiếc, 2 anh em Andre và Edouard đã nhận thấy tiềm năng từ việc giúp cho tài xế có được hành trình thú vị nhằm thúc đẩy doanh thu từ việc bán xe và lốp. Vì thế họ tạo ra cẩm nang hướng dẫn cho khách du lịch. Từ việc đổ xăng ở đâu, thay lốp ở đâu, ăn uống ở đâu, nghỉ ngơi ở đâu. Trong hơn 2 thập kỷ đầu, cuốn cẩm nang có chứa danh sách khách sạn, nhà hàng ở Paris được chia theo danh mục cụ thể hoàn toàn miễn phí. Tới năm 1920, cuốn cẩm nang đó được bán với giá 7 franc. Nếu quy đổi theo lạm phát, cuốn cẩm nang đó có giá khoảng 32.000 VND vào năm 2026. Và đó là khởi đầu của giải thưởng Sao Michelin ngày nay. &lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt;&lt;/p&gt;
@@ -2047,54 +2184,54 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Một số nơi chứa ý tưởng mới</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>mot-so-noi-chua-y-tuong-moi</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Tư duy</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Quy Hai Ng</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>26-08-2026</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>Hải đoán là mỗi một ngày khi anh em lướt feed và đọc tin tức, sẽ có khoảng vài chục đến vài trăm lần anh em bắt gặp các cụm từ `đổi mới`, `sáng tạo`, `start-up`. Nói đúng ra, nếu không có ý tưởng mới, chúng ta sẽ mãi rơi vào vòng lặp bảo th...</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>data\blogs\Một số nơi chứa ý tưởng mới.md</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t># Một số nơi chứa ý tưởng mới
 Hải đoán là mỗi một ngày khi anh em lướt feed và đọc tin tức, sẽ có khoảng vài chục đến vài trăm lần anh em bắt gặp các cụm từ `đổi mới`, `sáng tạo`, `start-up`. Nói đúng ra, nếu không có ý tưởng mới, chúng ta sẽ mãi rơi vào vòng lặp bảo thủ trong khi mọi thứ xung quanh đều đang thay đổi. Điều này không chỉ đúng với các cá nhân hay SME, mà còn đúng với cả các tập đoàn lớn.
@@ -2122,7 +2259,7 @@
 [^1]: [Một cách kiếm tiền không mới nhưng luôn mới mẻ](https://haicogihay.com/blog/mot-cach-kiem-tien-khong-moi-nhung-luon-moi-me)</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>&lt;h1 id="mot-so-noi-chua-y-tuong-moi"&gt;Một số nơi chứa ý tưởng mới&lt;/h1&gt;
 &lt;p&gt;Hải đoán là mỗi một ngày khi anh em lướt feed và đọc tin tức, sẽ có khoảng vài chục đến vài trăm lần anh em bắt gặp các cụm từ &lt;code&gt;đổi mới&lt;/code&gt;, &lt;code&gt;sáng tạo&lt;/code&gt;, &lt;code&gt;start-up&lt;/code&gt;. Nói đúng ra, nếu không có ý tưởng mới, chúng ta sẽ mãi rơi vào vòng lặp bảo thủ trong khi mọi thứ xung quanh đều đang thay đổi. Điều này không chỉ đúng với các cá nhân hay SME, mà còn đúng với cả các tập đoàn lớn.&lt;/p&gt;
@@ -2163,58 +2300,58 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Một vài góc nhìn nhìn từ thí ngiệm "Vũ trụ 25"</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>mot-vai-goc-nhin-nhin-tu-thi-ngiem-vu-tru-25</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>universe25, tâm lý, thiên đường của loài chuột</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Vào ngày 22 tháng 6 năm 1972, nhà khoa học John Calhoun đã thực hiệm 1 thí nghiệm để trả lời cho câu hỏi: "Nếu loài sinh vật được sống trong thiên đường không lo cạnh tranh về thức ăn, về chỗ ở, liệu chúng có thể duy trì và phát triển mãi m...</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>data\blogs\Một vài góc nhìn từ thí nghiệm vũ trụ 25.md</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t># Một vài góc nhìn từ thí nghiệm "Vũ trụ 25"
 Vào ngày 22 tháng 6 năm 1972, nhà khoa học John Calhoun đã thực hiệm 1 thí nghiệm để trả lời cho câu hỏi: "Nếu loài sinh vật được sống trong thiên đường không lo cạnh tranh về thức ăn, về chỗ ở, liệu chúng có thể duy trì và phát triển mãi mãi hay không?  [^1] Ông chọn ra 4 cặp chuột khỏe mạnh đã được sàng lọc kỹ càng về sức khỏe. Sau đó, đưa chúng vào môi trường 3m x 4.3m, chia thành 16 tháp, tạo được thành 256 hộp tổ, mỗi hộp có sức chứa đủ cho 15 chuột cùng ở - thiên đường đủ để chứa 4000 con chuột. Thức ăn, nước đều được cung cấp đầy đủ, nhiệt độ môi trường được kiểm soát, chất thải của chúng cũng được dọn dẹp, và hoàn toàn không có thú săn mồi. 
@@ -2255,7 +2392,7 @@
 [^4]: [Sáng Thế Ký 3 - Người Nam và Người Nữ Phạm Tội](https://www.bible.com/vi/bible/1638/GEN.3.KTHD)</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>&lt;h1 id="mot-vai-goc-nhin-tu-thi-nghiem-vu-tru-25"&gt;Một vài góc nhìn từ thí nghiệm "Vũ trụ 25"&lt;/h1&gt;
 &lt;p&gt;Vào ngày 22 tháng 6 năm 1972, nhà khoa học John Calhoun đã thực hiệm 1 thí nghiệm để trả lời cho câu hỏi: "Nếu loài sinh vật được sống trong thiên đường không lo cạnh tranh về thức ăn, về chỗ ở, liệu chúng có thể duy trì và phát triển mãi mãi hay không?  &lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt; Ông chọn ra 4 cặp chuột khỏe mạnh đã được sàng lọc kỹ càng về sức khỏe. Sau đó, đưa chúng vào môi trường 3m x 4.3m, chia thành 16 tháp, tạo được thành 256 hộp tổ, mỗi hộp có sức chứa đủ cho 15 chuột cùng ở - thiên đường đủ để chứa 4000 con chuột. Thức ăn, nước đều được cung cấp đầy đủ, nhiệt độ môi trường được kiểm soát, chất thải của chúng cũng được dọn dẹp, và hoàn toàn không có thú săn mồi. &lt;/p&gt;
@@ -2314,50 +2451,50 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Nói về bán hàng</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>noi-ve-ban-hang</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
         <is>
           <t>26-07-2026</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>27-07-2026</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>Dạy con làm giàu hay cha giàu cha nghèo là bộ sách cực kỳ nổi tiếng làm nên tên tuổi và thưởng hiệu của tác giả Robert Kiyosaki. Dù có nhiều tranh cãi, nhưng đây vẫn là bộ sách có doanh số bán rất khủng khiếp: Hơn 32 triệu bản, dịch sang 51...</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>data\blogs\Nói về bán hàng.md</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t># Nói về bán hàng
 Dạy con làm giàu hay cha giàu cha nghèo là bộ sách cực kỳ nổi tiếng làm nên tên tuổi và thưởng hiệu của tác giả Robert Kiyosaki. Dù có nhiều tranh cãi, nhưng đây vẫn là bộ sách có doanh số bán rất khủng khiếp: Hơn 32 triệu bản, dịch sang 51 thứ tiếng và xuất hiện ở 109 quốc gia. Robert Kiyosaki có lần chia sẻ về câu chuyện hỏi người cha nuôi của mình tên Tommy cách để giàu như cha ông: 
@@ -2379,7 +2516,7 @@
 - [ ] Kỹ năng</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>&lt;h1 id="noi-ve-ban-hang"&gt;Nói về bán hàng&lt;/h1&gt;
 &lt;p&gt;Dạy con làm giàu hay cha giàu cha nghèo là bộ sách cực kỳ nổi tiếng làm nên tên tuổi và thưởng hiệu của tác giả Robert Kiyosaki. Dù có nhiều tranh cãi, nhưng đây vẫn là bộ sách có doanh số bán rất khủng khiếp: Hơn 32 triệu bản, dịch sang 51 thứ tiếng và xuất hiện ở 109 quốc gia. Robert Kiyosaki có lần chia sẻ về câu chuyện hỏi người cha nuôi của mình tên Tommy cách để giàu như cha ông: &lt;/p&gt;
@@ -2408,54 +2545,54 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Sách self-help có thật sự hữu ích?</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>sach-self-help-co-that-su-huu-ich</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
         <is>
           <t>10-06-2026</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>12-06-2026</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>Sách Self-help có thể hiểu nôm na là cuốn sách tự phát triển bản thân. Chúng đồng hành với các độc giả thông qua việc đề cập đến các phương pháp, giải pháp để đi đến thành công, hạnh phúc hay chân - thiện - mĩ. Những cuốn sách đó thường có...</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>data\blogs\Sách self-help có thật sự hữu ích.md</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t># Sách self-help có thật sự hữu ích?
 Sách Self-help có thể hiểu nôm na là cuốn sách tự phát triển bản thân. Chúng đồng hành với các độc giả thông qua việc đề cập đến các phương pháp, giải pháp để đi đến thành công, hạnh phúc hay chân - thiện - mĩ. Những cuốn sách đó thường có đặc điểm chung là bán chạy bởi dễ đọc - dễ hiểu nếu so với những cuốn giáo trình khô khan. Tiêu biểu những cuốn điển hình mà anh em có lẽ đã quá quen thuộc là Đắc nhân tâm, Những kẻ xuất chúng, Nghĩ giàu làm giàu, 7 thói quen để thành đạt, Atomic Habit… 
@@ -2482,7 +2619,7 @@
 Một lần nữa, Hải muốn nhấn mạnh rằng: “Tri thức không chỉ phát triển nhờ sự đồng thuận tuyệt đối, mà nhờ những cuộc đối thoại tử tế. Vì vậy, mong anh em đọc bài viết như một góc nhìn để suy ngẫm, thay vì một kết luận cuối cùng. Mọi quan điểm ít nhiều đều mang dấu vết của trải nghiệm cá nhân. Mục đích của mỗi bài viết không phải là để ai đúng tuyệt đối, mà là liệu chúng ta có thể cùng nhau suy nghĩ sâu hơn sau mỗi bài viết hay không? Vì vậy, hãy đọc với tinh thần cởi mở và phản biện hoặc góp ý khi anh em có suy nghĩ khác nha!”.</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>&lt;h1 id="sach-self-help-co-that-su-huu-ich"&gt;Sách self-help có thật sự hữu ích?&lt;/h1&gt;
 &lt;p&gt;Sách Self-help có thể hiểu nôm na là cuốn sách tự phát triển bản thân. Chúng đồng hành với các độc giả thông qua việc đề cập đến các phương pháp, giải pháp để đi đến thành công, hạnh phúc hay chân - thiện - mĩ. Những cuốn sách đó thường có đặc điểm chung là bán chạy bởi dễ đọc - dễ hiểu nếu so với những cuốn giáo trình khô khan. Tiêu biểu những cuốn điển hình mà anh em có lẽ đã quá quen thuộc là Đắc nhân tâm, Những kẻ xuất chúng, Nghĩ giàu làm giàu, 7 thói quen để thành đạt, Atomic Habit… &lt;/p&gt;
@@ -2510,92 +2647,92 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Thử thay đổi cách đặt câu hỏi</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>thu-thay-doi-cach-dat-cau-hoi</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
         <is>
           <t>09-07-2026</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr">
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
         <is>
           <t>data\blogs\Thử thay đổi cách đặt câu hỏi.md</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Thử thay đổi góc nhìn</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>thu-thay-doi-goc-nhin</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
         <is>
           <t>09-07-2026</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>Một anh tài xế ở một nước phương Tây nào đó làm việc 11 tiếng mỗi ngày. Anh ta thường xuyên sử dụng đồ hộp, mì gói và nước tăng lực - thứ mà người Việt hay gọi là combo chạy thận. Anh ta có một mức thu nhập đủ để lo cho bản thân và để dành....</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>data\blogs\Thử thay đổi góc nhìn.md</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t># Thử thay đổi góc nhìn
 Một anh tài xế ở một nước phương Tây nào đó làm việc 11 tiếng mỗi ngày. Anh ta thường xuyên sử dụng đồ hộp, mì gói và nước tăng lực - thứ mà người Việt hay gọi là combo chạy thận. Anh ta có một mức thu nhập đủ để lo cho bản thân và để dành. Anh ta luôn tự hào mình làm việc chăm chỉ. Cho tới một ngày, một sự cố ập đến, anh ta bị bệnh nặng và phải nhập viện. Sau gần 3 tháng điều trị, anh ta cũng đã khỏi bệnh. Vì không có bảo hiểm, tổng chi phí cho hóa đơn dài hơn 100 trang gồm tiền giường, tiền thuốc, tiền mổ và loạt chi phí khác đã chạm ngưỡng 1 triệu đô. Và tất nhiên, số tiền anh ta dành giụm rất nhỏ khi so với chi phí điều trị. Người từng tự đắc rằng mình không bao giờ nợ ai bất kỳ điều gì trên đời này cuối cùng lại nhận món nợ 1 triệu đô theo một cách mà không ai ngờ tới - viện phí.
@@ -2603,7 +2740,7 @@
 ## Thật ra tất cả mọi thứ còn tồn tại là vì còn nợ</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>&lt;h1 id="thu-thay-oi-goc-nhin"&gt;Thử thay đổi góc nhìn&lt;/h1&gt;
 &lt;p&gt;Một anh tài xế ở một nước phương Tây nào đó làm việc 11 tiếng mỗi ngày. Anh ta thường xuyên sử dụng đồ hộp, mì gói và nước tăng lực - thứ mà người Việt hay gọi là combo chạy thận. Anh ta có một mức thu nhập đủ để lo cho bản thân và để dành. Anh ta luôn tự hào mình làm việc chăm chỉ. Cho tới một ngày, một sự cố ập đến, anh ta bị bệnh nặng và phải nhập viện. Sau gần 3 tháng điều trị, anh ta cũng đã khỏi bệnh. Vì không có bảo hiểm, tổng chi phí cho hóa đơn dài hơn 100 trang gồm tiền giường, tiền thuốc, tiền mổ và loạt chi phí khác đã chạm ngưỡng 1 triệu đô. Và tất nhiên, số tiền anh ta dành giụm rất nhỏ khi so với chi phí điều trị. Người từng tự đắc rằng mình không bao giờ nợ ai bất kỳ điều gì trên đời này cuối cùng lại nhận món nợ 1 triệu đô theo một cách mà không ai ngờ tới - viện phí.&lt;/p&gt;
@@ -2612,50 +2749,50 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Tài sản lớn nhất của một người</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>tai-san-lon-nhat-cua-mot-nguoi</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>Tôi thích tiền, bạn thích tiền. Tất cả mọi người đều thích tiền. Những ai nói rằng tôi không thích tiền đều là nói dối. Nói dối những người xung quanh và lừa dối chính bản thân mình. Để kiếm tiền, con người có thể phải đánh đổi rất nhiều th...</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>data\blogs\Tài sản lớn nhất của một người.md</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t># Tài sản lớn nhất của một người
 Tôi thích tiền, bạn thích tiền. Tất cả mọi người đều thích tiền. Những ai nói rằng tôi không thích tiền đều là nói dối. Nói dối những người xung quanh và lừa dối chính bản thân mình. Để kiếm tiền, con người có thể phải đánh đổi rất nhiều thứ. Có người chấp nhận làm ăn xa xứ. Có người bỏ thời gian 8 - 16 tiếng mỗi ngày để làm việc. Có người nâng cao giá trị bản thân để kiếm nhiều tiền hơn. 
@@ -2711,7 +2848,7 @@
 Tuy nhiên, cũng nên lưu ý rằng câu **"Tài sản lớn nhất của một người là sự uy tín"** là một nhận định mang tính giá trị, không phải chân lý tuyệt đối. Với người khác, họ có thể cho rằng sức khỏe, thời gian hay tri thức mới là tài sản lớn nhất. Điều hợp lý hơn là xem **uy tín là một trong những tài sản vô hình giá trị nhất**, đặc biệt trong kinh doanh, lãnh đạo và các mối quan hệ lâu dài.</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>&lt;h1 id="tai-san-lon-nhat-cua-mot-nguoi"&gt;Tài sản lớn nhất của một người&lt;/h1&gt;
 &lt;p&gt;Tôi thích tiền, bạn thích tiền. Tất cả mọi người đều thích tiền. Những ai nói rằng tôi không thích tiền đều là nói dối. Nói dối những người xung quanh và lừa dối chính bản thân mình. Để kiếm tiền, con người có thể phải đánh đổi rất nhiều thứ. Có người chấp nhận làm ăn xa xứ. Có người bỏ thời gian 8 - 16 tiếng mỗi ngày để làm việc. Có người nâng cao giá trị bản thân để kiếm nhiều tiền hơn. &lt;/p&gt;
@@ -2817,54 +2954,54 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Tâm lý học blogger - Tại sao Hải viết blog?</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>tam-ly-hoc-blogger---tai-sao-hai-viet-blog</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
         <is>
           <t>web, blog</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>01-06-2026</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>Hôm nay, Hải vào xem lại trận Argentina gặp Pháp vào mùa World Cup năm 2018. Đó là năm Mbappe 19 tuổi và đã khiến Messi dừng bước với 1 kiến tạo Penalty và ghi 2 bàn thắng. Tất cả những phút chạy của Mbappe đều được tường thuật trực tiếp và...</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học blogger -Tại sao Hải viết blog.md</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t># Tâm lý học blogger - Tại sao Hải lập blog riêng?
 Hôm nay, Hải vào xem lại trận Argentina gặp Pháp vào mùa World Cup năm 2018. Đó là năm Mbappe 19 tuổi và đã khiến Messi dừng bước với 1 kiến tạo Penalty và ghi 2 bàn thắng. Tất cả những phút chạy của Mbappe đều được tường thuật trực tiếp và ghi lại để bất kỳ ai có thể xem lại sau này. Tất cả người xem bóng đá đều biết Mbappe, biết khả năng chơi bóng của anh ta, biết tốc độ của anh ta. Hàng loạt câu lạc bộ lớn muốn ký hợp đồng với anh ta với mức giá không tưởng.
@@ -2900,7 +3037,7 @@
 ---</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-blogger-tai-sao-hai-lap-blog-rieng"&gt;Tâm lý học blogger - Tại sao Hải lập blog riêng?&lt;/h1&gt;
 &lt;p&gt;Hôm nay, Hải vào xem lại trận Argentina gặp Pháp vào mùa World Cup năm 2018. Đó là năm Mbappe 19 tuổi và đã khiến Messi dừng bước với 1 kiến tạo Penalty và ghi 2 bàn thắng. Tất cả những phút chạy của Mbappe đều được tường thuật trực tiếp và ghi lại để bất kỳ ai có thể xem lại sau này. Tất cả người xem bóng đá đều biết Mbappe, biết khả năng chơi bóng của anh ta, biết tốc độ của anh ta. Hàng loạt câu lạc bộ lớn muốn ký hợp đồng với anh ta với mức giá không tưởng.&lt;/p&gt;
@@ -2937,84 +3074,84 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Tâm lý học cá độ - Vì sao người không chơi là người thắng</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>tam-ly-hoc-ca-do---vi-sao-nguoi-khong-choi-la-nguoi-thang</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>02-07-2026</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học cá độ - Vì sao người không chơi là người thắng.md</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Tâm lý học của người lười nhưng tham vọng lớn</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>tam-ly-hoc-cua-nguoi-luoi-nhung-tham-vong-lon</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
         <is>
           <t>26-05-2026</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>Theo lẽ thường, người lười thường sẽ chọn sống yên ổn thay vì tham vọng còn người đã tham vọng thì không được phép lười biếng. Nhưng có 1 kiểu tâm lý nghe qua có vẻ lạ vì nó khá đặc biệt và giống như đang trêu đùa logic nhưng nó vẫn đang xu...</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học của người lười nhưng tham vọng đạt được thành tựu lớn.md</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t># Tâm lý học của người lười nhưng tham vọng lớn
 Theo lẽ thường, người lười thường sẽ chọn sống yên ổn thay vì tham vọng còn người đã tham vọng thì không được phép lười biếng. Nhưng có 1 kiểu tâm lý nghe qua có vẻ lạ vì nó khá đặc biệt và giống như đang trêu đùa logic nhưng nó vẫn đang xuất hiện trong hàng triệu triệu người mỗi ngày. Đó chính là tâm lý của người lười nhưng tham vọng lớn. 
@@ -3043,7 +3180,7 @@
 Giáo sư Jiang Xue Qin</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-cua-nguoi-luoi-nhung-tham-vong-lon"&gt;Tâm lý học của người lười nhưng tham vọng lớn&lt;/h1&gt;
 &lt;p&gt;Theo lẽ thường, người lười thường sẽ chọn sống yên ổn thay vì tham vọng còn người đã tham vọng thì không được phép lười biếng. Nhưng có 1 kiểu tâm lý nghe qua có vẻ lạ vì nó khá đặc biệt và giống như đang trêu đùa logic nhưng nó vẫn đang xuất hiện trong hàng triệu triệu người mỗi ngày. Đó chính là tâm lý của người lười nhưng tham vọng lớn. &lt;/p&gt;
@@ -3073,54 +3210,54 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Tâm lý học FOMO</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>tam-ly-hoc-fomo</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
         <is>
           <t>fomo</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>28-05-2026</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>Từ thời nguyên thủy, con người đã luôn sợ bỏ lỡ. Nếu bộ lạc săn được thức ăn mà 1 cá thể trong bầy không biết, cá thể đó có thể bị đói. Nếu 1 thành viên nào trong bầy người nguyên thủy bỏ lỡ việc di dời theo bầy vì thời tiết cực đoan, thành...</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học FOMO.md</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t># Tâm lý học FOMO
 Từ thời nguyên thủy, con người đã luôn sợ bỏ lỡ. Nếu bộ lạc săn được thức ăn mà 1 cá thể trong bầy không biết, cá thể đó có thể bị đói. Nếu 1 thành viên nào trong bầy người nguyên thủy bỏ lỡ việc di dời theo bầy vì thời tiết cực đoan, thành viên đó sẽ gặp nguy hiểm. Ngày nay, chúng ta thấy tâm lý FOMO (fear-of-missing-out) ở khắp mọi nơi: cái áo chỉ giảm giá trong ngày, drama trên mạng xã hội, sóng đầu tư tiền ảo, tin tức thời sự,... Khai thác FOMO là ngành công nghiệp kiếm rất nhiều tiền bởi con người không chỉ sợ thất bại, họ còn sợ mình đang đứng yên trong khi người khác vẫn chạy.
@@ -3143,7 +3280,7 @@
 FOMO không phải dấu hiệu của sự nhu nhược, hay sự thiếu quyết đoán. Nó là phản ứng rất bình thường của não bộ con người từ xưa tới nay. Từ thời kỳ săn bắt hái lượm tới thời kỳ drama và trào lưu trên mạng xã hội. Xóa bỏ hoàn toàn tâm lý FOMO là vô ích và tự hủy cơ chế bảo vệ bản thân mà tạo hóa ban tặng.</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-fomo"&gt;Tâm lý học FOMO&lt;/h1&gt;
 &lt;p&gt;Từ thời nguyên thủy, con người đã luôn sợ bỏ lỡ. Nếu bộ lạc săn được thức ăn mà 1 cá thể trong bầy không biết, cá thể đó có thể bị đói. Nếu 1 thành viên nào trong bầy người nguyên thủy bỏ lỡ việc di dời theo bầy vì thời tiết cực đoan, thành viên đó sẽ gặp nguy hiểm. Ngày nay, chúng ta thấy tâm lý FOMO (fear-of-missing-out) ở khắp mọi nơi: cái áo chỉ giảm giá trong ngày, drama trên mạng xã hội, sóng đầu tư tiền ảo, tin tức thời sự,... Khai thác FOMO là ngành công nghiệp kiếm rất nhiều tiền bởi con người không chỉ sợ thất bại, họ còn sợ mình đang đứng yên trong khi người khác vẫn chạy.&lt;/p&gt;
@@ -3167,49 +3304,49 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Tâm lý học kinh nghiệm</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>tam-ly-hoc-kinh-nghiem</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>Anh đọc bài viết em cũng ổn.</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học kinh nghiệm.md</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>Anh đọc bài viết em cũng ổn.
 Ví dụ tâm lý học nhà thầu, em phân tích mục đích và hành động của nhiều nhóm người chơi nhưng không đưa ra được hệ phương trình vi phân để mô hình hóa sự thay đổi động lực của các người chơi trong dự án. Em cũng không đưa ra được mô hình xác suất có điều kiện trong trường hợp nào nhà thầu sẽ ưu tiên tìm đối tác giá rẻ và trong trường hợp nào họ ưu tiên sự yên tâm. 
 Hay 1 ví dụ khác</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>&lt;p&gt;Anh đọc bài viết em cũng ổn.&lt;/p&gt;
 &lt;p&gt;Ví dụ tâm lý học nhà thầu, em phân tích mục đích và hành động của nhiều nhóm người chơi nhưng không đưa ra được hệ phương trình vi phân để mô hình hóa sự thay đổi động lực của các người chơi trong dự án. Em cũng không đưa ra được mô hình xác suất có điều kiện trong trường hợp nào nhà thầu sẽ ưu tiên tìm đối tác giá rẻ và trong trường hợp nào họ ưu tiên sự yên tâm. &lt;/p&gt;
@@ -3217,50 +3354,50 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Tâm lý học Michelin Boy</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>tam-ly-hoc-michelin-boy</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>indraft</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr">
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
         <is>
           <t>07-06-2026</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>23-06-2026</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>Vì sao chúng ta không bao giờ nghe đến từ Michelin Girl.</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học Michelin Boy.md</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t># Tâm lý học Michelin Boy
 Vì sao chúng ta không bao giờ nghe đến từ Michelin Girl.
@@ -3283,7 +3420,7 @@
 [^1]: This is the footnote.</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-michelin-boy"&gt;Tâm lý học Michelin Boy&lt;/h1&gt;
 &lt;p&gt;Vì sao chúng ta không bao giờ nghe đến từ Michelin Girl.&lt;/p&gt;
@@ -3312,100 +3449,100 @@
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Tâm lý học một view</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>tam-ly-hoc-mot-view</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr">
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học một view.md</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t># Tâm lý học một view</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-mot-view"&gt;Tâm lý học một view&lt;/h1&gt;</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Tâm lý học nghiện xem video phát triển bản thân</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>tam-ly-hoc-nghien-xem-video-phat-trien-ban-than</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr">
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
         <is>
           <t>29-05-2026</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>30-05-2026</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>Con người luôn muốn hoàn thiện mình và hướng tới chân thiện mỹ. Đó là lý do chúng ta luôn tìm cách để bản thân mình tốt lên hằng ngày. Tập thể dục, học tập, rèn luyện, học kỹ năng mới hay mở rộng vòng tròn các mối quan hệ xã hội - tất cả nh...</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học nghiện xem video phát triển bản thân.md</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t># Tâm lý học nghiện xem video phát triển bản thân
 Con người luôn muốn hoàn thiện mình và hướng tới chân thiện mỹ. Đó là lý do chúng ta luôn tìm cách để bản thân mình tốt lên hằng ngày. Tập thể dục, học tập, rèn luyện, học kỹ năng mới hay mở rộng vòng tròn các mối quan hệ xã hội - tất cả nhằm 1 mục đích là nâng cấp bản thân. Cũng từ đó, có một thứ nghiện khá mới trong thời đại mạng xã hội ngày nay, không phải nghiện game, không phải nghiện phim mà là nghiện xem video phát triển bản thân. 
@@ -3416,7 +3553,7 @@
 ##</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-nghien-xem-video-phat-trien-ban-than"&gt;Tâm lý học nghiện xem video phát triển bản thân&lt;/h1&gt;
 &lt;p&gt;Con người luôn muốn hoàn thiện mình và hướng tới chân thiện mỹ. Đó là lý do chúng ta luôn tìm cách để bản thân mình tốt lên hằng ngày. Tập thể dục, học tập, rèn luyện, học kỹ năng mới hay mở rộng vòng tròn các mối quan hệ xã hội - tất cả nhằm 1 mục đích là nâng cấp bản thân. Cũng từ đó, có một thứ nghiện khá mới trong thời đại mạng xã hội ngày nay, không phải nghiện game, không phải nghiện phim mà là nghiện xem video phát triển bản thân. &lt;/p&gt;
@@ -3428,58 +3565,58 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Tâm lý học ngành bột mì</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>tam-ly-hoc-nganh-bot-mi</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>bột mì</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>28-05-2026</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>Chỉ trong 1 thời gian ngắn trước lúc Hải viết bài này, đã có rất nhiều người nhận kết quả test dương tính với bột mì. Trong số đó có cả những người nổi tiếng, có sức ảnh hưởng. Đa phần chúng ta đều thắc mắc tại sao những người đã giàu, đã c...</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học ngành bột mì.md</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t># Tâm lý học ngành bột mì
 Chỉ trong 1 thời gian ngắn trước lúc Hải viết bài này, đã có rất nhiều người nhận kết quả test dương tính với bột mì. Trong số đó có cả những người nổi tiếng, có sức ảnh hưởng. Đa phần chúng ta đều thắc mắc tại sao những người đã giàu, đã có gần như tất cả mọi thứ lại dính vào thứ tệ nạn này? Và tại sao trong rất nhiều thập kỷ, ngành công nghiệp này vẫn tồn tại bất kể luật pháp trừng phạt rất mạnh tay?
@@ -3516,7 +3653,7 @@
 Đứng trước lợi nhuận khổng lồ, nhiều cá nhân chấp nhận rủi ro đối mặt án tử để đi sản xuất, tàng trữ và vận chuyển bột mì. Và tất nhiên, phía bên kia của lợi nhuận đó chính là những cuộc đời bị phá hủy, những gia đình tan vỡ, những người trẻ đánh mất tương lai. Bản thân ngành công nghiệp bột mì còn tồn tại không phải chỉ nằm ở việc nó là chất kích thích, nó khai thác vào cảm giác cô đơn, áp lực, muốn hòa nhập, muốn thoát khỏi thực tại của mỗi người. Nó không chỉ là câu chuyện của pháp luật, nó còn là câu chuyện của giáo dục, môi trường sống và các mối quan hệ.</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-nganh-bot-mi"&gt;Tâm lý học ngành bột mì&lt;/h1&gt;
 &lt;p&gt;Chỉ trong 1 thời gian ngắn trước lúc Hải viết bài này, đã có rất nhiều người nhận kết quả test dương tính với bột mì. Trong số đó có cả những người nổi tiếng, có sức ảnh hưởng. Đa phần chúng ta đều thắc mắc tại sao những người đã giàu, đã có gần như tất cả mọi thứ lại dính vào thứ tệ nạn này? Và tại sao trong rất nhiều thập kỷ, ngành công nghiệp này vẫn tồn tại bất kể luật pháp trừng phạt rất mạnh tay?&lt;/p&gt;
@@ -3579,58 +3716,58 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Tâm lý học nhà thầu</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>tam-ly-hoc-nha-thau</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>thầu, dự án</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>26-05-2026</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>Trước khi bắt đầu bài viết, Hải muốn lưu ý rằng đấu thầu và quản lý dự án là lĩnh vực cực kỳ rộng. Mỗi người tham gia dự án đều đứng ở một vị trí khác nhau nên sẽ nhìn thấy những vấn đề khác nhau. Một chủ đầu tư sẽ có góc nhìn khác nhà thầu...</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học nhà thầu.md</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t># Tâm lý học nhà thầu
 Trước khi bắt đầu bài viết, Hải muốn lưu ý rằng đấu thầu và quản lý dự án là lĩnh vực cực kỳ rộng. Mỗi người tham gia dự án đều đứng ở một vị trí khác nhau nên sẽ nhìn thấy những vấn đề khác nhau. Một chủ đầu tư sẽ có góc nhìn khác nhà thầu. Một kỹ sư hiện trường sẽ có góc nhìn khác đơn vị thiết kế. Một công nhân sẽ có góc nhìn khác người quản lý dự án. Vì vậy, bài viết chỉ là một góc nhìn của Hải dưới lăng kính tâm lý học và lý thuyết trò chơi.
@@ -3675,7 +3812,7 @@
 Bài viết này chủ yếu được nhìn dưới lăng kính tâm lý học, kinh tế học và lý thuyết trò chơi. Hải hiểu rằng thực tế ngoài công trường luôn phức tạp hơn rất nhiều so với những gì có thể trình bày trong một bài blog. Nên nếu anh em đang làm trong lĩnh vực xây dựng, đấu thầu, quản lý dự án, giám sát, thiết kế hoặc từng tham gia các dự án lớn, Hải rất mong nhận được những góp ý, phản biện hoặc góc nhìn khác của anh em qua email **nguyenquyhai2002@gmail.com**.</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-nha-thau"&gt;Tâm lý học nhà thầu&lt;/h1&gt;
 &lt;p&gt;Trước khi bắt đầu bài viết, Hải muốn lưu ý rằng đấu thầu và quản lý dự án là lĩnh vực cực kỳ rộng. Mỗi người tham gia dự án đều đứng ở một vị trí khác nhau nên sẽ nhìn thấy những vấn đề khác nhau. Một chủ đầu tư sẽ có góc nhìn khác nhà thầu. Một kỹ sư hiện trường sẽ có góc nhìn khác đơn vị thiết kế. Một công nhân sẽ có góc nhìn khác người quản lý dự án. Vì vậy, bài viết chỉ là một góc nhìn của Hải dưới lăng kính tâm lý học và lý thuyết trò chơi.&lt;/p&gt;
@@ -3758,83 +3895,15 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Tâm lý học phông bạt</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>tam-ly-hoc-phong-bat</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>26-05-2026</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>26-05-2026</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>data\blogs\Tâm lý học phông bạt.md</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Tâm lý học sưu tầm tài liệu nhưng không đọc</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>tam-ly-hoc-suu-tam-tai-lieu-nhung-khong-doc</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>29-05-2026</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>29-05-2026</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>data\blogs\Tâm lý học sưu tầm tài liệu nhưng không đọc.md</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-    </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Tâm lý học trái tim em nhỏ lắm nên chỉ chứa được một người</t>
+          <t>Tâm lý học phông bạt</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>tam-ly-hoc-trai-tim-em-nho-lam-nen-chi-chua-duoc-mot-nguoi</t>
+          <t>tam-ly-hoc-phong-bat</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -3848,45 +3917,27 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học l...</t>
-        </is>
-      </c>
+          <t>26-05-2026</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
-          <t>data\blogs\Tâm lý học trái tim em nhỏ lắm nên chỉ chứa được một người.md</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học lớn? Tất nhiên là không phải chỉ là tải 1 hay 2 cuốn mà là tải rất rất nhiều, rồi lưu chúng vào thư mục trên máy tính hoặc điện thoại. Sau đó, chúng được mở ra từ 1-2 lần và không có sau đó nữa. Kể từ đó, đống tài liệu trên chỉ còn là file được lưu trữ trên máy tính mà không bao giờ được mở. Nếu anh em đã từng rơi vào tình huống như vậy thì đây là bài viết dành cho anh em.
-## Cảm xúc mới lạ
-## Tại sao chúng ta không bao giờ đọc
-##</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học lớn? Tất nhiên là không phải chỉ là tải 1 hay 2 cuốn mà là tải rất rất nhiều, rồi lưu chúng vào thư mục trên máy tính hoặc điện thoại. Sau đó, chúng được mở ra từ 1-2 lần và không có sau đó nữa. Kể từ đó, đống tài liệu trên chỉ còn là file được lưu trữ trên máy tính mà không bao giờ được mở. Nếu anh em đã từng rơi vào tình huống như vậy thì đây là bài viết dành cho anh em.&lt;/p&gt;
-&lt;h2 id="cam-xuc-moi-la"&gt;Cảm xúc mới lạ&lt;/h2&gt;
-&lt;h2 id="tai-sao-chung-ta-khong-bao-gio-oc"&gt;Tại sao chúng ta không bao giờ đọc&lt;/h2&gt;
-&lt;h2 id="_1"&gt;&lt;/h2&gt;</t>
-        </is>
-      </c>
+          <t>data\blogs\Tâm lý học phông bạt.md</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Tâm lý học xổ số - vì sao người trúng số thường về nợ sau vài năm</t>
+          <t>Tâm lý học sưu tầm tài liệu nhưng không đọc</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>tam-ly-hoc-xo-so---vi-sao-nguoi-trung-so-thuong-ve-no-sau-vai-nam</t>
+          <t>tam-ly-hoc-suu-tam-tai-lieu-nhung-khong-doc</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -3895,18 +3946,18 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>26-05-2026</t>
+          <t>29-05-2026</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>26-05-2026</t>
+          <t>29-05-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>data\blogs\Tâm lý học xổ số - vì sao người trúng số thường về nợ sau vài năm.md</t>
+          <t>data\blogs\Tâm lý học sưu tầm tài liệu nhưng không đọc.md</t>
         </is>
       </c>
       <c r="K37" t="inlineStr"/>
@@ -3915,51 +3966,137 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Tìm hiểu về MCP</t>
+          <t>Tâm lý học trái tim em nhỏ lắm nên chỉ chứa được một người</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>tim-hieu-ve-mcp</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>in-draft</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Công nghệ</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Quý Hải Ng</t>
-        </is>
-      </c>
+          <t>tam-ly-hoc-trai-tim-em-nho-lam-nen-chi-chua-duoc-mot-nguoi</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
+          <t>26-05-2026</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>08-06-2026</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học l...</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>data\blogs\Tâm lý học trái tim em nhỏ lắm nên chỉ chứa được một người.md</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học lớn? Tất nhiên là không phải chỉ là tải 1 hay 2 cuốn mà là tải rất rất nhiều, rồi lưu chúng vào thư mục trên máy tính hoặc điện thoại. Sau đó, chúng được mở ra từ 1-2 lần và không có sau đó nữa. Kể từ đó, đống tài liệu trên chỉ còn là file được lưu trữ trên máy tính mà không bao giờ được mở. Nếu anh em đã từng rơi vào tình huống như vậy thì đây là bài viết dành cho anh em.
+## Cảm xúc mới lạ
+## Tại sao chúng ta không bao giờ đọc
+##</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học lớn? Tất nhiên là không phải chỉ là tải 1 hay 2 cuốn mà là tải rất rất nhiều, rồi lưu chúng vào thư mục trên máy tính hoặc điện thoại. Sau đó, chúng được mở ra từ 1-2 lần và không có sau đó nữa. Kể từ đó, đống tài liệu trên chỉ còn là file được lưu trữ trên máy tính mà không bao giờ được mở. Nếu anh em đã từng rơi vào tình huống như vậy thì đây là bài viết dành cho anh em.&lt;/p&gt;
+&lt;h2 id="cam-xuc-moi-la"&gt;Cảm xúc mới lạ&lt;/h2&gt;
+&lt;h2 id="tai-sao-chung-ta-khong-bao-gio-oc"&gt;Tại sao chúng ta không bao giờ đọc&lt;/h2&gt;
+&lt;h2 id="_1"&gt;&lt;/h2&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Tâm lý học xổ số - vì sao người trúng số thường về nợ sau vài năm</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>tam-ly-hoc-xo-so---vi-sao-nguoi-trung-so-thuong-ve-no-sau-vai-nam</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>26-05-2026</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>26-05-2026</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>data\blogs\Tâm lý học xổ số - vì sao người trúng số thường về nợ sau vài năm.md</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Tìm hiểu về MCP</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>tim-hieu-ve-mcp</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Công nghệ</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
           <t>06-07-2026</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>15-07-2026</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>Hãy bắt đầu với 1 công cụ mà chúng ta đều biết - ChatGPT. Khi 1 người muốn nhờ ChatGPT làm 1 điều gì đó, họ sẽ gửi prompt và sau đó ChatGPT sẽ phản hồi lại người đó. Và xuyên suốt quá trình này chỉ nhận văn bản và trả về văn bản. Không có 1...</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>data\blogs\Tìm hiểu về MCP.md</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t># Tìm hiểu về MCP
 ## Tại sao chúng ta cần MCP
@@ -3970,7 +4107,7 @@
 *MCP như cổng kết nối USB. Nguồn: modelcontextprotocol.io*</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>&lt;h1 id="tim-hieu-ve-mcp"&gt;Tìm hiểu về MCP&lt;/h1&gt;
 &lt;h2 id="tai-sao-chung-ta-can-mcp"&gt;Tại sao chúng ta cần MCP&lt;/h2&gt;
@@ -3982,50 +4119,50 @@
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Tư duy cắt chuỗi</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>tu-duy-cat-chuoi</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr">
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr">
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>Để có thể thích nghi với hầu hết toàn bộ nền tảng, môi trường triển khai trong ngành phần mềm và thông tin, có 1 kỹ thuật mang tên cắt chuỗi. Nó giúp chúng ta vượt qua mọi tư duy và rảo cản về môi trường triển khai, chi phí vận hành. Nó hỗ...</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>data\blogs\Tư duy cắt chuỗi.md</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t># Tư duy cắt chuỗi
 Để có thể thích nghi với hầu hết toàn bộ nền tảng, môi trường triển khai trong ngành phần mềm và thông tin, có 1 kỹ thuật mang tên cắt chuỗi. Nó giúp chúng ta vượt qua mọi tư duy và rảo cản về môi trường triển khai, chi phí vận hành. Nó hỗ trợ chúng ta có nền tảng để tự dụng lên mọi nội dung, hệ thống. Nó chính là bước khác biệt và cũng là bước khó nhất trong toàn bộ quy trình tự động.   
@@ -4040,7 +4177,7 @@
 ## Kết</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>&lt;h1 id="tu-duy-cat-chuoi"&gt;Tư duy cắt chuỗi&lt;/h1&gt;
 &lt;p&gt;Để có thể thích nghi với hầu hết toàn bộ nền tảng, môi trường triển khai trong ngành phần mềm và thông tin, có 1 kỹ thuật mang tên cắt chuỗi. Nó giúp chúng ta vượt qua mọi tư duy và rảo cản về môi trường triển khai, chi phí vận hành. Nó hỗ trợ chúng ta có nền tảng để tự dụng lên mọi nội dung, hệ thống. Nó chính là bước khác biệt và cũng là bước khó nhất trong toàn bộ quy trình tự động.   &lt;/p&gt;
@@ -4056,84 +4193,84 @@
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Tư duy Excel</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>tu-duy-excel</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr">
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr">
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
         <is>
           <t>data\blogs\Tư duy Excel.md</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Tư duy ngược và tư duy mở ngành phần mềm</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>tu-duy-nguoc-va-tu-duy-mo-nganh-phan-mem</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr">
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>Linux - Windows - Mac</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>data\blogs\Tư duy ngược và tư duy mở ngành phần mềm.md</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t># Tư duy ngược và tư duy mở ngành phần mềm
 ## Những thứ có giá trị nhất đôi khi là rẻ nhất hoặc miễn phí
@@ -4142,7 +4279,7 @@
 ## Giải pháp triệu đô</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>&lt;h1 id="tu-duy-nguoc-va-tu-duy-mo-nganh-phan-mem"&gt;Tư duy ngược và tư duy mở ngành phần mềm&lt;/h1&gt;
 &lt;h2 id="nhung-thu-co-gia-tri-nhat-oi-khi-la-re-nhat-hoac-mien-phi"&gt;Những thứ có giá trị nhất đôi khi là rẻ nhất hoặc miễn phí&lt;/h2&gt;
@@ -4152,58 +4289,58 @@
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>Tư duy xô nước</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>tu-duy-xo-nuoc</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>Tư duy</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>xô nước, đường ống</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>15-06-2026</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>16-06-2026</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>Câu chuyện kể về một thị trấn nọ nơi những ngày đầu các hộ dân đều mang theo xô đến sông để mang nước về nhà mỗi ngày. Về sau, các gia đình chọn trả tiền để thuê những thanh niên trai tráng trong làng xách nước thay vì tự mình mang xô đến....</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>data\blogs\Tư duy xô nước.md</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t># Tư duy xô nước
 Câu chuyện kể về một thị trấn nọ nơi những ngày đầu các hộ dân đều mang theo xô đến sông để mang nước về nhà mỗi ngày. Về sau, các gia đình chọn trả tiền để thuê những thanh niên trai tráng trong làng xách nước thay vì tự mình mang xô đến.  Giai đoạn đầu, các thanh niên trong làng hứng khởi và xách xô nước vì số tiền họ kiếm được phụ thuộc vào số xô nước họ giao. Các gia đình ai ai cũng muốn gả con gái cho những thanh niên chăm chỉ sẵn sàng đi xách nước vào cả khung giờ chiều tối, nửa đêm để đáp ứng nhu cầu sử dụng nước cho nhiều gia đình. Sự thành đạt, tinh thần làm việc chăm chỉ, tương lai cầu tiến được thể hiện bằng số giờ đi xách xô nước và số xô nước họ đã mang đến từng nhà. Các thanh niên ốm yếu, gầy gò trong làng lúc này cũng đã tham gia vì công việc này ngày nào cũng có và không hết việc. Và đó cũng là việc mà các thanh thiếu niên chí khí trong làng lúc bấy giờ nên dấn thân. 
@@ -4233,7 +4370,7 @@
 Một trong những thứ có thể tồn tại lâu hơn tuổi thọ của con người đó là đường ống. Con người rồi sẽ già đi. Sức khỏe rồi sẽ suy giảm. Thời gian của mỗi người đều có giới hạn. Nhưng những gì chúng ta để lại thì không nhất thiết phải biến mất. Ai cũng có thể phải xách xô ở một giai đoạn nào đó của cuộc đời. Không có gì đáng xấu hổ khi dùng thời gian và sức lao động để kiếm sống. Vấn đề chỉ nằm ở chỗ: liệu sau mỗi ngày xách xô, chúng ta có dành ra một phần thời gian để xây đường ống hay không? Bởi vì đến một lúc nào đó, thứ quyết định giá trị của một con người không còn là họ đã đổ bao nhiêu mồ hôi, thức bao nhiêu đêm hay làm việc bao nhiêu giờ mỗi ngày, mà là những gì vẫn tiếp tục tạo ra giá trị ngay cả khi họ không còn ở đó.</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>&lt;h1 id="tu-duy-xo-nuoc"&gt;Tư duy xô nước&lt;/h1&gt;
 &lt;p&gt;Câu chuyện kể về một thị trấn nọ nơi những ngày đầu các hộ dân đều mang theo xô đến sông để mang nước về nhà mỗi ngày. Về sau, các gia đình chọn trả tiền để thuê những thanh niên trai tráng trong làng xách nước thay vì tự mình mang xô đến.  Giai đoạn đầu, các thanh niên trong làng hứng khởi và xách xô nước vì số tiền họ kiếm được phụ thuộc vào số xô nước họ giao. Các gia đình ai ai cũng muốn gả con gái cho những thanh niên chăm chỉ sẵn sàng đi xách nước vào cả khung giờ chiều tối, nửa đêm để đáp ứng nhu cầu sử dụng nước cho nhiều gia đình. Sự thành đạt, tinh thần làm việc chăm chỉ, tương lai cầu tiến được thể hiện bằng số giờ đi xách xô nước và số xô nước họ đã mang đến từng nhà. Các thanh niên ốm yếu, gầy gò trong làng lúc này cũng đã tham gia vì công việc này ngày nào cũng có và không hết việc. Và đó cũng là việc mà các thanh thiếu niên chí khí trong làng lúc bấy giờ nên dấn thân. &lt;/p&gt;
@@ -4264,54 +4401,54 @@
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Tại sao Bitcoin cưa đôi?</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>tai-sao-bitcoin-cua-doi</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Công nghệ</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr">
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải...</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>data\blogs\Tại sao Bitcon cưa đôi.md</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t># Tại sao Bitcoin cưa đôi?
 Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải có đáng để đọc và có đủ sức thuyết phục hay không?". Hải hoàn toàn hiểu, và cũng theo một góc độ nào đó, chính vì Hải chưa từng được hưởng lợi hay chịu thiệt hại từ Bitcoin, anh em có thể tham khảo bài viết từ một người có góc nhìn trung lập. Mục tiêu của bài viết là đưa ra thật nhiều góc nhìn vì cho tới nay vẫn có rất nhiều ý kiến trái chiều về tiền mã hóa. Có người thì bảo rằng đó là công nghệ tương lai của nhân loại, cũng có người nói đó là trò lừa bịp, lừa đảo và rửa tiền. Vì vậy, muốn biết nó thực sự là gì, chúng ta phải thảo luận về nó, phải đặt câu hỏi về nó, phải xem qua các trường hợp trước đây nó được sử dụng cho mục đích gì?
@@ -4377,7 +4514,7 @@
 [^3]: [Controlled supply - Bitcoin Wiki](https://en.bitcoin.it/wiki/Controlled_supply)</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>&lt;h1 id="tai-sao-bitcoin-cua-oi"&gt;Tại sao Bitcoin cưa đôi?&lt;/h1&gt;
 &lt;p&gt;Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải có đáng để đọc và có đủ sức thuyết phục hay không?". Hải hoàn toàn hiểu, và cũng theo một góc độ nào đó, chính vì Hải chưa từng được hưởng lợi hay chịu thiệt hại từ Bitcoin, anh em có thể tham khảo bài viết từ một người có góc nhìn trung lập. Mục tiêu của bài viết là đưa ra thật nhiều góc nhìn vì cho tới nay vẫn có rất nhiều ý kiến trái chiều về tiền mã hóa. Có người thì bảo rằng đó là công nghệ tương lai của nhân loại, cũng có người nói đó là trò lừa bịp, lừa đảo và rửa tiền. Vì vậy, muốn biết nó thực sự là gì, chúng ta phải thảo luận về nó, phải đặt câu hỏi về nó, phải xem qua các trường hợp trước đây nó được sử dụng cho mục đích gì?&lt;/p&gt;
@@ -4469,104 +4606,104 @@
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Tại sao lại là Blockchain</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>tai-sao-lai-la-blockchain</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>Công nghệ</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr">
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H46" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr">
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
         <is>
           <t>data\blogs\Tại sao lại là Blockchain.md</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t># Tại sao lại là Blockchain?</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="L46" t="inlineStr">
         <is>
           <t>&lt;h1 id="tai-sao-lai-la-blockchain"&gt;Tại sao lại là Blockchain?&lt;/h1&gt;</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Tại sao lại là start-up?</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>tai-sao-lai-la-start-up</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr">
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr">
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
         <is>
           <t>27-08-2026</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>02-09-2026</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>&gt; "Đừng bao giờ đánh mất đi ước mơ và khát vọng của chính mình. Vì nếu bạn làm thế, bạn có lẽ vẫn sẽ tồn tại nhưng bạn đã ngừng sống mất rồi!" &gt; &gt; _- Henry David Thoreau_</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>data\blogs\Tại sao lại là start-up.md</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t># Tại sao lại là start-up?
 &gt; "Đừng bao giờ đánh mất đi ước mơ và khát vọng của chính mình. Vì nếu bạn làm thế, bạn có lẽ vẫn sẽ tồn tại nhưng bạn đã ngừng sống mất rồi!"
@@ -4597,7 +4734,7 @@
 Xã hội thay đổi thì con người và tổ chức cũng cần đổi thay. Và bất kể sự lựa chọn của mỗi người có là gì, miễn là sống thật tốt - đều xứng đáng được trân trọng.</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>&lt;h1 id="tai-sao-lai-la-start-up"&gt;Tại sao lại là start-up?&lt;/h1&gt;
 &lt;blockquote&gt;
@@ -4631,56 +4768,56 @@
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Vì sao con người tự ti</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>vi-sao-con-nguoi-tu-ti</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr">
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
         <is>
           <t>23-07-2026</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H48" t="inlineStr">
         <is>
           <t>23-07-2026</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>- [ ] họ không tự hào về bản thân họ, về môi trường họ sinh ra, về</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>data\blogs\Vì sao con người tự ti.md</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t># Vì sao con người tự ti?
 - [ ] họ không tự hào về bản thân họ, về môi trường họ sinh ra, về</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L48" t="inlineStr">
         <is>
           <t>&lt;h1 id="vi-sao-con-nguoi-tu-ti"&gt;Vì sao con người tự ti?&lt;/h1&gt;
 &lt;ul class="task-list"&gt;
@@ -4689,84 +4826,84 @@
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>Vì sao khởi nghiệp thất bại</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>vi-sao-khoi-nghiep-that-bai</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr">
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr">
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
         <is>
           <t>data\blogs\Vì sao khởi nghiệp thất bại.md</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>Vì sao người giàu thích nợ?</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>vi-sao-nguoi-giau-thich-no</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr">
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr">
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
         <is>
           <t>23-06-2026</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>02-07-2026</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>Có 1 lần trong cuộc phỏng vấn, tổng thống thứ 45 và 47 của Hoa Kỳ - Donald Trump có chia sẻ về câu chuyện cho tiền người giàu hơn ông khoảng 900 triệu đô. Đó là một ngày khi ông cùng người đẹp dạo phố và ông Trump nói với cô gái: “Em biết n...</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>data\blogs\Vì sao người giàu thích nợ.md</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t># Vì sao người giàu thích nợ
 Có 1 lần trong cuộc phỏng vấn, tổng thống thứ 45 và 47 của Hoa Kỳ - Donald Trump có chia sẻ về câu chuyện cho tiền người giàu hơn ông khoảng 900 triệu đô. Đó là một ngày khi ông cùng người đẹp dạo phố và ông Trump nói với cô gái: “Em biết người đàn ông đó là ai không?”. “Em biết, ông ấy là ăn xin” - cô gái đáp. Ông Trump nói tiếp: “Ngay bây giờ, ông ấy đang có nhiều hơn anh 900 triệu đô”. Và cô gái thắc mắc: “Làm sao người ăn xin có thể có nhiều tiền hơn ông được?”. Bởi vì người ăn xin tuy  không có đồng nào nhưng cũng không có nợ. Trong khi đó, ông Trump nợ 900 triệu đô. Đó là thời điểm bất động sản ở Mỹ đang ở dưới đáy chu kỳ vào những năm đầu thập niên 90. Và tất nhiên sau đó, thị trường bất động sản ở New York mà ông Trump đầu tư xây dựng đã phát triển bùng nổ.
@@ -4801,7 +4938,7 @@
 Cái gì quan trọng thì nhắc lại ba lần: “Ai sinh ra trên đời cũng chỉ có 2 bàn tay trắng và sẽ không cầm theo được bất cứ thứ gì khi rời đi”. Nhìn nhận về nợ ra sao, đó là quan điểm của mỗi người. Chúng ta chỉ biết rằng, trong lịch sử loài người, nếu không có thứ đó, sẽ mất rất lâu nữa để có hàng ngàn sa số những công trình, công nghệ được xây dựng và phát triển tới tận ngày nay. Không có thứ đó, hàng triệu triệu người sẽ phải chôn vùi giấc mơ, những điều mình muốn làm và mang theo nó sang thế giới bên kia thay vì để lại cho nhân loại.</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="L50" t="inlineStr">
         <is>
           <t>&lt;h1 id="vi-sao-nguoi-giau-thich-no"&gt;Vì sao người giàu thích nợ&lt;/h1&gt;
 &lt;p&gt;Có 1 lần trong cuộc phỏng vấn, tổng thống thứ 45 và 47 của Hoa Kỳ - Donald Trump có chia sẻ về câu chuyện cho tiền người giàu hơn ông khoảng 900 triệu đô. Đó là một ngày khi ông cùng người đẹp dạo phố và ông Trump nói với cô gái: “Em biết người đàn ông đó là ai không?”. “Em biết, ông ấy là ăn xin” - cô gái đáp. Ông Trump nói tiếp: “Ngay bây giờ, ông ấy đang có nhiều hơn anh 900 triệu đô”. Và cô gái thắc mắc: “Làm sao người ăn xin có thể có nhiều tiền hơn ông được?”. Bởi vì người ăn xin tuy  không có đồng nào nhưng cũng không có nợ. Trong khi đó, ông Trump nợ 900 triệu đô. Đó là thời điểm bất động sản ở Mỹ đang ở dưới đáy chu kỳ vào những năm đầu thập niên 90. Và tất nhiên sau đó, thị trường bất động sản ở New York mà ông Trump đầu tư xây dựng đã phát triển bùng nổ.&lt;/p&gt;
@@ -4837,50 +4974,50 @@
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>Điều mà nhà trường không bao giờ nói với anh em</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>dieu-ma-nha-truong-khong-bao-gio-noi-voi-anh-em</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>Kinh tế</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr">
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
         <is>
           <t>25-05-2026</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H51" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>Hầu hết chúng ta được dạy rằng, phải học thật giỏi, thi vào những trường tốt nhất thì mới có cơ hội vào được 1 công ty tốt. Sau đó làm việc thật chăm chỉ, 8 tiếng mỗi ngày, 5 ngày mỗi tuần, có thể chủ động xin tăng ca để tích lũy thêm tiền...</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="J51" t="inlineStr">
         <is>
           <t>data\blogs\Điều mà nhà trường không bao giờ nói với anh em.md</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t># Điều mà nhà trường không bao giờ nói với anh em
 ## 2 kiểu tư duy về tiền
@@ -4927,7 +5064,7 @@
 Tâm lý học về tiền</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="L51" t="inlineStr">
         <is>
           <t>&lt;h1 id="ieu-ma-nha-truong-khong-bao-gio-noi-voi-anh-em"&gt;Điều mà nhà trường không bao giờ nói với anh em&lt;/h1&gt;
 &lt;h2 id="2-kieu-tu-duy-ve-tien"&gt;2 kiểu tư duy về tiền&lt;/h2&gt;

</xml_diff>

<commit_message>
Gui Hai tuoi 35
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -1561,9 +1561,17 @@
           <t>gui-hai-tuoi-35</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
@@ -1572,17 +1580,83 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>06-09-2026</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
+          <t>15-09-2026</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>MrBeast có "Hi Me In 10 Years", IShowSpeed có "Hi Me In 3 Years", Miêu Công Tử có "999 lá thư gửi bản thân". Và Hải nghĩ rằng không có một lý gì để một người nào đó không có điều gì muốn gửi tới chính mình nhiều năm sau. Và Hải cũng không n...</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
           <t>data\blogs\Gửi Hải tuổi 35.md</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t># Gửi Hải tuổi 35
+MrBeast có "Hi Me In 10 Years", IShowSpeed có "Hi Me In 3 Years", Miêu Công Tử có "999 lá thư gửi bản thân". Và Hải nghĩ rằng không có một lý gì để một người nào đó không có điều gì muốn gửi tới chính mình nhiều năm sau. Và Hải cũng không ngoại lệ.
+## Tiêu đề
+- Chủ đề: Thư gửi Hải tuổi 35
+- Người gửi: Hải tuổi 24
+- Người nhận: Hải tuổi 35
+(Ghi chú: Thư có thể thất lạc trên đường hoặc ai đó đã xem chúng trước khi đến tay người nhận)
+## Nội dung
+Chào Hải tuổi 35,
+Đầu tiên, hi vọng cậu đọc được bức thư này. Bởi vì có rất nhiều khả năng để cậu không thể đọc được bức thư này. Ý tôi là cũng có thể vì bệnh tật hoặc một vụ tai nạn nào đó sẽ làm cho cậu không còn khả năng để đọc được nó. Hi vọng những thứ kiểu vậy sẽ không đến với cậu và cậu sẽ vượt qua mọi thứ cản trở cậu đọc bức thư này.
+Được rồi, thoáng cái đã 10 năm. Có lẽ lúc này cậu đang ngồi ghế, tay trái cầm 1 tách trà nóng, tay phải cầm chuột, cậu đọc bức thư này thông qua cái kính cận 2.5 độ mắt phải (hi vọng cậu sẽ không bị cận nặng thêm). Cậu nhìn ánh sáng đêm màn hình máy tính xen lẫn với đèn led để bàn màu vàng phiên bản cozy chiếu nội dung bức thư này vào mắt cậu. Không biết rằng sau 10 năm, lăng kính nhìn đời của cậu có nhiều thay đổi hay không? Và khi đọc lại bức thư này, cảm nghĩ của cậu có khác đi hay không?
+Gia đình của cậu như thế nào? Cả gia đình lớn và gia đình nhỏ luôn? À mà cậu có lập gia đình không? Cậu simp hay đã trở thành 1 trap boy chính hiệu? Cậu được mọi người đeo đuổi hay bị mọi người xua đuổi? 
+Thành tựu lớn nhất cậu đạt được trong 10 năm qua là gì? Mất mát lớn nhất của cậu trong ngần ấy năm là gì?
+Những người mới - đến với cuộc đời cậu - họ như thế nào? Những người trước đây - từng trò chuyện, từng rất thân với cậu - họ rời đi hay ở lại? Rời đi như thế nào? Họ có quay lại không?
+Cậu có mua được nhà không? Hay đang ở thuê? Hay cậu đã là đại gia sở hữu bất động sản khắp 5 châu rồi? 
+Vòng tròn quan hệ của cậu thế nào? Mọi người có yêu mến cậu không? Người mạnh hơn cậu có lựa chọn bảo vệ cậu hay không? Người yếu hơn cậu có loại bỏ cậu ngay khi họ mạnh hơn cậu không?
+Cậu đã từng khởi nghiệp chưa? Cậu đã từng phá sản chưa? Cậu từng thất bại bao nhiêu lần rồi? Mất bao lâu để cậu đứng dậy được? 
+Các độc giả, khán thính giả của của cậu có hóng cậu sẽ làm gì tiếp theo hay không? Hay cậu đến và năn nỉ người khác quan tâm cậu? Khách hàng có đổ xô đến sự kiện của cậu hay không? Nhà đầu tư có chen chân nhau để rót vốn cho cậu hay không? Hay cậu vẫn đến từng nơi, gọi từng cuộc và nghe từng lời từ chối?
+Wow, còn có rất nhiều thứ tôi muốn hỏi cậu sau 10 năm. Và thật khó để kỳ vọng cậu có thể trả lời hết.
+Cậu biết vì sao tôi lại viết gửi cậu vào lúc này không? Hôm nay tôi đã vô tình đọc lại bài viết về tôi 10 năm trước - nhưng đó không phải là do tôi viết. Đúng, họ đã viết về cậu lúc 20 năm trước, hi vọng nó còn tồn tại để cậu có thể đọc lại. Họ đã dành cho cậu những tính từ rất đẹp: chăm ngoan - học giỏi - hòa đồng. 
+Nếu cậu có quyền quay trở lại 10 năm trước và 20 năm trước, có điều gì cậu muốn thay đổi không? Hay cậu sẽ lựa chọn giữ nguyên mọi thứ như vậy? Và nếu gặp tôi bây giờ, cậu sẽ nói gì với tôi?
+Hỏi thăm cậu vậy đủ rồi, giờ đến lượt tôi nói. Chắc cậu cũng biết 10 năm qua tôi cũng đã có khá nhiều sự thay đổi - và thế giới xung quanh tôi cũng thế. Có những lần tôi trở về, một số người vẫn nhận ra tôi. Cô bán tạp hóa, anh cắt tóc cũng nhận ra tôi. Bạn bè thầy cô vẫn nhận ra tôi. Họ liên tục hỏi tôi thế nào và nhắc lại tôi của 10 năm trước. Họ biết tôi qua đâu, họ biết tôi thế nào, họ biết tôi ra làm sao?
+Tôi nghĩ rằng với tính cách của cậu, cậu sẽ muốn đi xa - và sẽ đi xa. Cậu không muốn ai đó đến và nói với cậu rằng cậu không được phép làm thế hay cậu không có quyền làm điều đó. Và vì vậy thứ mà tôi muốn nói với cậu là sự trở về. Nghĩa vụ của cậu là sự trở về! 
+Nếu cậu đang sinh sống và làm việc ở nước ngoài mà xảy ra bất ổn, cậu có nghĩa vụ phải tìm cách liên lạc với lãnh sự quán để thực hiện quyền bảo hộ công dân. Nếu cậu đang ở ngoài khơi và gặp nạn, cậu phải bám lấy chiếc phao và giữ chặt lấy nó tới khi lên được con tàu trở về. Nếu cậu đã đạt được mục đích hoặc sự thành công ở ngoài kia, cậu cần phải trở về. Nghĩa vụ của cậu là trở về. Trở về là nghĩa vụ của cậu. 
+Chúc cậu đạt được điều những điều mình muốn và mang chúng trở về!
+God blessing you,
+Hải tuổi 24./</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>&lt;h1 id="gui-hai-tuoi-35"&gt;Gửi Hải tuổi 35&lt;/h1&gt;
+&lt;p&gt;MrBeast có "Hi Me In 10 Years", IShowSpeed có "Hi Me In 3 Years", Miêu Công Tử có "999 lá thư gửi bản thân". Và Hải nghĩ rằng không có một lý gì để một người nào đó không có điều gì muốn gửi tới chính mình nhiều năm sau. Và Hải cũng không ngoại lệ.&lt;/p&gt;
+&lt;h2 id="tieu-e"&gt;Tiêu đề&lt;/h2&gt;
+&lt;ul&gt;
+&lt;li&gt;Chủ đề: Thư gửi Hải tuổi 35&lt;/li&gt;
+&lt;li&gt;Người gửi: Hải tuổi 24&lt;/li&gt;
+&lt;li&gt;Người nhận: Hải tuổi 35&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;(Ghi chú: Thư có thể thất lạc trên đường hoặc ai đó đã xem chúng trước khi đến tay người nhận)&lt;/p&gt;
+&lt;h2 id="noi-dung"&gt;Nội dung&lt;/h2&gt;
+&lt;p&gt;Chào Hải tuổi 35,&lt;/p&gt;
+&lt;p&gt;Đầu tiên, hi vọng cậu đọc được bức thư này. Bởi vì có rất nhiều khả năng để cậu không thể đọc được bức thư này. Ý tôi là cũng có thể vì bệnh tật hoặc một vụ tai nạn nào đó sẽ làm cho cậu không còn khả năng để đọc được nó. Hi vọng những thứ kiểu vậy sẽ không đến với cậu và cậu sẽ vượt qua mọi thứ cản trở cậu đọc bức thư này.&lt;/p&gt;
+&lt;p&gt;Được rồi, thoáng cái đã 10 năm. Có lẽ lúc này cậu đang ngồi ghế, tay trái cầm 1 tách trà nóng, tay phải cầm chuột, cậu đọc bức thư này thông qua cái kính cận 2.5 độ mắt phải (hi vọng cậu sẽ không bị cận nặng thêm). Cậu nhìn ánh sáng đêm màn hình máy tính xen lẫn với đèn led để bàn màu vàng phiên bản cozy chiếu nội dung bức thư này vào mắt cậu. Không biết rằng sau 10 năm, lăng kính nhìn đời của cậu có nhiều thay đổi hay không? Và khi đọc lại bức thư này, cảm nghĩ của cậu có khác đi hay không?&lt;/p&gt;
+&lt;p&gt;Gia đình của cậu như thế nào? Cả gia đình lớn và gia đình nhỏ luôn? À mà cậu có lập gia đình không? Cậu simp hay đã trở thành 1 trap boy chính hiệu? Cậu được mọi người đeo đuổi hay bị mọi người xua đuổi? &lt;/p&gt;
+&lt;p&gt;Thành tựu lớn nhất cậu đạt được trong 10 năm qua là gì? Mất mát lớn nhất của cậu trong ngần ấy năm là gì?&lt;/p&gt;
+&lt;p&gt;Những người mới - đến với cuộc đời cậu - họ như thế nào? Những người trước đây - từng trò chuyện, từng rất thân với cậu - họ rời đi hay ở lại? Rời đi như thế nào? Họ có quay lại không?&lt;/p&gt;
+&lt;p&gt;Cậu có mua được nhà không? Hay đang ở thuê? Hay cậu đã là đại gia sở hữu bất động sản khắp 5 châu rồi? &lt;/p&gt;
+&lt;p&gt;Vòng tròn quan hệ của cậu thế nào? Mọi người có yêu mến cậu không? Người mạnh hơn cậu có lựa chọn bảo vệ cậu hay không? Người yếu hơn cậu có loại bỏ cậu ngay khi họ mạnh hơn cậu không?&lt;/p&gt;
+&lt;p&gt;Cậu đã từng khởi nghiệp chưa? Cậu đã từng phá sản chưa? Cậu từng thất bại bao nhiêu lần rồi? Mất bao lâu để cậu đứng dậy được? &lt;/p&gt;
+&lt;p&gt;Các độc giả, khán thính giả của của cậu có hóng cậu sẽ làm gì tiếp theo hay không? Hay cậu đến và năn nỉ người khác quan tâm cậu? Khách hàng có đổ xô đến sự kiện của cậu hay không? Nhà đầu tư có chen chân nhau để rót vốn cho cậu hay không? Hay cậu vẫn đến từng nơi, gọi từng cuộc và nghe từng lời từ chối?&lt;/p&gt;
+&lt;p&gt;Wow, còn có rất nhiều thứ tôi muốn hỏi cậu sau 10 năm. Và thật khó để kỳ vọng cậu có thể trả lời hết.&lt;/p&gt;
+&lt;p&gt;Cậu biết vì sao tôi lại viết gửi cậu vào lúc này không? Hôm nay tôi đã vô tình đọc lại bài viết về tôi 10 năm trước - nhưng đó không phải là do tôi viết. Đúng, họ đã viết về cậu lúc 20 năm trước, hi vọng nó còn tồn tại để cậu có thể đọc lại. Họ đã dành cho cậu những tính từ rất đẹp: chăm ngoan - học giỏi - hòa đồng. &lt;/p&gt;
+&lt;p&gt;Nếu cậu có quyền quay trở lại 10 năm trước và 20 năm trước, có điều gì cậu muốn thay đổi không? Hay cậu sẽ lựa chọn giữ nguyên mọi thứ như vậy? Và nếu gặp tôi bây giờ, cậu sẽ nói gì với tôi?&lt;/p&gt;
+&lt;p&gt;Hỏi thăm cậu vậy đủ rồi, giờ đến lượt tôi nói. Chắc cậu cũng biết 10 năm qua tôi cũng đã có khá nhiều sự thay đổi - và thế giới xung quanh tôi cũng thế. Có những lần tôi trở về, một số người vẫn nhận ra tôi. Cô bán tạp hóa, anh cắt tóc cũng nhận ra tôi. Bạn bè thầy cô vẫn nhận ra tôi. Họ liên tục hỏi tôi thế nào và nhắc lại tôi của 10 năm trước. Họ biết tôi qua đâu, họ biết tôi thế nào, họ biết tôi ra làm sao?&lt;/p&gt;
+&lt;p&gt;Tôi nghĩ rằng với tính cách của cậu, cậu sẽ muốn đi xa - và sẽ đi xa. Cậu không muốn ai đó đến và nói với cậu rằng cậu không được phép làm thế hay cậu không có quyền làm điều đó. Và vì vậy thứ mà tôi muốn nói với cậu là sự trở về. Nghĩa vụ của cậu là sự trở về! &lt;/p&gt;
+&lt;p&gt;Nếu cậu đang sinh sống và làm việc ở nước ngoài mà xảy ra bất ổn, cậu có nghĩa vụ phải tìm cách liên lạc với lãnh sự quán để thực hiện quyền bảo hộ công dân. Nếu cậu đang ở ngoài khơi và gặp nạn, cậu phải bám lấy chiếc phao và giữ chặt lấy nó tới khi lên được con tàu trở về. Nếu cậu đã đạt được mục đích hoặc sự thành công ở ngoài kia, cậu cần phải trở về. Nghĩa vụ của cậu là trở về. Trở về là nghĩa vụ của cậu. &lt;/p&gt;
+&lt;p&gt;Chúc cậu đạt được điều những điều mình muốn và mang chúng trở về!&lt;/p&gt;
+&lt;p&gt;God blessing you,&lt;/p&gt;
+&lt;p&gt;Hải tuổi 24./&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">

</xml_diff>

<commit_message>
Gui Hai tuoi 35 edit 1
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -1585,7 +1585,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>MrBeast có "Hi Me In 10 Years", IShowSpeed có "Hi Me In 3 Years", Miêu Công Tử có "999 lá thư gửi bản thân". Và Hải nghĩ rằng không có một lý gì để một người nào đó không có điều gì muốn gửi tới chính mình nhiều năm sau. Và Hải cũng không n...</t>
+          <t>MrBeast có "Hi Me In 10 Years", IShowSpeed có "Hi Me In 3 Years", Miêu Công Tử có "999 lá thư gửi bản thân". Và Hải nghĩ rằng không có một lý do gì để một người nào đó không có điều gì muốn gửi tới chính mình nhiều năm sau. Và Hải cũng khôn...</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1596,7 +1596,7 @@
       <c r="K13" t="inlineStr">
         <is>
           <t># Gửi Hải tuổi 35
-MrBeast có "Hi Me In 10 Years", IShowSpeed có "Hi Me In 3 Years", Miêu Công Tử có "999 lá thư gửi bản thân". Và Hải nghĩ rằng không có một lý gì để một người nào đó không có điều gì muốn gửi tới chính mình nhiều năm sau. Và Hải cũng không ngoại lệ.
+MrBeast có "Hi Me In 10 Years", IShowSpeed có "Hi Me In 3 Years", Miêu Công Tử có "999 lá thư gửi bản thân". Và Hải nghĩ rằng không có một lý do gì để một người nào đó không có điều gì muốn gửi tới chính mình nhiều năm sau. Và Hải cũng không ngoại lệ.
 ## Tiêu đề
 - Chủ đề: Thư gửi Hải tuổi 35
 - Người gửi: Hải tuổi 24
@@ -1627,7 +1627,7 @@
       <c r="L13" t="inlineStr">
         <is>
           <t>&lt;h1 id="gui-hai-tuoi-35"&gt;Gửi Hải tuổi 35&lt;/h1&gt;
-&lt;p&gt;MrBeast có "Hi Me In 10 Years", IShowSpeed có "Hi Me In 3 Years", Miêu Công Tử có "999 lá thư gửi bản thân". Và Hải nghĩ rằng không có một lý gì để một người nào đó không có điều gì muốn gửi tới chính mình nhiều năm sau. Và Hải cũng không ngoại lệ.&lt;/p&gt;
+&lt;p&gt;MrBeast có "Hi Me In 10 Years", IShowSpeed có "Hi Me In 3 Years", Miêu Công Tử có "999 lá thư gửi bản thân". Và Hải nghĩ rằng không có một lý do gì để một người nào đó không có điều gì muốn gửi tới chính mình nhiều năm sau. Và Hải cũng không ngoại lệ.&lt;/p&gt;
 &lt;h2 id="tieu-e"&gt;Tiêu đề&lt;/h2&gt;
 &lt;ul&gt;
 &lt;li&gt;Chủ đề: Thư gửi Hải tuổi 35&lt;/li&gt;

</xml_diff>

<commit_message>
Gui Hai tuoi 35 edit 2
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -1620,7 +1620,7 @@
 Tôi nghĩ rằng với tính cách của cậu, cậu sẽ muốn đi xa - và sẽ đi xa. Cậu không muốn ai đó đến và nói với cậu rằng cậu không được phép làm thế hay cậu không có quyền làm điều đó. Và vì vậy thứ mà tôi muốn nói với cậu là sự trở về. Nghĩa vụ của cậu là sự trở về! 
 Nếu cậu đang sinh sống và làm việc ở nước ngoài mà xảy ra bất ổn, cậu có nghĩa vụ phải tìm cách liên lạc với lãnh sự quán để thực hiện quyền bảo hộ công dân. Nếu cậu đang ở ngoài khơi và gặp nạn, cậu phải bám lấy chiếc phao và giữ chặt lấy nó tới khi lên được con tàu trở về. Nếu cậu đã đạt được mục đích hoặc sự thành công ở ngoài kia, cậu cần phải trở về. Nghĩa vụ của cậu là trở về. Trở về là nghĩa vụ của cậu. 
 Chúc cậu đạt được điều những điều mình muốn và mang chúng trở về!
-God blessing you,
+God bless you,
 Hải tuổi 24./</t>
         </is>
       </c>
@@ -1653,7 +1653,7 @@
 &lt;p&gt;Tôi nghĩ rằng với tính cách của cậu, cậu sẽ muốn đi xa - và sẽ đi xa. Cậu không muốn ai đó đến và nói với cậu rằng cậu không được phép làm thế hay cậu không có quyền làm điều đó. Và vì vậy thứ mà tôi muốn nói với cậu là sự trở về. Nghĩa vụ của cậu là sự trở về! &lt;/p&gt;
 &lt;p&gt;Nếu cậu đang sinh sống và làm việc ở nước ngoài mà xảy ra bất ổn, cậu có nghĩa vụ phải tìm cách liên lạc với lãnh sự quán để thực hiện quyền bảo hộ công dân. Nếu cậu đang ở ngoài khơi và gặp nạn, cậu phải bám lấy chiếc phao và giữ chặt lấy nó tới khi lên được con tàu trở về. Nếu cậu đã đạt được mục đích hoặc sự thành công ở ngoài kia, cậu cần phải trở về. Nghĩa vụ của cậu là trở về. Trở về là nghĩa vụ của cậu. &lt;/p&gt;
 &lt;p&gt;Chúc cậu đạt được điều những điều mình muốn và mang chúng trở về!&lt;/p&gt;
-&lt;p&gt;God blessing you,&lt;/p&gt;
+&lt;p&gt;God bless you,&lt;/p&gt;
 &lt;p&gt;Hải tuổi 24./&lt;/p&gt;</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Gui Hai tuoi 35 edit 3
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -1619,7 +1619,7 @@
 Hỏi thăm cậu vậy đủ rồi, giờ đến lượt tôi nói. Chắc cậu cũng biết 10 năm qua tôi cũng đã có khá nhiều sự thay đổi - và thế giới xung quanh tôi cũng thế. Có những lần tôi trở về, một số người vẫn nhận ra tôi. Cô bán tạp hóa, anh cắt tóc cũng nhận ra tôi. Bạn bè thầy cô vẫn nhận ra tôi. Họ liên tục hỏi tôi thế nào và nhắc lại tôi của 10 năm trước. Họ biết tôi qua đâu, họ biết tôi thế nào, họ biết tôi ra làm sao?
 Tôi nghĩ rằng với tính cách của cậu, cậu sẽ muốn đi xa - và sẽ đi xa. Cậu không muốn ai đó đến và nói với cậu rằng cậu không được phép làm thế hay cậu không có quyền làm điều đó. Và vì vậy thứ mà tôi muốn nói với cậu là sự trở về. Nghĩa vụ của cậu là sự trở về! 
 Nếu cậu đang sinh sống và làm việc ở nước ngoài mà xảy ra bất ổn, cậu có nghĩa vụ phải tìm cách liên lạc với lãnh sự quán để thực hiện quyền bảo hộ công dân. Nếu cậu đang ở ngoài khơi và gặp nạn, cậu phải bám lấy chiếc phao và giữ chặt lấy nó tới khi lên được con tàu trở về. Nếu cậu đã đạt được mục đích hoặc sự thành công ở ngoài kia, cậu cần phải trở về. Nghĩa vụ của cậu là trở về. Trở về là nghĩa vụ của cậu. 
-Chúc cậu đạt được điều những điều mình muốn và mang chúng trở về!
+Chúc cậu đạt được những điều mình muốn và mang chúng trở về!
 God bless you,
 Hải tuổi 24./</t>
         </is>
@@ -1652,7 +1652,7 @@
 &lt;p&gt;Hỏi thăm cậu vậy đủ rồi, giờ đến lượt tôi nói. Chắc cậu cũng biết 10 năm qua tôi cũng đã có khá nhiều sự thay đổi - và thế giới xung quanh tôi cũng thế. Có những lần tôi trở về, một số người vẫn nhận ra tôi. Cô bán tạp hóa, anh cắt tóc cũng nhận ra tôi. Bạn bè thầy cô vẫn nhận ra tôi. Họ liên tục hỏi tôi thế nào và nhắc lại tôi của 10 năm trước. Họ biết tôi qua đâu, họ biết tôi thế nào, họ biết tôi ra làm sao?&lt;/p&gt;
 &lt;p&gt;Tôi nghĩ rằng với tính cách của cậu, cậu sẽ muốn đi xa - và sẽ đi xa. Cậu không muốn ai đó đến và nói với cậu rằng cậu không được phép làm thế hay cậu không có quyền làm điều đó. Và vì vậy thứ mà tôi muốn nói với cậu là sự trở về. Nghĩa vụ của cậu là sự trở về! &lt;/p&gt;
 &lt;p&gt;Nếu cậu đang sinh sống và làm việc ở nước ngoài mà xảy ra bất ổn, cậu có nghĩa vụ phải tìm cách liên lạc với lãnh sự quán để thực hiện quyền bảo hộ công dân. Nếu cậu đang ở ngoài khơi và gặp nạn, cậu phải bám lấy chiếc phao và giữ chặt lấy nó tới khi lên được con tàu trở về. Nếu cậu đã đạt được mục đích hoặc sự thành công ở ngoài kia, cậu cần phải trở về. Nghĩa vụ của cậu là trở về. Trở về là nghĩa vụ của cậu. &lt;/p&gt;
-&lt;p&gt;Chúc cậu đạt được điều những điều mình muốn và mang chúng trở về!&lt;/p&gt;
+&lt;p&gt;Chúc cậu đạt được những điều mình muốn và mang chúng trở về!&lt;/p&gt;
 &lt;p&gt;God bless you,&lt;/p&gt;
 &lt;p&gt;Hải tuổi 24./&lt;/p&gt;</t>
         </is>

</xml_diff>

<commit_message>
Kinh nghiem build SaaS
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -1888,10 +1888,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>in-draft</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Công nghệ</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
@@ -1905,12 +1909,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>21-09-2026</t>
+          <t>30-09-2026</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>- [ ] Xác định chi phí</t>
+          <t>Nếu phải nói rằng ngành công nghiệp nào phát triển mạnh mẽ nhất và thay đổi nhiều nhất trong vòng 10 năm trở lại đây, Hải nghĩ đó là ngành công nghiệp phần mềm dịch vụ hay còn được biết đến với tên gọi SaaS (Software-as-a-Service). Cổ phiếu...</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1921,25 +1925,114 @@
       <c r="K16" t="inlineStr">
         <is>
           <t># Kinh nghiệm build SaaS
-- [ ] Xác định chi phí
-- [ ] Quan sát trải nghiệm người dùng
-- [ ] Bạn muốn giỏi cái gì thì phải nói và thảo luận nhiều về cái đó</t>
+Nếu phải nói rằng ngành công nghiệp nào phát triển mạnh mẽ nhất và thay đổi nhiều nhất trong vòng 10 năm trở lại đây, Hải nghĩ đó là ngành công nghiệp phần mềm dịch vụ hay còn được biết đến với tên gọi SaaS (Software-as-a-Service). Cổ phiếu của những công ty phần mềm tăng từ 5-10 lần bất chấp có thời điểm kinh tế suy thoái do tác động của dịch bệnh và chiến tranh. Các công ty start-up công nghệ mới liên tục ra đời và được định giá với những con số không tưởng, điển hình là OpenAI, Anthropic, Anysphere. 
+## Thay đổi của SaaS trong 10 năm
+Xu hướng chung về số lượng phần mềm dịch vụ ra đời cũng như lượng người dùng phần lớn là tăng trưởng. Nhờ vào việc SaaS được triển khai trên Cloud, các cá nhân hoặc doanh nghiệp làm SaaS có thể nhanh chóng thực hiện chỉnh sửa để thích nghi với sự thay đổi của người dùng. 
+Thống kê từ Exploding Topics [^1] cuối 2026 chỉ ra trung bình mỗi người dành 4 giờ 37 phút mỗi ngày để dùng điện thoại. Mỗi ngày, mỗi người dùng mở điện thoại khoảng 58 lần: 3 lần để sử dụng trên 10 phút, 40 lần để kiểm tra thông báo nhanh dưới 2 phút. 52% khoảng thời gian check điện thoại mỗi tháng diễn ra trong giờ làm việc. 
+Nhiều thống kê khác nhau tại Việt Nam cũng chỉ ra thời lượng sử dụng điện thoại trung bình của người Việt là từ 6-8 tiếng mỗi ngày, thậm chí có bài báo giật tít tiêu đề từ 9-13 tiếng. Nói như vậy để hiểu nhu cầu thực cho ngành phần mềm và Internet nói chung vẫn là **rất lớn**.
+### Hướng tới mô hình trả phí để nhận một số đặc quyền (freemium)
+Đây là điều dễ thấy nhất hiện nay. SaaS được nhắc tới nhiều nhất về việc này có lẽ là Youtube khi ra mắt tính năng Premium để tắt quảng cáo. Và điều này cũng từng gây ra tranh cãi khi nhiều người cho rằng họ tự tạo ra vấn đề là chèn thêm quảng cáo và bán giải pháp để giải quyết vấn đề do chính họ tạo ra. Nhưng nhìn chung, khi nhắc tới trải nghiệm người dùng, mỗi người sẽ có cảm nhận khác nhau về việc có đáng xuống tiền hay không?
+Cho tới ngày nay, hầu hết các SaaS sẽ tìm cách thu phí của người dùng theo cách này hoặc cách khác. Từ ứng dụng chỉnh sửa ảnh, quản lý tài liệu / nội dung, từ các app môi giới như việc làm hay ứng dụng hẹn hò cho tới mạng xã hội. Có thể là dùng nhiêu trả nhiêu (Pay-as-you-go) hoặc là đăng ký thuê bao (Subscription).
+Và sẽ thật thiếu xót nếu như không nói về việc Duolingo cũng lựa chọn tư bản hóa giáo dục. Bạn sẽ bị hạn chế nội dung hoặc thời lượng nếu như bạn không mua các gói tháng/năm do cú xanh đề xuất. Nhưng biết sao được, ai cũng cần phải ăn cơm mà - có lẽ doanh thu từ quảng cáo là chưa đủ. 
+### SaaS ngày càng ứng dụng AI nhiều hơn
+Đây là điều không cần phải bàn cãi. AI dù còn nhiều thiếu sót nhưng chúng làm rất tốt từ việc lập lịch, đặt lịch, tự động hóa, hỗ trợ hoàn thiện nội dung cho tới việc làm trợ lý toàn thời gian. CRM, ERP bây giờ cần AI. Các ứng dụng văn phòng cần AI. Các kỹ sư từ khắp các ngành nghề khác nhau cần AI. Sự ra đời của ChatGPT, sau đó kéo theo sự ra đời của hàng loạt LLM và AI Agents khác thực sự đã làm thay đổi mọi thứ không chỉ riêng SaaS.
+## Trải nghiệm cá nhân trong gần 10 năm
+### Rào cản khi Hải mới chập chững làm SaaS
+Hầu hết mọi người đều học code từ những khung đen Console - Hải cũng vậy. Quay lại 8 năm trước, học ngôn ngữ gì, framework gì đã là một rào cản. Bởi vì có quá nhiều lựa chọn khi xét tới việc chúng làm được gì, mất bao lâu để học, chi phí để triển khai một ứng dụng hoàn chỉnh là bao nhiêu? Chúng có hỗ trợ trên hệ điều hành X hay không? Để đóng gói mã nguồn thành file cài đặt thì phải làm sao, mất bao nhiêu tiền? Thương mại hóa chúng thế nào? Có sợ bị ăn cắp mã nguồn không? Code có tối ưu về mặt hiệu năng hay không?
+Thời điểm đó, việc cân nhắc lựa chọn thuê cloud hay host cho rẻ và có nên cúng tiền cho domain hay không cũng đã là vấn đề lớn với Hải. Có quá nhiều ngôn ngữ, framework cho tới công ty cung cấp giải pháp điện toán và offer nhiều mức giá khác nhau. Không trả lời được câu hỏi này thì mã nguồn chỉ có thể chạy local và đưa lên Github. Còn nếu tự build server? - Tiền điện 24/7 và tiền mua hardware có khi còn mắc hơn!
+Theo trải nghiệm của Hải, vấn đề tích hợp từ giải pháp từ bên ngoài cũng là trở ngại. Nhẹ nhất là kết nối .NET với máy in qua thư viện để xuất báo cáo, máy scan để đọc barcode. Nặng hơn là làm sao để liên hệ với hàng loạt ngân hàng hoặc khác nhau để gom chung về 1 cổng thanh toán?
+### Thay đổi từ "công nhân viết code" sang "kỹ sư phần mềm"
+Nếu như trước đây, việc dành ra 1 buổi đi cafe nói chuyện với ai đó sẽ lấy đi thời gian làm SaaS của Hải thì bây giờ Hải đã có thể vừa cafe trò chuyện, vừa build SaaS. Thậm chí, Hải có thể nhanh chóng thay đổi hoặc bổ sung thêm tính năng gì đó mới đến từ cuộc trò chuyện với người khác. Quả thật AI đã có thể viết code, review và tự test nhanh và tốt hơn 1 Dev trình độ Junior. Việc của Hải chỉ đơn giản là quản lý tốt context, kiến trúc và cấp quyền cho Agents. 
+**Nói nhiều hơn về nhu cầu và trải nghiệm người dùng thay vì code**
+Thực lực của Hải hiện tại cộng với sự giúp sức của 1 AI agent hoàn toàn có thể cho ra 1-2 SaaS mới mỗi tuần. Nếu bạn không thấy SaaS mới từ Hải sau 1 tháng, hoặc là Hải đang tập trung cải thiện trải nghiệm người dùng của các SaaS cũ, hoặc là Hải đang bí ý tưởng, hoặc cũng còn một khả năng khác cao hơn là hết tiền làm SaaS. 
+Rõ ràng các AI Agent như Cursor và Claude ngày nay có thể nhanh chóng code giao diện, thiết kế và kết nối cơ sở dữ liệu. Điều đó làm giảm đáng kể thời gian phát triển và triển khai ứng dụng. Vì vậy, nếu phải nói một câu công bằng - thì các SaaS hơn nhau ở việc hiểu người dùng chứ không phải là độ dài của mã nguồn. Vì vậy, phần lớn thời gian dành cho xây dựng SaaS ngày nay nên đến từ việc:
+1. Xác định vấn đề và nhu cầu người dùng để tìm kiếm cửa sổ cơ hội và thị trường đủ lớn.
+2. Quản lý tốt context để build SaaS nhanh chóng (tham khảo Mô hình Canvas và ứng dụng CaaS - Lean2Pitch [^2])
+3. Thu thập trải nghiệm của người dùng để cải tiến ứng dụng (tiếp tục lặp đi lặp lại)
+## SaaS thực dụng: Chi phí và doanh thu
+Nhớ nhé, cái gì bạn không tự làm được mà phải nhờ đến người khác (hoặc đã ăn độc quyền) thì đó là chi phí. Còn những gì bạn tự làm được nhưng vẫn phải bỏ thời gian thì đó vẫn là chi phí - nhưng nếu bạn thấy đáng thì vẫn sẽ làm (miễn là còn gồng được). Một số chi phí làm SaaS mà anh em có thể phải đối mặt:
+- Phát triển, bảo trì và cải tiến SaaS
+- Hosting, lưu trữ, CDN
+- Tên miền, công cụ vận hành và bản quyền tài nguyên
+- SEO, quảng cáo để tiếp cận người dùng
+- Hỗ trợ người dùng và phí thanh toán nếu áp dụng gói trả phí
+Còn về doanh thu, khả năng cao chúng sẽ đến từ quảng cáo, các offer trả phí khác nhau. Vì thế, nếu không có inverstors, rất có thể anh em sẽ đói trong giai đoạn đầu làm SaaS đấy!
+**Không tham vọng lớn khi nguồn lực nhỏ!**
+Một trong những tham vọng dẫn tới thất bại phổ biến nhất của người mới bắt đầu làm SaaS đó là làm mạng xã hội. Đã rất nhiều công ty lớn nhỏ khác nhau thất bại và quay xe ở mảng này. Tại sao phải làm mạng xã hội? Mạng xã hội bạn đưa ra giải quyết vấn đề gì mà các mạng xã hội hiện tại chưa có? Bạn đã tính tới các chi phí để có hệ thống chưa? Bạn đã tính tới chi phí để có được người dùng, chi phí để giữ ngọn lửa kết nối và tương tác của người dùng chưa? Bạn đã tính tới chi phí để có được lượng nội dung đầy đặn, đa dạng và thuật toán phân phối chúng hiệu quả chưa? Bạn đã tính tới chi phí để giải quyết các vấn đề pháp lý do "nội dung sáng tạo" từ người dùng tạo ra chưa?
+Có thể bạn không tin nhưng hồi còn là sinh viên năm 2, Hải đã từng lóe lên ý tưởng làm mạng xã hội khuyến khích người dùng chia sẻ ý tưởng, phản biện ngay cả khi ý tưởng mới hình thành và còn sơ khai bởi vì AI sẽ được tích hợp để hỗ trợ trả lời bên dưới bài đăng khi bạn hỏi. Ý tưởng khá giống mạng xã hội Thread này xuất hiện vào năm 2021 (trước khi Thread ra đời được 2 năm) khi Hải nhìn thấy tính năng bình luận trên Facebook và Youtube chỉ chấp nhận tối đa 2 lớp phản hồi và không cho phép tự bình luận khi nội dung chưa được tạo. Hải từng đặt tên cho nó là "Vô tri" - nhưng tất nhiên là Hải đã nhanh chóng dừng lại vì chưa trả lời được hết những câu hỏi ở bên trên. 
+## Tập trung cho ý tưởng và trải nghiệm người dùng
+SaaS ngày nay đã build dễ hơn 5-10 năm trước rất nhiều rồi. Vì thế, hãy cố gắng khai thác nhu cầu, vấn dề, sự bất tiện, sự khó chịu của người khác. Chúng xuất hiện ở khắp mọi nơi từ ngoài đời đến Internet. Chúng mới là động lực để bạn làm SaaS. Hãy cố gắng đưa ra lời đề nghị người khác dùng SaaS của bạn và ngày càng nhiều hơn. Quan sát xem khi họ dùng SaaS, mắt họ tập trung vào đâu, tay họ thao tác như thế nào, họ tương tác và phản hồi ra làm sao. Những thứ đó sẽ khiến cho SaaS của bạn ngày càng phát triển và trở nên cạnh tranh hơn.
+## Muốn giỏi cái gì thì hãy nói nhiều về nó
+Cách hiệu quả nhất để giỏi lên - bất kể thứ đó là gì - chính là trao đổi nhiều về nó. Đó là lắng nghe và ghi nhận nhiều luồng ý kiến của nhiều người khác nhau, trao đổi và tương tác với họ. Hỏi họ và xem họ đáp gì và khuyến khích họ làm điều ngược lại. Dù cho bạn đang ở bất kỳ giai đoạn nào của quá trình làm SaaS (học công nghệ - tìm kiếm vấn đề và giải pháp - phát triển sản phẩm - thử nghiệm sản phẩm). Bạn nên - kể cả người bạn đối thoại có là học sinh / sinh viên, người lao động, nhân viên văn phòng - miễn là họ đã có nhiều trải nghiệm ứng dụng và có khả năng thụ hưởng giá trị từ SaaS mới!
+Không nhất thiết phải là kỹ sư phần mềm hạng ưu thì mới có đặc quyền được nói về SaaS - hoàn toàn không! Bạn xuất hiện với tư cách là người dùng, như thế đã là quá đủ. Bản thân SaaS không phải là thứ bị cô lập bởi đội ngũ phát triển. SaaS trở nên hữu ích và có giá trị là bởi vì được sử dụng để giải quyết vấn đề và được quan tâm bởi nhiều người - từ đó mang lại doanh thu cho đội ngũ phát triển.
+[^1]: [Time Spent Using Smartphones (2026 Statistics) by Fabio Duarte](https://explodingtopics.com/blog/smartphone-usage-stats)
+[^2]: Quý Hải Ng, "Bộ khung Canvas tinh gọn," Hải có gì hay, 2026. https://haicogihay.com/blog/bo-khung-canvas-tinh-gon.html</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>&lt;h1 id="kinh-nghiem-build-saas"&gt;Kinh nghiệm build SaaS&lt;/h1&gt;
-&lt;ul class="task-list"&gt;
-&lt;li class="task-list-item"&gt;
-&lt;p&gt;&lt;input type="checkbox"/&gt; Xác định chi phí&lt;/p&gt;
+&lt;p&gt;Nếu phải nói rằng ngành công nghiệp nào phát triển mạnh mẽ nhất và thay đổi nhiều nhất trong vòng 10 năm trở lại đây, Hải nghĩ đó là ngành công nghiệp phần mềm dịch vụ hay còn được biết đến với tên gọi SaaS (Software-as-a-Service). Cổ phiếu của những công ty phần mềm tăng từ 5-10 lần bất chấp có thời điểm kinh tế suy thoái do tác động của dịch bệnh và chiến tranh. Các công ty start-up công nghệ mới liên tục ra đời và được định giá với những con số không tưởng, điển hình là OpenAI, Anthropic, Anysphere. &lt;/p&gt;
+&lt;h2 id="thay-oi-cua-saas-trong-10-nam"&gt;Thay đổi của SaaS trong 10 năm&lt;/h2&gt;
+&lt;p&gt;Xu hướng chung về số lượng phần mềm dịch vụ ra đời cũng như lượng người dùng phần lớn là tăng trưởng. Nhờ vào việc SaaS được triển khai trên Cloud, các cá nhân hoặc doanh nghiệp làm SaaS có thể nhanh chóng thực hiện chỉnh sửa để thích nghi với sự thay đổi của người dùng. &lt;/p&gt;
+&lt;p&gt;Thống kê từ Exploding Topics &lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt; cuối 2026 chỉ ra trung bình mỗi người dành 4 giờ 37 phút mỗi ngày để dùng điện thoại. Mỗi ngày, mỗi người dùng mở điện thoại khoảng 58 lần: 3 lần để sử dụng trên 10 phút, 40 lần để kiểm tra thông báo nhanh dưới 2 phút. 52% khoảng thời gian check điện thoại mỗi tháng diễn ra trong giờ làm việc. &lt;/p&gt;
+&lt;p&gt;Nhiều thống kê khác nhau tại Việt Nam cũng chỉ ra thời lượng sử dụng điện thoại trung bình của người Việt là từ 6-8 tiếng mỗi ngày, thậm chí có bài báo giật tít tiêu đề từ 9-13 tiếng. Nói như vậy để hiểu nhu cầu thực cho ngành phần mềm và Internet nói chung vẫn là &lt;strong&gt;rất lớn&lt;/strong&gt;.&lt;/p&gt;
+&lt;h3 id="huong-toi-mo-hinh-tra-phi-e-nhan-mot-so-ac-quyen-freemium"&gt;Hướng tới mô hình trả phí để nhận một số đặc quyền (freemium)&lt;/h3&gt;
+&lt;p&gt;Đây là điều dễ thấy nhất hiện nay. SaaS được nhắc tới nhiều nhất về việc này có lẽ là Youtube khi ra mắt tính năng Premium để tắt quảng cáo. Và điều này cũng từng gây ra tranh cãi khi nhiều người cho rằng họ tự tạo ra vấn đề là chèn thêm quảng cáo và bán giải pháp để giải quyết vấn đề do chính họ tạo ra. Nhưng nhìn chung, khi nhắc tới trải nghiệm người dùng, mỗi người sẽ có cảm nhận khác nhau về việc có đáng xuống tiền hay không?&lt;/p&gt;
+&lt;p&gt;Cho tới ngày nay, hầu hết các SaaS sẽ tìm cách thu phí của người dùng theo cách này hoặc cách khác. Từ ứng dụng chỉnh sửa ảnh, quản lý tài liệu / nội dung, từ các app môi giới như việc làm hay ứng dụng hẹn hò cho tới mạng xã hội. Có thể là dùng nhiêu trả nhiêu (Pay-as-you-go) hoặc là đăng ký thuê bao (Subscription).&lt;/p&gt;
+&lt;p&gt;Và sẽ thật thiếu xót nếu như không nói về việc Duolingo cũng lựa chọn tư bản hóa giáo dục. Bạn sẽ bị hạn chế nội dung hoặc thời lượng nếu như bạn không mua các gói tháng/năm do cú xanh đề xuất. Nhưng biết sao được, ai cũng cần phải ăn cơm mà - có lẽ doanh thu từ quảng cáo là chưa đủ. &lt;/p&gt;
+&lt;h3 id="saas-ngay-cang-ung-dung-ai-nhieu-hon"&gt;SaaS ngày càng ứng dụng AI nhiều hơn&lt;/h3&gt;
+&lt;p&gt;Đây là điều không cần phải bàn cãi. AI dù còn nhiều thiếu sót nhưng chúng làm rất tốt từ việc lập lịch, đặt lịch, tự động hóa, hỗ trợ hoàn thiện nội dung cho tới việc làm trợ lý toàn thời gian. CRM, ERP bây giờ cần AI. Các ứng dụng văn phòng cần AI. Các kỹ sư từ khắp các ngành nghề khác nhau cần AI. Sự ra đời của ChatGPT, sau đó kéo theo sự ra đời của hàng loạt LLM và AI Agents khác thực sự đã làm thay đổi mọi thứ không chỉ riêng SaaS.&lt;/p&gt;
+&lt;h2 id="trai-nghiem-ca-nhan-trong-gan-10-nam"&gt;Trải nghiệm cá nhân trong gần 10 năm&lt;/h2&gt;
+&lt;h3 id="rao-can-khi-hai-moi-chap-chung-lam-saas"&gt;Rào cản khi Hải mới chập chững làm SaaS&lt;/h3&gt;
+&lt;p&gt;Hầu hết mọi người đều học code từ những khung đen Console - Hải cũng vậy. Quay lại 8 năm trước, học ngôn ngữ gì, framework gì đã là một rào cản. Bởi vì có quá nhiều lựa chọn khi xét tới việc chúng làm được gì, mất bao lâu để học, chi phí để triển khai một ứng dụng hoàn chỉnh là bao nhiêu? Chúng có hỗ trợ trên hệ điều hành X hay không? Để đóng gói mã nguồn thành file cài đặt thì phải làm sao, mất bao nhiêu tiền? Thương mại hóa chúng thế nào? Có sợ bị ăn cắp mã nguồn không? Code có tối ưu về mặt hiệu năng hay không?&lt;/p&gt;
+&lt;p&gt;Thời điểm đó, việc cân nhắc lựa chọn thuê cloud hay host cho rẻ và có nên cúng tiền cho domain hay không cũng đã là vấn đề lớn với Hải. Có quá nhiều ngôn ngữ, framework cho tới công ty cung cấp giải pháp điện toán và offer nhiều mức giá khác nhau. Không trả lời được câu hỏi này thì mã nguồn chỉ có thể chạy local và đưa lên Github. Còn nếu tự build server? - Tiền điện 24/7 và tiền mua hardware có khi còn mắc hơn!&lt;/p&gt;
+&lt;p&gt;Theo trải nghiệm của Hải, vấn đề tích hợp từ giải pháp từ bên ngoài cũng là trở ngại. Nhẹ nhất là kết nối .NET với máy in qua thư viện để xuất báo cáo, máy scan để đọc barcode. Nặng hơn là làm sao để liên hệ với hàng loạt ngân hàng hoặc khác nhau để gom chung về 1 cổng thanh toán?&lt;/p&gt;
+&lt;h3 id="thay-oi-tu-cong-nhan-viet-code-sang-ky-su-phan-mem"&gt;Thay đổi từ "công nhân viết code" sang "kỹ sư phần mềm"&lt;/h3&gt;
+&lt;p&gt;Nếu như trước đây, việc dành ra 1 buổi đi cafe nói chuyện với ai đó sẽ lấy đi thời gian làm SaaS của Hải thì bây giờ Hải đã có thể vừa cafe trò chuyện, vừa build SaaS. Thậm chí, Hải có thể nhanh chóng thay đổi hoặc bổ sung thêm tính năng gì đó mới đến từ cuộc trò chuyện với người khác. Quả thật AI đã có thể viết code, review và tự test nhanh và tốt hơn 1 Dev trình độ Junior. Việc của Hải chỉ đơn giản là quản lý tốt context, kiến trúc và cấp quyền cho Agents. &lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Nói nhiều hơn về nhu cầu và trải nghiệm người dùng thay vì code&lt;/strong&gt;&lt;/p&gt;
+&lt;p&gt;Thực lực của Hải hiện tại cộng với sự giúp sức của 1 AI agent hoàn toàn có thể cho ra 1-2 SaaS mới mỗi tuần. Nếu bạn không thấy SaaS mới từ Hải sau 1 tháng, hoặc là Hải đang tập trung cải thiện trải nghiệm người dùng của các SaaS cũ, hoặc là Hải đang bí ý tưởng, hoặc cũng còn một khả năng khác cao hơn là hết tiền làm SaaS. &lt;/p&gt;
+&lt;p&gt;Rõ ràng các AI Agent như Cursor và Claude ngày nay có thể nhanh chóng code giao diện, thiết kế và kết nối cơ sở dữ liệu. Điều đó làm giảm đáng kể thời gian phát triển và triển khai ứng dụng. Vì vậy, nếu phải nói một câu công bằng - thì các SaaS hơn nhau ở việc hiểu người dùng chứ không phải là độ dài của mã nguồn. Vì vậy, phần lớn thời gian dành cho xây dựng SaaS ngày nay nên đến từ việc:&lt;/p&gt;
+&lt;ol&gt;
+&lt;li&gt;
+&lt;p&gt;Xác định vấn đề và nhu cầu người dùng để tìm kiếm cửa sổ cơ hội và thị trường đủ lớn.&lt;/p&gt;
 &lt;/li&gt;
-&lt;li class="task-list-item"&gt;
-&lt;p&gt;&lt;input type="checkbox"/&gt; Quan sát trải nghiệm người dùng&lt;/p&gt;
+&lt;li&gt;
+&lt;p&gt;Quản lý tốt context để build SaaS nhanh chóng (tham khảo Mô hình Canvas và ứng dụng CaaS - Lean2Pitch &lt;sup id="fnref:2"&gt;&lt;a class="footnote-ref" href="#fn:2"&gt;2&lt;/a&gt;&lt;/sup&gt;)&lt;/p&gt;
 &lt;/li&gt;
-&lt;li class="task-list-item"&gt;
-&lt;p&gt;&lt;input type="checkbox"/&gt; Bạn muốn giỏi cái gì thì phải nói và thảo luận nhiều về cái đó&lt;/p&gt;
+&lt;li&gt;
+&lt;p&gt;Thu thập trải nghiệm của người dùng để cải tiến ứng dụng (tiếp tục lặp đi lặp lại)&lt;/p&gt;
 &lt;/li&gt;
-&lt;/ul&gt;</t>
+&lt;/ol&gt;
+&lt;h2 id="saas-thuc-dung-chi-phi-va-doanh-thu"&gt;SaaS thực dụng: Chi phí và doanh thu&lt;/h2&gt;
+&lt;p&gt;Nhớ nhé, cái gì bạn không tự làm được mà phải nhờ đến người khác (hoặc đã ăn độc quyền) thì đó là chi phí. Còn những gì bạn tự làm được nhưng vẫn phải bỏ thời gian thì đó vẫn là chi phí - nhưng nếu bạn thấy đáng thì vẫn sẽ làm (miễn là còn gồng được). Một số chi phí làm SaaS mà anh em có thể phải đối mặt:&lt;/p&gt;
+&lt;ul&gt;
+&lt;li&gt;Phát triển, bảo trì và cải tiến SaaS&lt;/li&gt;
+&lt;li&gt;Hosting, lưu trữ, CDN&lt;/li&gt;
+&lt;li&gt;Tên miền, công cụ vận hành và bản quyền tài nguyên&lt;/li&gt;
+&lt;li&gt;SEO, quảng cáo để tiếp cận người dùng&lt;/li&gt;
+&lt;li&gt;Hỗ trợ người dùng và phí thanh toán nếu áp dụng gói trả phí&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;Còn về doanh thu, khả năng cao chúng sẽ đến từ quảng cáo, các offer trả phí khác nhau. Vì thế, nếu không có inverstors, rất có thể anh em sẽ đói trong giai đoạn đầu làm SaaS đấy!&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Không tham vọng lớn khi nguồn lực nhỏ!&lt;/strong&gt;&lt;/p&gt;
+&lt;p&gt;Một trong những tham vọng dẫn tới thất bại phổ biến nhất của người mới bắt đầu làm SaaS đó là làm mạng xã hội. Đã rất nhiều công ty lớn nhỏ khác nhau thất bại và quay xe ở mảng này. Tại sao phải làm mạng xã hội? Mạng xã hội bạn đưa ra giải quyết vấn đề gì mà các mạng xã hội hiện tại chưa có? Bạn đã tính tới các chi phí để có hệ thống chưa? Bạn đã tính tới chi phí để có được người dùng, chi phí để giữ ngọn lửa kết nối và tương tác của người dùng chưa? Bạn đã tính tới chi phí để có được lượng nội dung đầy đặn, đa dạng và thuật toán phân phối chúng hiệu quả chưa? Bạn đã tính tới chi phí để giải quyết các vấn đề pháp lý do "nội dung sáng tạo" từ người dùng tạo ra chưa?&lt;/p&gt;
+&lt;p&gt;Có thể bạn không tin nhưng hồi còn là sinh viên năm 2, Hải đã từng lóe lên ý tưởng làm mạng xã hội khuyến khích người dùng chia sẻ ý tưởng, phản biện ngay cả khi ý tưởng mới hình thành và còn sơ khai bởi vì AI sẽ được tích hợp để hỗ trợ trả lời bên dưới bài đăng khi bạn hỏi. Ý tưởng khá giống mạng xã hội Thread này xuất hiện vào năm 2021 (trước khi Thread ra đời được 2 năm) khi Hải nhìn thấy tính năng bình luận trên Facebook và Youtube chỉ chấp nhận tối đa 2 lớp phản hồi và không cho phép tự bình luận khi nội dung chưa được tạo. Hải từng đặt tên cho nó là "Vô tri" - nhưng tất nhiên là Hải đã nhanh chóng dừng lại vì chưa trả lời được hết những câu hỏi ở bên trên. &lt;/p&gt;
+&lt;h2 id="tap-trung-cho-y-tuong-va-trai-nghiem-nguoi-dung"&gt;Tập trung cho ý tưởng và trải nghiệm người dùng&lt;/h2&gt;
+&lt;p&gt;SaaS ngày nay đã build dễ hơn 5-10 năm trước rất nhiều rồi. Vì thế, hãy cố gắng khai thác nhu cầu, vấn dề, sự bất tiện, sự khó chịu của người khác. Chúng xuất hiện ở khắp mọi nơi từ ngoài đời đến Internet. Chúng mới là động lực để bạn làm SaaS. Hãy cố gắng đưa ra lời đề nghị người khác dùng SaaS của bạn và ngày càng nhiều hơn. Quan sát xem khi họ dùng SaaS, mắt họ tập trung vào đâu, tay họ thao tác như thế nào, họ tương tác và phản hồi ra làm sao. Những thứ đó sẽ khiến cho SaaS của bạn ngày càng phát triển và trở nên cạnh tranh hơn.&lt;/p&gt;
+&lt;h2 id="muon-gioi-cai-gi-thi-hay-noi-nhieu-ve-no"&gt;Muốn giỏi cái gì thì hãy nói nhiều về nó&lt;/h2&gt;
+&lt;p&gt;Cách hiệu quả nhất để giỏi lên - bất kể thứ đó là gì - chính là trao đổi nhiều về nó. Đó là lắng nghe và ghi nhận nhiều luồng ý kiến của nhiều người khác nhau, trao đổi và tương tác với họ. Hỏi họ và xem họ đáp gì và khuyến khích họ làm điều ngược lại. Dù cho bạn đang ở bất kỳ giai đoạn nào của quá trình làm SaaS (học công nghệ - tìm kiếm vấn đề và giải pháp - phát triển sản phẩm - thử nghiệm sản phẩm). Bạn nên - kể cả người bạn đối thoại có là học sinh / sinh viên, người lao động, nhân viên văn phòng - miễn là họ đã có nhiều trải nghiệm ứng dụng và có khả năng thụ hưởng giá trị từ SaaS mới!&lt;/p&gt;
+&lt;p&gt;Không nhất thiết phải là kỹ sư phần mềm hạng ưu thì mới có đặc quyền được nói về SaaS - hoàn toàn không! Bạn xuất hiện với tư cách là người dùng, như thế đã là quá đủ. Bản thân SaaS không phải là thứ bị cô lập bởi đội ngũ phát triển. SaaS trở nên hữu ích và có giá trị là bởi vì được sử dụng để giải quyết vấn đề và được quan tâm bởi nhiều người - từ đó mang lại doanh thu cho đội ngũ phát triển.&lt;/p&gt;
+&lt;div class="footnote"&gt;
+&lt;hr /&gt;
+&lt;ol&gt;
+&lt;li id="fn:1"&gt;
+&lt;p&gt;&lt;a href="https://explodingtopics.com/blog/smartphone-usage-stats"&gt;Time Spent Using Smartphones (2026 Statistics) by Fabio Duarte&lt;/a&gt;&amp;#160;&lt;a class="footnote-backref" href="#fnref:1" title="Jump back to footnote 1 in the text"&gt;&amp;#8617;&lt;/a&gt;&lt;/p&gt;
+&lt;/li&gt;
+&lt;li id="fn:2"&gt;
+&lt;p&gt;Quý Hải Ng, "Bộ khung Canvas tinh gọn," Hải có gì hay, 2026. https://haicogihay.com/blog/bo-khung-canvas-tinh-gon.html&amp;#160;&lt;a class="footnote-backref" href="#fnref:2" title="Jump back to footnote 2 in the text"&gt;&amp;#8617;&lt;/a&gt;&lt;/p&gt;
+&lt;/li&gt;
+&lt;/ol&gt;
+&lt;/div&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kinh nghiem build SaaS edited
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -1909,7 +1909,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>30-09-2026</t>
+          <t>01-10-2026</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1928,7 +1928,7 @@
 Nếu phải nói rằng ngành công nghiệp nào phát triển mạnh mẽ nhất và thay đổi nhiều nhất trong vòng 10 năm trở lại đây, Hải nghĩ đó là ngành công nghiệp phần mềm dịch vụ hay còn được biết đến với tên gọi SaaS (Software-as-a-Service). Cổ phiếu của những công ty phần mềm tăng từ 5-10 lần bất chấp có thời điểm kinh tế suy thoái do tác động của dịch bệnh và chiến tranh. Các công ty start-up công nghệ mới liên tục ra đời và được định giá với những con số không tưởng, điển hình là OpenAI, Anthropic, Anysphere. 
 ## Thay đổi của SaaS trong 10 năm
 Xu hướng chung về số lượng phần mềm dịch vụ ra đời cũng như lượng người dùng phần lớn là tăng trưởng. Nhờ vào việc SaaS được triển khai trên Cloud, các cá nhân hoặc doanh nghiệp làm SaaS có thể nhanh chóng thực hiện chỉnh sửa để thích nghi với sự thay đổi của người dùng. 
-Thống kê từ Exploding Topics [^1] cuối 2026 chỉ ra trung bình mỗi người dành 4 giờ 37 phút mỗi ngày để dùng điện thoại. Mỗi ngày, mỗi người dùng mở điện thoại khoảng 58 lần: 3 lần để sử dụng trên 10 phút, 40 lần để kiểm tra thông báo nhanh dưới 2 phút. 52% khoảng thời gian check điện thoại mỗi tháng diễn ra trong giờ làm việc. 
+Thống kê từ Exploding Topics cuối 2026 [^1] chỉ ra trung bình mỗi người dành 4 giờ 37 phút mỗi ngày để dùng điện thoại. Mỗi ngày, mỗi người dùng mở điện thoại khoảng 58 lần: 3 lần để sử dụng trên 10 phút, 40 lần để kiểm tra thông báo nhanh dưới 2 phút. 52% khoảng thời gian check điện thoại mỗi tháng diễn ra trong giờ làm việc. 
 Nhiều thống kê khác nhau tại Việt Nam cũng chỉ ra thời lượng sử dụng điện thoại trung bình của người Việt là từ 6-8 tiếng mỗi ngày, thậm chí có bài báo giật tít tiêu đề từ 9-13 tiếng. Nói như vậy để hiểu nhu cầu thực cho ngành phần mềm và Internet nói chung vẫn là **rất lớn**.
 ### Hướng tới mô hình trả phí để nhận một số đặc quyền (freemium)
 Đây là điều dễ thấy nhất hiện nay. SaaS được nhắc tới nhiều nhất về việc này có lẽ là Youtube khi ra mắt tính năng Premium để tắt quảng cáo. Và điều này cũng từng gây ra tranh cãi khi nhiều người cho rằng họ tự tạo ra vấn đề là chèn thêm quảng cáo và bán giải pháp để giải quyết vấn đề do chính họ tạo ra. Nhưng nhìn chung, khi nhắc tới trải nghiệm người dùng, mỗi người sẽ có cảm nhận khác nhau về việc có đáng xuống tiền hay không?
@@ -1940,7 +1940,7 @@
 ### Rào cản khi Hải mới chập chững làm SaaS
 Hầu hết mọi người đều học code từ những khung đen Console - Hải cũng vậy. Quay lại 8 năm trước, học ngôn ngữ gì, framework gì đã là một rào cản. Bởi vì có quá nhiều lựa chọn khi xét tới việc chúng làm được gì, mất bao lâu để học, chi phí để triển khai một ứng dụng hoàn chỉnh là bao nhiêu? Chúng có hỗ trợ trên hệ điều hành X hay không? Để đóng gói mã nguồn thành file cài đặt thì phải làm sao, mất bao nhiêu tiền? Thương mại hóa chúng thế nào? Có sợ bị ăn cắp mã nguồn không? Code có tối ưu về mặt hiệu năng hay không?
 Thời điểm đó, việc cân nhắc lựa chọn thuê cloud hay host cho rẻ và có nên cúng tiền cho domain hay không cũng đã là vấn đề lớn với Hải. Có quá nhiều ngôn ngữ, framework cho tới công ty cung cấp giải pháp điện toán và offer nhiều mức giá khác nhau. Không trả lời được câu hỏi này thì mã nguồn chỉ có thể chạy local và đưa lên Github. Còn nếu tự build server? - Tiền điện 24/7 và tiền mua hardware có khi còn mắc hơn!
-Theo trải nghiệm của Hải, vấn đề tích hợp từ giải pháp từ bên ngoài cũng là trở ngại. Nhẹ nhất là kết nối .NET với máy in qua thư viện để xuất báo cáo, máy scan để đọc barcode. Nặng hơn là làm sao để liên hệ với hàng loạt ngân hàng hoặc khác nhau để gom chung về 1 cổng thanh toán?
+Theo trải nghiệm của Hải, vấn đề tích hợp giải pháp từ bên ngoài cũng là trở ngại. Nhẹ nhất là kết nối .NET với máy in qua thư viện để xuất báo cáo, máy scan để đọc barcode. Nặng hơn là làm sao để liên hệ với hàng loạt ngân hàng khác nhau để gom chung về 1 cổng thanh toán?
 ### Thay đổi từ "công nhân viết code" sang "kỹ sư phần mềm"
 Nếu như trước đây, việc dành ra 1 buổi đi cafe nói chuyện với ai đó sẽ lấy đi thời gian làm SaaS của Hải thì bây giờ Hải đã có thể vừa cafe trò chuyện, vừa build SaaS. Thậm chí, Hải có thể nhanh chóng thay đổi hoặc bổ sung thêm tính năng gì đó mới đến từ cuộc trò chuyện với người khác. Quả thật AI đã có thể viết code, review và tự test nhanh và tốt hơn 1 Dev trình độ Junior. Việc của Hải chỉ đơn giản là quản lý tốt context, kiến trúc và cấp quyền cho Agents. 
 **Nói nhiều hơn về nhu cầu và trải nghiệm người dùng thay vì code**
@@ -1956,14 +1956,14 @@
 - Tên miền, công cụ vận hành và bản quyền tài nguyên
 - SEO, quảng cáo để tiếp cận người dùng
 - Hỗ trợ người dùng và phí thanh toán nếu áp dụng gói trả phí
-Còn về doanh thu, khả năng cao chúng sẽ đến từ quảng cáo, các offer trả phí khác nhau. Vì thế, nếu không có inverstors, rất có thể anh em sẽ đói trong giai đoạn đầu làm SaaS đấy!
+Còn về doanh thu, khả năng cao chúng sẽ đến từ quảng cáo, các offer trả phí khác nhau. Vì thế, nếu không có investors, rất có thể anh em sẽ đói trong giai đoạn đầu làm SaaS đấy!
 **Không tham vọng lớn khi nguồn lực nhỏ!**
 Một trong những tham vọng dẫn tới thất bại phổ biến nhất của người mới bắt đầu làm SaaS đó là làm mạng xã hội. Đã rất nhiều công ty lớn nhỏ khác nhau thất bại và quay xe ở mảng này. Tại sao phải làm mạng xã hội? Mạng xã hội bạn đưa ra giải quyết vấn đề gì mà các mạng xã hội hiện tại chưa có? Bạn đã tính tới các chi phí để có hệ thống chưa? Bạn đã tính tới chi phí để có được người dùng, chi phí để giữ ngọn lửa kết nối và tương tác của người dùng chưa? Bạn đã tính tới chi phí để có được lượng nội dung đầy đặn, đa dạng và thuật toán phân phối chúng hiệu quả chưa? Bạn đã tính tới chi phí để giải quyết các vấn đề pháp lý do "nội dung sáng tạo" từ người dùng tạo ra chưa?
 Có thể bạn không tin nhưng hồi còn là sinh viên năm 2, Hải đã từng lóe lên ý tưởng làm mạng xã hội khuyến khích người dùng chia sẻ ý tưởng, phản biện ngay cả khi ý tưởng mới hình thành và còn sơ khai bởi vì AI sẽ được tích hợp để hỗ trợ trả lời bên dưới bài đăng khi bạn hỏi. Ý tưởng khá giống mạng xã hội Thread này xuất hiện vào năm 2021 (trước khi Thread ra đời được 2 năm) khi Hải nhìn thấy tính năng bình luận trên Facebook và Youtube chỉ chấp nhận tối đa 2 lớp phản hồi và không cho phép tự bình luận khi nội dung chưa được tạo. Hải từng đặt tên cho nó là "Vô tri" - nhưng tất nhiên là Hải đã nhanh chóng dừng lại vì chưa trả lời được hết những câu hỏi ở bên trên. 
 ## Tập trung cho ý tưởng và trải nghiệm người dùng
-SaaS ngày nay đã build dễ hơn 5-10 năm trước rất nhiều rồi. Vì thế, hãy cố gắng khai thác nhu cầu, vấn dề, sự bất tiện, sự khó chịu của người khác. Chúng xuất hiện ở khắp mọi nơi từ ngoài đời đến Internet. Chúng mới là động lực để bạn làm SaaS. Hãy cố gắng đưa ra lời đề nghị người khác dùng SaaS của bạn và ngày càng nhiều hơn. Quan sát xem khi họ dùng SaaS, mắt họ tập trung vào đâu, tay họ thao tác như thế nào, họ tương tác và phản hồi ra làm sao. Những thứ đó sẽ khiến cho SaaS của bạn ngày càng phát triển và trở nên cạnh tranh hơn.
+SaaS ngày nay đã dễ build hơn 5-10 năm trước rất nhiều rồi. Vì thế, hãy cố gắng khai thác nhu cầu, vấn đề, sự bất tiện, sự khó chịu của người khác. Chúng xuất hiện ở khắp mọi nơi từ ngoài đời đến Internet. Chúng mới là động lực để bạn làm SaaS. Hãy cố gắng đưa ra lời đề nghị người khác dùng thử SaaS của bạn - và ngày càng nhiều hơn. Quan sát xem khi họ dùng SaaS, mắt họ tập trung vào đâu, tay họ thao tác như thế nào, họ tương tác và phản hồi ra làm sao. Những thứ đó sẽ khiến cho SaaS của bạn ngày càng phát triển và trở nên cạnh tranh hơn.
 ## Muốn giỏi cái gì thì hãy nói nhiều về nó
-Cách hiệu quả nhất để giỏi lên - bất kể thứ đó là gì - chính là trao đổi nhiều về nó. Đó là lắng nghe và ghi nhận nhiều luồng ý kiến của nhiều người khác nhau, trao đổi và tương tác với họ. Hỏi họ và xem họ đáp gì và khuyến khích họ làm điều ngược lại. Dù cho bạn đang ở bất kỳ giai đoạn nào của quá trình làm SaaS (học công nghệ - tìm kiếm vấn đề và giải pháp - phát triển sản phẩm - thử nghiệm sản phẩm). Bạn nên - kể cả người bạn đối thoại có là học sinh / sinh viên, người lao động, nhân viên văn phòng - miễn là họ đã có nhiều trải nghiệm ứng dụng và có khả năng thụ hưởng giá trị từ SaaS mới!
+Cách hiệu quả nhất để giỏi lên - bất kể thứ đó là gì - chính là trao đổi nhiều về nó. Đó là lắng nghe và ghi nhận nhiều luồng ý kiến của nhiều người khác nhau, trao đổi và tương tác với họ. Hỏi họ và xem họ đáp gì và khuyến khích họ làm điều ngược lại với bạn. Dù cho bạn đang ở bất kỳ giai đoạn nào của quá trình làm SaaS (học công nghệ - tìm kiếm vấn đề và giải pháp - phát triển sản phẩm - thử nghiệm sản phẩm). Bạn nên - kể cả người bạn đối thoại có là học sinh / sinh viên, người lao động, nhân viên văn phòng hay bảo vệ trông xe - miễn là họ đã có nhiều trải nghiệm ứng dụng và có khả năng thụ hưởng giá trị từ SaaS mới!
 Không nhất thiết phải là kỹ sư phần mềm hạng ưu thì mới có đặc quyền được nói về SaaS - hoàn toàn không! Bạn xuất hiện với tư cách là người dùng, như thế đã là quá đủ. Bản thân SaaS không phải là thứ bị cô lập bởi đội ngũ phát triển. SaaS trở nên hữu ích và có giá trị là bởi vì được sử dụng để giải quyết vấn đề và được quan tâm bởi nhiều người - từ đó mang lại doanh thu cho đội ngũ phát triển.
 [^1]: [Time Spent Using Smartphones (2026 Statistics) by Fabio Duarte](https://explodingtopics.com/blog/smartphone-usage-stats)
 [^2]: Quý Hải Ng, "Bộ khung Canvas tinh gọn," Hải có gì hay, 2026. https://haicogihay.com/blog/bo-khung-canvas-tinh-gon.html</t>
@@ -1975,7 +1975,7 @@
 &lt;p&gt;Nếu phải nói rằng ngành công nghiệp nào phát triển mạnh mẽ nhất và thay đổi nhiều nhất trong vòng 10 năm trở lại đây, Hải nghĩ đó là ngành công nghiệp phần mềm dịch vụ hay còn được biết đến với tên gọi SaaS (Software-as-a-Service). Cổ phiếu của những công ty phần mềm tăng từ 5-10 lần bất chấp có thời điểm kinh tế suy thoái do tác động của dịch bệnh và chiến tranh. Các công ty start-up công nghệ mới liên tục ra đời và được định giá với những con số không tưởng, điển hình là OpenAI, Anthropic, Anysphere. &lt;/p&gt;
 &lt;h2 id="thay-oi-cua-saas-trong-10-nam"&gt;Thay đổi của SaaS trong 10 năm&lt;/h2&gt;
 &lt;p&gt;Xu hướng chung về số lượng phần mềm dịch vụ ra đời cũng như lượng người dùng phần lớn là tăng trưởng. Nhờ vào việc SaaS được triển khai trên Cloud, các cá nhân hoặc doanh nghiệp làm SaaS có thể nhanh chóng thực hiện chỉnh sửa để thích nghi với sự thay đổi của người dùng. &lt;/p&gt;
-&lt;p&gt;Thống kê từ Exploding Topics &lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt; cuối 2026 chỉ ra trung bình mỗi người dành 4 giờ 37 phút mỗi ngày để dùng điện thoại. Mỗi ngày, mỗi người dùng mở điện thoại khoảng 58 lần: 3 lần để sử dụng trên 10 phút, 40 lần để kiểm tra thông báo nhanh dưới 2 phút. 52% khoảng thời gian check điện thoại mỗi tháng diễn ra trong giờ làm việc. &lt;/p&gt;
+&lt;p&gt;Thống kê từ Exploding Topics cuối 2026 &lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt; chỉ ra trung bình mỗi người dành 4 giờ 37 phút mỗi ngày để dùng điện thoại. Mỗi ngày, mỗi người dùng mở điện thoại khoảng 58 lần: 3 lần để sử dụng trên 10 phút, 40 lần để kiểm tra thông báo nhanh dưới 2 phút. 52% khoảng thời gian check điện thoại mỗi tháng diễn ra trong giờ làm việc. &lt;/p&gt;
 &lt;p&gt;Nhiều thống kê khác nhau tại Việt Nam cũng chỉ ra thời lượng sử dụng điện thoại trung bình của người Việt là từ 6-8 tiếng mỗi ngày, thậm chí có bài báo giật tít tiêu đề từ 9-13 tiếng. Nói như vậy để hiểu nhu cầu thực cho ngành phần mềm và Internet nói chung vẫn là &lt;strong&gt;rất lớn&lt;/strong&gt;.&lt;/p&gt;
 &lt;h3 id="huong-toi-mo-hinh-tra-phi-e-nhan-mot-so-ac-quyen-freemium"&gt;Hướng tới mô hình trả phí để nhận một số đặc quyền (freemium)&lt;/h3&gt;
 &lt;p&gt;Đây là điều dễ thấy nhất hiện nay. SaaS được nhắc tới nhiều nhất về việc này có lẽ là Youtube khi ra mắt tính năng Premium để tắt quảng cáo. Và điều này cũng từng gây ra tranh cãi khi nhiều người cho rằng họ tự tạo ra vấn đề là chèn thêm quảng cáo và bán giải pháp để giải quyết vấn đề do chính họ tạo ra. Nhưng nhìn chung, khi nhắc tới trải nghiệm người dùng, mỗi người sẽ có cảm nhận khác nhau về việc có đáng xuống tiền hay không?&lt;/p&gt;
@@ -1987,7 +1987,7 @@
 &lt;h3 id="rao-can-khi-hai-moi-chap-chung-lam-saas"&gt;Rào cản khi Hải mới chập chững làm SaaS&lt;/h3&gt;
 &lt;p&gt;Hầu hết mọi người đều học code từ những khung đen Console - Hải cũng vậy. Quay lại 8 năm trước, học ngôn ngữ gì, framework gì đã là một rào cản. Bởi vì có quá nhiều lựa chọn khi xét tới việc chúng làm được gì, mất bao lâu để học, chi phí để triển khai một ứng dụng hoàn chỉnh là bao nhiêu? Chúng có hỗ trợ trên hệ điều hành X hay không? Để đóng gói mã nguồn thành file cài đặt thì phải làm sao, mất bao nhiêu tiền? Thương mại hóa chúng thế nào? Có sợ bị ăn cắp mã nguồn không? Code có tối ưu về mặt hiệu năng hay không?&lt;/p&gt;
 &lt;p&gt;Thời điểm đó, việc cân nhắc lựa chọn thuê cloud hay host cho rẻ và có nên cúng tiền cho domain hay không cũng đã là vấn đề lớn với Hải. Có quá nhiều ngôn ngữ, framework cho tới công ty cung cấp giải pháp điện toán và offer nhiều mức giá khác nhau. Không trả lời được câu hỏi này thì mã nguồn chỉ có thể chạy local và đưa lên Github. Còn nếu tự build server? - Tiền điện 24/7 và tiền mua hardware có khi còn mắc hơn!&lt;/p&gt;
-&lt;p&gt;Theo trải nghiệm của Hải, vấn đề tích hợp từ giải pháp từ bên ngoài cũng là trở ngại. Nhẹ nhất là kết nối .NET với máy in qua thư viện để xuất báo cáo, máy scan để đọc barcode. Nặng hơn là làm sao để liên hệ với hàng loạt ngân hàng hoặc khác nhau để gom chung về 1 cổng thanh toán?&lt;/p&gt;
+&lt;p&gt;Theo trải nghiệm của Hải, vấn đề tích hợp giải pháp từ bên ngoài cũng là trở ngại. Nhẹ nhất là kết nối .NET với máy in qua thư viện để xuất báo cáo, máy scan để đọc barcode. Nặng hơn là làm sao để liên hệ với hàng loạt ngân hàng khác nhau để gom chung về 1 cổng thanh toán?&lt;/p&gt;
 &lt;h3 id="thay-oi-tu-cong-nhan-viet-code-sang-ky-su-phan-mem"&gt;Thay đổi từ "công nhân viết code" sang "kỹ sư phần mềm"&lt;/h3&gt;
 &lt;p&gt;Nếu như trước đây, việc dành ra 1 buổi đi cafe nói chuyện với ai đó sẽ lấy đi thời gian làm SaaS của Hải thì bây giờ Hải đã có thể vừa cafe trò chuyện, vừa build SaaS. Thậm chí, Hải có thể nhanh chóng thay đổi hoặc bổ sung thêm tính năng gì đó mới đến từ cuộc trò chuyện với người khác. Quả thật AI đã có thể viết code, review và tự test nhanh và tốt hơn 1 Dev trình độ Junior. Việc của Hải chỉ đơn giản là quản lý tốt context, kiến trúc và cấp quyền cho Agents. &lt;/p&gt;
 &lt;p&gt;&lt;strong&gt;Nói nhiều hơn về nhu cầu và trải nghiệm người dùng thay vì code&lt;/strong&gt;&lt;/p&gt;
@@ -2013,14 +2013,14 @@
 &lt;li&gt;SEO, quảng cáo để tiếp cận người dùng&lt;/li&gt;
 &lt;li&gt;Hỗ trợ người dùng và phí thanh toán nếu áp dụng gói trả phí&lt;/li&gt;
 &lt;/ul&gt;
-&lt;p&gt;Còn về doanh thu, khả năng cao chúng sẽ đến từ quảng cáo, các offer trả phí khác nhau. Vì thế, nếu không có inverstors, rất có thể anh em sẽ đói trong giai đoạn đầu làm SaaS đấy!&lt;/p&gt;
+&lt;p&gt;Còn về doanh thu, khả năng cao chúng sẽ đến từ quảng cáo, các offer trả phí khác nhau. Vì thế, nếu không có investors, rất có thể anh em sẽ đói trong giai đoạn đầu làm SaaS đấy!&lt;/p&gt;
 &lt;p&gt;&lt;strong&gt;Không tham vọng lớn khi nguồn lực nhỏ!&lt;/strong&gt;&lt;/p&gt;
 &lt;p&gt;Một trong những tham vọng dẫn tới thất bại phổ biến nhất của người mới bắt đầu làm SaaS đó là làm mạng xã hội. Đã rất nhiều công ty lớn nhỏ khác nhau thất bại và quay xe ở mảng này. Tại sao phải làm mạng xã hội? Mạng xã hội bạn đưa ra giải quyết vấn đề gì mà các mạng xã hội hiện tại chưa có? Bạn đã tính tới các chi phí để có hệ thống chưa? Bạn đã tính tới chi phí để có được người dùng, chi phí để giữ ngọn lửa kết nối và tương tác của người dùng chưa? Bạn đã tính tới chi phí để có được lượng nội dung đầy đặn, đa dạng và thuật toán phân phối chúng hiệu quả chưa? Bạn đã tính tới chi phí để giải quyết các vấn đề pháp lý do "nội dung sáng tạo" từ người dùng tạo ra chưa?&lt;/p&gt;
 &lt;p&gt;Có thể bạn không tin nhưng hồi còn là sinh viên năm 2, Hải đã từng lóe lên ý tưởng làm mạng xã hội khuyến khích người dùng chia sẻ ý tưởng, phản biện ngay cả khi ý tưởng mới hình thành và còn sơ khai bởi vì AI sẽ được tích hợp để hỗ trợ trả lời bên dưới bài đăng khi bạn hỏi. Ý tưởng khá giống mạng xã hội Thread này xuất hiện vào năm 2021 (trước khi Thread ra đời được 2 năm) khi Hải nhìn thấy tính năng bình luận trên Facebook và Youtube chỉ chấp nhận tối đa 2 lớp phản hồi và không cho phép tự bình luận khi nội dung chưa được tạo. Hải từng đặt tên cho nó là "Vô tri" - nhưng tất nhiên là Hải đã nhanh chóng dừng lại vì chưa trả lời được hết những câu hỏi ở bên trên. &lt;/p&gt;
 &lt;h2 id="tap-trung-cho-y-tuong-va-trai-nghiem-nguoi-dung"&gt;Tập trung cho ý tưởng và trải nghiệm người dùng&lt;/h2&gt;
-&lt;p&gt;SaaS ngày nay đã build dễ hơn 5-10 năm trước rất nhiều rồi. Vì thế, hãy cố gắng khai thác nhu cầu, vấn dề, sự bất tiện, sự khó chịu của người khác. Chúng xuất hiện ở khắp mọi nơi từ ngoài đời đến Internet. Chúng mới là động lực để bạn làm SaaS. Hãy cố gắng đưa ra lời đề nghị người khác dùng SaaS của bạn và ngày càng nhiều hơn. Quan sát xem khi họ dùng SaaS, mắt họ tập trung vào đâu, tay họ thao tác như thế nào, họ tương tác và phản hồi ra làm sao. Những thứ đó sẽ khiến cho SaaS của bạn ngày càng phát triển và trở nên cạnh tranh hơn.&lt;/p&gt;
+&lt;p&gt;SaaS ngày nay đã dễ build hơn 5-10 năm trước rất nhiều rồi. Vì thế, hãy cố gắng khai thác nhu cầu, vấn đề, sự bất tiện, sự khó chịu của người khác. Chúng xuất hiện ở khắp mọi nơi từ ngoài đời đến Internet. Chúng mới là động lực để bạn làm SaaS. Hãy cố gắng đưa ra lời đề nghị người khác dùng thử SaaS của bạn - và ngày càng nhiều hơn. Quan sát xem khi họ dùng SaaS, mắt họ tập trung vào đâu, tay họ thao tác như thế nào, họ tương tác và phản hồi ra làm sao. Những thứ đó sẽ khiến cho SaaS của bạn ngày càng phát triển và trở nên cạnh tranh hơn.&lt;/p&gt;
 &lt;h2 id="muon-gioi-cai-gi-thi-hay-noi-nhieu-ve-no"&gt;Muốn giỏi cái gì thì hãy nói nhiều về nó&lt;/h2&gt;
-&lt;p&gt;Cách hiệu quả nhất để giỏi lên - bất kể thứ đó là gì - chính là trao đổi nhiều về nó. Đó là lắng nghe và ghi nhận nhiều luồng ý kiến của nhiều người khác nhau, trao đổi và tương tác với họ. Hỏi họ và xem họ đáp gì và khuyến khích họ làm điều ngược lại. Dù cho bạn đang ở bất kỳ giai đoạn nào của quá trình làm SaaS (học công nghệ - tìm kiếm vấn đề và giải pháp - phát triển sản phẩm - thử nghiệm sản phẩm). Bạn nên - kể cả người bạn đối thoại có là học sinh / sinh viên, người lao động, nhân viên văn phòng - miễn là họ đã có nhiều trải nghiệm ứng dụng và có khả năng thụ hưởng giá trị từ SaaS mới!&lt;/p&gt;
+&lt;p&gt;Cách hiệu quả nhất để giỏi lên - bất kể thứ đó là gì - chính là trao đổi nhiều về nó. Đó là lắng nghe và ghi nhận nhiều luồng ý kiến của nhiều người khác nhau, trao đổi và tương tác với họ. Hỏi họ và xem họ đáp gì và khuyến khích họ làm điều ngược lại với bạn. Dù cho bạn đang ở bất kỳ giai đoạn nào của quá trình làm SaaS (học công nghệ - tìm kiếm vấn đề và giải pháp - phát triển sản phẩm - thử nghiệm sản phẩm). Bạn nên - kể cả người bạn đối thoại có là học sinh / sinh viên, người lao động, nhân viên văn phòng hay bảo vệ trông xe - miễn là họ đã có nhiều trải nghiệm ứng dụng và có khả năng thụ hưởng giá trị từ SaaS mới!&lt;/p&gt;
 &lt;p&gt;Không nhất thiết phải là kỹ sư phần mềm hạng ưu thì mới có đặc quyền được nói về SaaS - hoàn toàn không! Bạn xuất hiện với tư cách là người dùng, như thế đã là quá đủ. Bản thân SaaS không phải là thứ bị cô lập bởi đội ngũ phát triển. SaaS trở nên hữu ích và có giá trị là bởi vì được sử dụng để giải quyết vấn đề và được quan tâm bởi nhiều người - từ đó mang lại doanh thu cho đội ngũ phát triển.&lt;/p&gt;
 &lt;div class="footnote"&gt;
 &lt;hr /&gt;

</xml_diff>

<commit_message>
Tu ban khong the xuat hien ben ngoai luu thong
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="91" customWidth="1" min="1" max="1"/>
@@ -1221,32 +1221,40 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cách mà content-engine vận hành và thay đổi tư duy dùng content management system (CMS)</t>
+          <t>Context quăng cho AI nên chứa những gì?</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>cach-ma-content-engine-van-hanh-va-thay-doi-tu-duy-dung-content-management-system-cms</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>context-quang-cho-ai-nen-chua-nhung-gi</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>25-05-2026</t>
+          <t>12-10-2026</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>25-05-2026</t>
+          <t>12-10-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>data\blogs\Cách mà content-engine vận hành và thay đổi tư duy dùng content management system (CMS).md</t>
+          <t>data\blogs\Context quăng cho AI nên chứa những gì.md</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -1255,19 +1263,15 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cách PR bản thân hay nhất là nâng tầm đối thủ</t>
+          <t>Cách mà content-engine vận hành và thay đổi tư duy dùng content management system (CMS)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>cach-pr-ban-than-hay-nhat-la-nang-tam-doi-thu</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
+          <t>cach-ma-content-engine-van-hanh-va-thay-doi-tu-duy-dung-content-management-system-cms</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
@@ -1278,20 +1282,58 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>25-05-2026</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>data\blogs\Cách mà content-engine vận hành và thay đổi tư duy dùng content management system (CMS).md</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cách PR bản thân hay nhất là nâng tầm đối thủ</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>cach-pr-ban-than-hay-nhat-la-nang-tam-doi-thu</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>25-05-2026</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>30-05-2026</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Có 1 kiểu tâm lý khá phổ biến để bản thân mình trở nên an toàn và có giá trị. Đó là bình thường hóa, tầm thường hóa cá nhân hoặc nhóm khác và nói rằng mình không giống họ. Anh em có thể bắt gặp tâm lý này ở bất kỳ đâu. `Học sinh trường chuy...</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>data\blogs\Cách PR bản thân hay nhất là nâng tầm đối thủ.md</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t># Cách PR bản thân hay nhất là nâng tầm đối thủ
 Có 1 kiểu tâm lý khá phổ biến để bản thân mình trở nên an toàn và có giá trị. Đó là bình thường hóa, tầm thường hóa cá nhân hoặc nhóm khác và nói rằng mình không giống họ. Anh em có thể bắt gặp tâm lý này ở bất kỳ đâu. `Học sinh trường chuyên toàn là gà công nghiệp, không học đều các môn. Giáo sư tiến sĩ Việt Nam toàn là trên giấy. Đại gia Việt chỉ giỏi phân lô bán nền. Công nghệ của Việt Nam toàn là sao chép, thay nhãn. Con nhà giàu mà có sự nghiệp thì cũng chẳng có gì đặc biệt, nền tảng gia đình để lại sẵn rồi, không giàu được nữa thì coi như vứt.`
@@ -1306,7 +1348,7 @@
 # Kết</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>&lt;h1 id="cach-pr-ban-than-hay-nhat-la-nang-tam-oi-thu"&gt;Cách PR bản thân hay nhất là nâng tầm đối thủ&lt;/h1&gt;
 &lt;p&gt;Có 1 kiểu tâm lý khá phổ biến để bản thân mình trở nên an toàn và có giá trị. Đó là bình thường hóa, tầm thường hóa cá nhân hoặc nhóm khác và nói rằng mình không giống họ. Anh em có thể bắt gặp tâm lý này ở bất kỳ đâu. &lt;code&gt;Học sinh trường chuyên toàn là gà công nghiệp, không học đều các môn. Giáo sư tiến sĩ Việt Nam toàn là trên giấy. Đại gia Việt chỉ giỏi phân lô bán nền. Công nghệ của Việt Nam toàn là sao chép, thay nhãn. Con nhà giàu mà có sự nghiệp thì cũng chẳng có gì đặc biệt, nền tảng gia đình để lại sẵn rồi, không giàu được nữa thì coi như vứt.&lt;/code&gt;&lt;/p&gt;
@@ -1322,54 +1364,54 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Giá trị thặng dư</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>gia-tri-thang-du</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Kinh tế</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>09-09-2026</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Chắc hẳn anh em đã được nghe đâu đó đại loại rằng một nền kinh tế thực sự phát triển là một nền kinh tế tạo ra thật nhiều giá trị và phân phối chúng đi khắp nơi. Anh em nghe điều đó bất kể là anh em đang học ở đâu - Đông hay Tây, xưa hay na...</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>data\blogs\Giá trị thặng dư.md</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t># Giá trị thặng dư
 Chắc hẳn anh em đã được nghe đâu đó đại loại rằng một nền kinh tế thực sự phát triển là một nền kinh tế tạo ra thật nhiều giá trị và phân phối chúng đi khắp nơi. Anh em nghe điều đó bất kể là anh em đang học ở đâu - Đông hay Tây, xưa hay nay. Mức sống của một quốc gia phụ thuộc vào năng lực sản xuất hàng hóa và dịch vụ của quốc gia đó.[^1] Sản xuất vật chất là cơ sở của sự tồn tại và phát triển xã hội.[^2] Và rồi sau mỗi giai đoạn, mỗi thời kỳ, mỗi một sự đổi mới được hình thành, anh em bắt đầu nhìn lại và coi lại cách chúng áp dụng trong thời đại hiện tại. Và đây cũng là chủ đề mà Hải được nghe nhiều nhất từ thời đi học. 
@@ -1396,7 +1438,7 @@
 [^3]: Kinh tế chính trị Mác - Lênin</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>&lt;h1 id="gia-tri-thang-du"&gt;Giá trị thặng dư&lt;/h1&gt;
 &lt;p&gt;Chắc hẳn anh em đã được nghe đâu đó đại loại rằng một nền kinh tế thực sự phát triển là một nền kinh tế tạo ra thật nhiều giá trị và phân phối chúng đi khắp nơi. Anh em nghe điều đó bất kể là anh em đang học ở đâu - Đông hay Tây, xưa hay nay. Mức sống của một quốc gia phụ thuộc vào năng lực sản xuất hàng hóa và dịch vụ của quốc gia đó.&lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt; Sản xuất vật chất là cơ sở của sự tồn tại và phát triển xã hội.&lt;sup id="fnref:2"&gt;&lt;a class="footnote-ref" href="#fn:2"&gt;2&lt;/a&gt;&lt;/sup&gt; Và rồi sau mỗi giai đoạn, mỗi thời kỳ, mỗi một sự đổi mới được hình thành, anh em bắt đầu nhìn lại và coi lại cách chúng áp dụng trong thời đại hiện tại. Và đây cũng là chủ đề mà Hải được nghe nhiều nhất từ thời đi học. &lt;/p&gt;
@@ -1443,50 +1485,50 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Giáp kèo môi giới</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>giap-keo-moi-gioi</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
         <is>
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>15-07-2026</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Khi nhắc tới 2 chữ môi giới, một vài người sẽ có suy nghĩ không mấy tích cực về công việc này. Đặc biệt là môi giới bất động sản khi mà có hẳn 1 thuật ngữ dành riêng cho nghề này - cò đất. Nhưng trên thực tế, nghề môi giới cũng như những ng...</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>data\blogs\Giáp kèo môi giới.md</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t># Giáp kèo môi giới
 Khi nhắc tới 2 chữ môi giới, một vài người sẽ có suy nghĩ không mấy tích cực về công việc này. Đặc biệt là môi giới bất động sản khi mà có hẳn 1 thuật ngữ dành riêng cho nghề này - cò đất. Nhưng trên thực tế, nghề môi giới cũng như những ngành nghề khác, tạo ra giá trị và tồn tại tới tận ngày nay là vì giải quyết vấn đề cho người khác và có thể tạo ra thu nhập. Từ nông sản, bảo hiểm, tài chính - chứng khoán, gia sư, nhà đất cho tới việc làm hay thậm chí là mai mối. Những ngành nghề đó phát triển mạnh tới tận ngày nay là vì xã hội thực sự cần chúng. 
@@ -1509,7 +1551,7 @@
 Cuối cùng, khi 2 bên đang lệch xa suy nghĩ về sản phẩm dịch vụ và về tiền, đừng cố đưa họ đi đến giao dịch vì ngoài kia cũng còn rất nhiều người khác có khả năng cung cấp giải pháp. Tiếp tục tìm kiếm cho tới khi tìm được thì dừng. Tiếp tục tìm giáo viên cho học viên tới khi tìm được người phù hợp về năng lực và về giá. Tiếp tục tìm công việc cho người thất nghiệp cho tới khi tìm được chỗ phù hợp về JD và lương. Tiếp tục tìm quỹ đầu tư cho start-up cho tới khi họ tìm được nhà đầu tư và kêu gọi đủ vốn. Tiếp tục tìm khách để giải ngân cho tới khi đạt chỉ tiêu. Tiếp tục tìm nhà cho tới khi tìm được căn phù hợp trong khả năng tài chính của khách thì thôi.</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>&lt;h1 id="giap-keo-moi-gioi"&gt;Giáp kèo môi giới&lt;/h1&gt;
 &lt;p&gt;Khi nhắc tới 2 chữ môi giới, một vài người sẽ có suy nghĩ không mấy tích cực về công việc này. Đặc biệt là môi giới bất động sản khi mà có hẳn 1 thuật ngữ dành riêng cho nghề này - cò đất. Nhưng trên thực tế, nghề môi giới cũng như những ngành nghề khác, tạo ra giá trị và tồn tại tới tận ngày nay là vì giải quyết vấn đề cho người khác và có thể tạo ra thu nhập. Từ nông sản, bảo hiểm, tài chính - chứng khoán, gia sư, nhà đất cho tới việc làm hay thậm chí là mai mối. Những ngành nghề đó phát triển mạnh tới tận ngày nay là vì xã hội thực sự cần chúng. &lt;/p&gt;
@@ -1533,114 +1575,114 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Góc nhìn về Sandbox</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>goc-nhin-ve-sandbox</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Công nghệ</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>sandbox, thử nghiệm</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>09-07-2026</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>09-07-2026</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Sandbox - nếu giải thích theo nghĩa đen trần trụi thì nó giống như một chiếc hộp bên trong có cát.</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>data\blogs\Góc nhìn về sandbox.md</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t># Góc nhìn về Sandbox
 Sandbox - nếu giải thích theo nghĩa đen trần trụi thì nó giống như một chiếc hộp bên trong có cát.</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>&lt;h1 id="goc-nhin-ve-sandbox"&gt;Góc nhìn về Sandbox&lt;/h1&gt;
 &lt;p&gt;Sandbox - nếu giải thích theo nghĩa đen trần trụi thì nó giống như một chiếc hộp bên trong có cát.&lt;/p&gt;</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Góc nhìn về thành công và thất bại từ cao thủ TFT 3 mùa</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>goc-nhin-ve-thanh-cong-va-that-bai-tu-cao-thu-tft-3-mua</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>05-08-2026</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Winners &amp; Losers là chủ đề muôn thuở, không bao giờ có thể khai thác hết và luôn nhận được sự chú ý từ nhiều người. Vì thời nào ai cũng so sánh, ai cũng hiếu kỳ và ai cũng thích sự thành công. Làm sao để thành công, làm gì để đừng thất bại?...</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>data\blogs\Góc nhìn về thành công và thất bại của cao thủ TFT ba mùa.md</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t># Góc nhìn về thành công và thất bại từ cao thủ TFT 3 mùa
 Winners &amp; Losers là chủ đề muôn thuở, không bao giờ có thể khai thác hết và luôn nhận được sự chú ý từ nhiều người. Vì thời nào ai cũng so sánh, ai cũng hiếu kỳ và ai cũng thích sự thành công. Làm sao để thành công, làm gì để đừng thất bại? Thật khó để tìm công thức chung. Vì nếu có, ai ai cũng đã thành công và chẳng còn ai thất bại. 3 mùa đạt mức rank cao thủ TFT, Hải nhìn thấy điều này rất rõ.
@@ -1677,7 +1719,7 @@
 Nhờ cơ chế reset mỗi mùa, Hải không còn áp lực mình là cao thủ, không còn bám víu lấy sự thành công của mùa trước mà thay vào đó là niềm vui bắt đầu lại từ đầu. Niềm vui cạnh tranh với những người chơi mới. Niềm vui được thỏa sức thử lại, được sáng tạo và được vấp ngã. Nếu có DNA của cao thủ TFT, Hải sẽ quay trở lại mức rank cao thủ vào mùa mới như cách Hải đã làm ở những mùa cũ. Còn không, mức rank của Hải khi kết thúc mùa mới sẽ là mức rank chính thức của Hải. Những người giỏi hơn và nỗ lực hơn Hải ở mùa mới, họ hoàn toàn xứng đáng có mức rank cao hơn Hải.</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>&lt;h1 id="goc-nhin-ve-thanh-cong-va-that-bai-tu-cao-thu-tft-3-mua"&gt;Góc nhìn về thành công và thất bại từ cao thủ TFT 3 mùa&lt;/h1&gt;
 &lt;p&gt;Winners &amp;amp; Losers là chủ đề muôn thuở, không bao giờ có thể khai thác hết và luôn nhận được sự chú ý từ nhiều người. Vì thời nào ai cũng so sánh, ai cũng hiếu kỳ và ai cũng thích sự thành công. Làm sao để thành công, làm gì để đừng thất bại? Thật khó để tìm công thức chung. Vì nếu có, ai ai cũng đã thành công và chẳng còn ai thất bại. 3 mùa đạt mức rank cao thủ TFT, Hải nhìn thấy điều này rất rõ.&lt;/p&gt;
@@ -1717,50 +1759,50 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Gửi Hải tuổi 35</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>gui-hai-tuoi-35</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
         <is>
           <t>06-09-2026</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>15-09-2026</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>MrBeast có "Hi Me In 10 Years", IShowSpeed có "Hi Me In 3 Years", Miêu Công Tử có "999 lá thư gửi bản thân". Và Hải nghĩ rằng không có một lý do gì để một người nào đó không có điều gì muốn gửi tới chính mình nhiều năm sau. Và Hải cũng khôn...</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>data\blogs\Gửi Hải tuổi 35.md</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t># Gửi Hải tuổi 35
 MrBeast có "Hi Me In 10 Years", IShowSpeed có "Hi Me In 3 Years", Miêu Công Tử có "999 lá thư gửi bản thân". Và Hải nghĩ rằng không có một lý do gì để một người nào đó không có điều gì muốn gửi tới chính mình nhiều năm sau. Và Hải cũng không ngoại lệ.
@@ -1791,7 +1833,7 @@
 Hải tuổi 24./</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>&lt;h1 id="gui-hai-tuoi-35"&gt;Gửi Hải tuổi 35&lt;/h1&gt;
 &lt;p&gt;MrBeast có "Hi Me In 10 Years", IShowSpeed có "Hi Me In 3 Years", Miêu Công Tử có "999 lá thư gửi bản thân". Và Hải nghĩ rằng không có một lý do gì để một người nào đó không có điều gì muốn gửi tới chính mình nhiều năm sau. Và Hải cũng không ngoại lệ.&lt;/p&gt;
@@ -1825,77 +1867,23 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Học cách kể chuyện</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>hoc-cach-ke-chuyen</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>in-draft</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Quý Hải Ng</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>04-09-2026</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>04-09-2026</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>data\blogs\Học cách kể chuyện.md</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t># Học cách kể chuyện</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>&lt;h1 id="hoc-cach-ke-chuyen"&gt;Học cách kể chuyện&lt;/h1&gt;</t>
-        </is>
-      </c>
-    </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Kinh nghiệm build SaaS</t>
+          <t>Học cách kể chuyện</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>kinh-nghiem-build-saas</t>
+          <t>hoc-cach-ke-chuyen</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Công nghệ</t>
-        </is>
-      </c>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
@@ -1904,25 +1892,113 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
+          <t>04-09-2026</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>04-09-2026</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>data\blogs\Học cách kể chuyện.md</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t># Học cách kể chuyện</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>&lt;h1 id="hoc-cach-ke-chuyen"&gt;Học cách kể chuyện&lt;/h1&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm Build SaaS phần 2 - nhận định chi phí</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-build-saas-phan-2---nhan-dinh-chi-phi</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>04-10-2026</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>04-10-2026</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>data\blogs\Kinh nghiệm Build SaaS phần 2 - nhận định chi phí.md</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm build SaaS</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-build-saas</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Công nghệ</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
           <t>17-09-2026</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>01-10-2026</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>Nếu phải nói rằng ngành công nghiệp nào phát triển mạnh mẽ nhất và thay đổi nhiều nhất trong vòng 10 năm trở lại đây, Hải nghĩ đó là ngành công nghiệp phần mềm dịch vụ hay còn được biết đến với tên gọi SaaS (Software-as-a-Service). Cổ phiếu...</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>data\blogs\Kinh nghiệm build SaaS.md</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t># Kinh nghiệm build SaaS
 Nếu phải nói rằng ngành công nghiệp nào phát triển mạnh mẽ nhất và thay đổi nhiều nhất trong vòng 10 năm trở lại đây, Hải nghĩ đó là ngành công nghiệp phần mềm dịch vụ hay còn được biết đến với tên gọi SaaS (Software-as-a-Service). Cổ phiếu của những công ty phần mềm tăng từ 5-10 lần bất chấp có thời điểm kinh tế suy thoái do tác động của dịch bệnh và chiến tranh. Các công ty start-up công nghệ mới liên tục ra đời và được định giá với những con số không tưởng, điển hình là OpenAI, Anthropic, Anysphere. 
@@ -1969,7 +2045,7 @@
 [^2]: Quý Hải Ng, "Bộ khung Canvas tinh gọn," Hải có gì hay, 2026. https://haicogihay.com/blog/bo-khung-canvas-tinh-gon.html</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>&lt;h1 id="kinh-nghiem-build-saas"&gt;Kinh nghiệm build SaaS&lt;/h1&gt;
 &lt;p&gt;Nếu phải nói rằng ngành công nghiệp nào phát triển mạnh mẽ nhất và thay đổi nhiều nhất trong vòng 10 năm trở lại đây, Hải nghĩ đó là ngành công nghiệp phần mềm dịch vụ hay còn được biết đến với tên gọi SaaS (Software-as-a-Service). Cổ phiếu của những công ty phần mềm tăng từ 5-10 lần bất chấp có thời điểm kinh tế suy thoái do tác động của dịch bệnh và chiến tranh. Các công ty start-up công nghệ mới liên tục ra đời và được định giá với những con số không tưởng, điển hình là OpenAI, Anthropic, Anysphere. &lt;/p&gt;
@@ -2036,50 +2112,50 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>ky-nang-cot-loi-de-thanh-cong---danh-cho-tat-ca-moi-nguoi</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
         <is>
           <t>23-07-2026</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>Khi đọc sách self-help hay tham gia bất kỳ hội thảo khóa học nào, anh em có thể đã nghe que hàng trăm đức tính để trở nên thành công, thành đạt, thịnh vượng. Nào là cần cù, chịu thương, chịu khó. Nào là thông minh, sáng tạo, tư duy mở. Nào...</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>data\blogs\Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người.md</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t># Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người
 Khi đọc sách self-help hay tham gia bất kỳ hội thảo khóa học nào, anh em có thể đã nghe que hàng trăm đức tính để trở nên thành công, thành đạt, thịnh vượng. Nào là cần cù, chịu thương, chịu khó. Nào là thông minh, sáng tạo, tư duy mở. Nào là hình thành thói quen tốt, kỹ năng tự học, tính kỷ luật. Và hàng loạt yếu tố khác như tinh thần cầu tiến, sự tập trung, quản lý thời gian, dám chấp nhận rủi ro,...
@@ -2109,7 +2185,7 @@
 Là một người viết, thành công đối với Hải là thuyết phục được người khác đọc hết bài viết của mình. Vì thế Hải sẵn sàng đón nhận mọi ý kiến, bất kể là khen hay chê. Khi ai đó khen Hải, Hải sẽ kiểu: "Ok, cảm ơn bạn nhé, tầm ngày này tuần sau Hải sẽ lại ra bài mới, nhớ đón đọc nha!". Còn khi ai đó chê bai, Hải sẽ biết rằng : "Được rồi, có điều gì đó cần thay đổi!".</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>&lt;h1 id="ky-nang-cot-loi-e-thanh-cong-danh-cho-tat-ca-moi-nguoi"&gt;Kỹ năng cốt lõi để thành công - dành cho tất cả mọi người&lt;/h1&gt;
 &lt;p&gt;Khi đọc sách self-help hay tham gia bất kỳ hội thảo khóa học nào, anh em có thể đã nghe que hàng trăm đức tính để trở nên thành công, thành đạt, thịnh vượng. Nào là cần cù, chịu thương, chịu khó. Nào là thông minh, sáng tạo, tư duy mở. Nào là hình thành thói quen tốt, kỹ năng tự học, tính kỷ luật. Và hàng loạt yếu tố khác như tinh thần cầu tiến, sự tập trung, quản lý thời gian, dám chấp nhận rủi ro,...&lt;/p&gt;
@@ -2144,54 +2220,54 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Tạm biệt Wordpress - Vì sao mình chuyển sang content engine thay vì hệ thống back-end CMS</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>tam-biet-wordpress---vi-sao-minh-chuyen-sang-content-engine-thay-vi-he-thong-back-end-cms</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Công nghệ</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
         <is>
           <t>web, tech, wp</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>24-05-2026</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Từng nghiên cứu Wordpress 5 năm và thực chiến 2 năm, cũng xuất bản được kha khá blog. Bản thân Hải thấy Wordpress đem lại rất nhiều trải nghiệm thú vị nơi blogger chỉ cần quan tâm tới tuyến nội dung và quản trị thay vì đầu tư nhiều thời gia...</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>data\blogs\Lựa chọn content engine thay vì hệ thống back-end.md</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t># Tạm biệt Wordpress - Vì sao mình chuyển sang content engine thay vì hệ thống back-end CMS
 Từng nghiên cứu Wordpress 5 năm và thực chiến 2 năm, cũng xuất bản được kha khá blog. Bản thân Hải thấy Wordpress đem lại rất nhiều trải nghiệm thú vị nơi blogger chỉ cần quan tâm tới tuyến nội dung và quản trị thay vì đầu tư nhiều thời gian cho code, web, database, ...  Wordpress mang lại rất nhiều giá trị cho Hải. Với những anh em đã từng đau đầu hoặc đã trả giá vì hệ thống quản lý phân quyền, quản lý media, danh mục, bình luận,... thì sẽ hiểu rõ Wordpress có thể giúp anh em tiết kiệm cả tỷ đồng. Và trên hết nó là mã nguồn mở, miễn phí.
@@ -2244,7 +2320,7 @@
 Với 1 blogger, thay vì phải duy trì một CMS phức tạp với hàng loạt plugin, tài khoản quản trị, cơ sở dữ liệu và các bản vá bảo mật định kỳ, việc thuần tập trung vào sản xuất nội dung mới là ưu tiền hàng đầu. Toàn bộ quá trình còn lại được tự động hóa thông qua content engine để chuyển đổi cắt văn bản và nhúng vào các tập tin định dạng.</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-biet-wordpress-vi-sao-minh-chuyen-sang-content-engine-thay-vi-he-thong-back-end-cms"&gt;Tạm biệt Wordpress - Vì sao mình chuyển sang content engine thay vì hệ thống back-end CMS&lt;/h1&gt;
 &lt;p&gt;Từng nghiên cứu Wordpress 5 năm và thực chiến 2 năm, cũng xuất bản được kha khá blog. Bản thân Hải thấy Wordpress đem lại rất nhiều trải nghiệm thú vị nơi blogger chỉ cần quan tâm tới tuyến nội dung và quản trị thay vì đầu tư nhiều thời gian cho code, web, database, ...  Wordpress mang lại rất nhiều giá trị cho Hải. Với những anh em đã từng đau đầu hoặc đã trả giá vì hệ thống quản lý phân quyền, quản lý media, danh mục, bình luận,... thì sẽ hiểu rõ Wordpress có thể giúp anh em tiết kiệm cả tỷ đồng. Và trên hết nó là mã nguồn mở, miễn phí.&lt;/p&gt;
@@ -2298,42 +2374,42 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Markdown_Example</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>markdownexample</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>21-07-2026</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>Example paragraph</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>data\blogs\Markdown_Example.md</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t># This is heading 1 for title
 Example paragraph
@@ -2382,7 +2458,7 @@
 [^1]: This is the footnote.</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>&lt;h1 id="this-is-heading-1-for-title"&gt;This is heading 1 for title&lt;/h1&gt;
 &lt;p&gt;Example paragraph&lt;/p&gt;
@@ -2441,50 +2517,50 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Một cách kiếm tiền không mới nhưng luôn mới mẻ</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>mot-cach-kiem-tien-khong-moi-nhung-luon-moi-me</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>22-07-2026</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>Năm 1889, vào thời điểm chưa có Google Map và thị trường xe hơi ở Pháp chưa có tới 3000 chiếc, 2 anh em Andre và Edouard đã nhận thấy tiềm năng từ việc giúp cho tài xế có được hành trình thú vị nhằm thúc đẩy doanh thu từ việc bán xe và lốp....</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>data\blogs\Một cách kiếm tiền không mới nhưng luôn mới mẻ.md</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t># Một cách kiếm tiền không mới nhưng luôn mới mẻ
 Năm 1889, vào thời điểm chưa có Google Map và thị trường xe hơi ở Pháp chưa có tới 3000 chiếc, 2 anh em Andre và Edouard đã nhận thấy tiềm năng từ việc giúp cho tài xế có được hành trình thú vị nhằm thúc đẩy doanh thu từ việc bán xe và lốp. Vì thế họ tạo ra cẩm nang hướng dẫn cho khách du lịch. Từ việc đổ xăng ở đâu, thay lốp ở đâu, ăn uống ở đâu, nghỉ ngơi ở đâu. Trong hơn 2 thập kỷ đầu, cuốn cẩm nang có chứa danh sách khách sạn, nhà hàng ở Paris được chia theo danh mục cụ thể hoàn toàn miễn phí. Tới năm 1920, cuốn cẩm nang đó được bán với giá 7 franc. Nếu quy đổi theo lạm phát, cuốn cẩm nang đó có giá khoảng 32.000 VND vào năm 2026. Và đó là khởi đầu của giải thưởng Sao Michelin ngày nay. [^1]
@@ -2528,7 +2604,7 @@
 [^3]: [Content Engine - Vì sao các cá nhân và doanh nghiệp nên quan tâm?](https://haicogihay.com/blog/content-engine---vi-sao-cac-ca-nhan-va-doanh-nghiep-nen-quan-tam)</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>&lt;h1 id="mot-cach-kiem-tien-khong-moi-nhung-luon-moi-me"&gt;Một cách kiếm tiền không mới nhưng luôn mới mẻ&lt;/h1&gt;
 &lt;p&gt;Năm 1889, vào thời điểm chưa có Google Map và thị trường xe hơi ở Pháp chưa có tới 3000 chiếc, 2 anh em Andre và Edouard đã nhận thấy tiềm năng từ việc giúp cho tài xế có được hành trình thú vị nhằm thúc đẩy doanh thu từ việc bán xe và lốp. Vì thế họ tạo ra cẩm nang hướng dẫn cho khách du lịch. Từ việc đổ xăng ở đâu, thay lốp ở đâu, ăn uống ở đâu, nghỉ ngơi ở đâu. Trong hơn 2 thập kỷ đầu, cuốn cẩm nang có chứa danh sách khách sạn, nhà hàng ở Paris được chia theo danh mục cụ thể hoàn toàn miễn phí. Tới năm 1920, cuốn cẩm nang đó được bán với giá 7 franc. Nếu quy đổi theo lạm phát, cuốn cẩm nang đó có giá khoảng 32.000 VND vào năm 2026. Và đó là khởi đầu của giải thưởng Sao Michelin ngày nay. &lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt;&lt;/p&gt;
@@ -2586,54 +2662,54 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Một số nơi chứa ý tưởng mới</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>mot-so-noi-chua-y-tuong-moi</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Tư duy</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Quy Hai Ng</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>26-08-2026</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>Hải đoán là mỗi một ngày khi anh em lướt feed và đọc tin tức, sẽ có khoảng vài chục đến vài trăm lần anh em bắt gặp các cụm từ `đổi mới`, `sáng tạo`, `start-up`. Nói đúng ra, nếu không có ý tưởng mới, chúng ta sẽ mãi rơi vào vòng lặp bảo th...</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>data\blogs\Một số nơi chứa ý tưởng mới.md</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t># Một số nơi chứa ý tưởng mới
 Hải đoán là mỗi một ngày khi anh em lướt feed và đọc tin tức, sẽ có khoảng vài chục đến vài trăm lần anh em bắt gặp các cụm từ `đổi mới`, `sáng tạo`, `start-up`. Nói đúng ra, nếu không có ý tưởng mới, chúng ta sẽ mãi rơi vào vòng lặp bảo thủ trong khi mọi thứ xung quanh đều đang thay đổi. Điều này không chỉ đúng với các cá nhân hay SME, mà còn đúng với cả các tập đoàn lớn.
@@ -2661,7 +2737,7 @@
 [^1]: [Một cách kiếm tiền không mới nhưng luôn mới mẻ](https://haicogihay.com/blog/mot-cach-kiem-tien-khong-moi-nhung-luon-moi-me)</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>&lt;h1 id="mot-so-noi-chua-y-tuong-moi"&gt;Một số nơi chứa ý tưởng mới&lt;/h1&gt;
 &lt;p&gt;Hải đoán là mỗi một ngày khi anh em lướt feed và đọc tin tức, sẽ có khoảng vài chục đến vài trăm lần anh em bắt gặp các cụm từ &lt;code&gt;đổi mới&lt;/code&gt;, &lt;code&gt;sáng tạo&lt;/code&gt;, &lt;code&gt;start-up&lt;/code&gt;. Nói đúng ra, nếu không có ý tưởng mới, chúng ta sẽ mãi rơi vào vòng lặp bảo thủ trong khi mọi thứ xung quanh đều đang thay đổi. Điều này không chỉ đúng với các cá nhân hay SME, mà còn đúng với cả các tập đoàn lớn.&lt;/p&gt;
@@ -2702,58 +2778,58 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Một vài góc nhìn nhìn từ thí ngiệm "Vũ trụ 25"</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>mot-vai-goc-nhin-nhin-tu-thi-ngiem-vu-tru-25</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>universe25, tâm lý, thiên đường của loài chuột</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>12-08-2026</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>Vào ngày 22 tháng 6 năm 1972, nhà khoa học John Calhoun đã thực hiệm 1 thí nghiệm để trả lời cho câu hỏi: "Nếu loài sinh vật được sống trong thiên đường không lo cạnh tranh về thức ăn, về chỗ ở, liệu chúng có thể duy trì và phát triển mãi m...</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>data\blogs\Một vài góc nhìn từ thí nghiệm vũ trụ 25.md</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t># Một vài góc nhìn từ thí nghiệm "Vũ trụ 25"
 Vào ngày 22 tháng 6 năm 1972, nhà khoa học John Calhoun đã thực hiệm 1 thí nghiệm để trả lời cho câu hỏi: "Nếu loài sinh vật được sống trong thiên đường không lo cạnh tranh về thức ăn, về chỗ ở, liệu chúng có thể duy trì và phát triển mãi mãi hay không?  [^1] Ông chọn ra 4 cặp chuột khỏe mạnh đã được sàng lọc kỹ càng về sức khỏe. Sau đó, đưa chúng vào môi trường 3m x 4.3m, chia thành 16 tháp, tạo được thành 256 hộp tổ, mỗi hộp có sức chứa đủ cho 15 chuột cùng ở - thiên đường đủ để chứa 4000 con chuột. Thức ăn, nước đều được cung cấp đầy đủ, nhiệt độ môi trường được kiểm soát, chất thải của chúng cũng được dọn dẹp, và hoàn toàn không có thú săn mồi. 
@@ -2794,7 +2870,7 @@
 [^4]: [Sáng Thế Ký 3 - Người Nam và Người Nữ Phạm Tội](https://www.bible.com/vi/bible/1638/GEN.3.KTHD)</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>&lt;h1 id="mot-vai-goc-nhin-tu-thi-nghiem-vu-tru-25"&gt;Một vài góc nhìn từ thí nghiệm "Vũ trụ 25"&lt;/h1&gt;
 &lt;p&gt;Vào ngày 22 tháng 6 năm 1972, nhà khoa học John Calhoun đã thực hiệm 1 thí nghiệm để trả lời cho câu hỏi: "Nếu loài sinh vật được sống trong thiên đường không lo cạnh tranh về thức ăn, về chỗ ở, liệu chúng có thể duy trì và phát triển mãi mãi hay không?  &lt;sup id="fnref:1"&gt;&lt;a class="footnote-ref" href="#fn:1"&gt;1&lt;/a&gt;&lt;/sup&gt; Ông chọn ra 4 cặp chuột khỏe mạnh đã được sàng lọc kỹ càng về sức khỏe. Sau đó, đưa chúng vào môi trường 3m x 4.3m, chia thành 16 tháp, tạo được thành 256 hộp tổ, mỗi hộp có sức chứa đủ cho 15 chuột cùng ở - thiên đường đủ để chứa 4000 con chuột. Thức ăn, nước đều được cung cấp đầy đủ, nhiệt độ môi trường được kiểm soát, chất thải của chúng cũng được dọn dẹp, và hoàn toàn không có thú săn mồi. &lt;/p&gt;
@@ -2853,50 +2929,50 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Nói về bán hàng</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>noi-ve-ban-hang</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
         <is>
           <t>26-07-2026</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>27-07-2026</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>Dạy con làm giàu hay cha giàu cha nghèo là bộ sách cực kỳ nổi tiếng làm nên tên tuổi và thưởng hiệu của tác giả Robert Kiyosaki. Dù có nhiều tranh cãi, nhưng đây vẫn là bộ sách có doanh số bán rất khủng khiếp: Hơn 32 triệu bản, dịch sang 51...</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>data\blogs\Nói về bán hàng.md</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t># Nói về bán hàng
 Dạy con làm giàu hay cha giàu cha nghèo là bộ sách cực kỳ nổi tiếng làm nên tên tuổi và thưởng hiệu của tác giả Robert Kiyosaki. Dù có nhiều tranh cãi, nhưng đây vẫn là bộ sách có doanh số bán rất khủng khiếp: Hơn 32 triệu bản, dịch sang 51 thứ tiếng và xuất hiện ở 109 quốc gia. Robert Kiyosaki có lần chia sẻ về câu chuyện hỏi người cha nuôi của mình tên Tommy cách để giàu như cha ông: 
@@ -2918,7 +2994,7 @@
 - [ ] Kỹ năng</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>&lt;h1 id="noi-ve-ban-hang"&gt;Nói về bán hàng&lt;/h1&gt;
 &lt;p&gt;Dạy con làm giàu hay cha giàu cha nghèo là bộ sách cực kỳ nổi tiếng làm nên tên tuổi và thưởng hiệu của tác giả Robert Kiyosaki. Dù có nhiều tranh cãi, nhưng đây vẫn là bộ sách có doanh số bán rất khủng khiếp: Hơn 32 triệu bản, dịch sang 51 thứ tiếng và xuất hiện ở 109 quốc gia. Robert Kiyosaki có lần chia sẻ về câu chuyện hỏi người cha nuôi của mình tên Tommy cách để giàu như cha ông: &lt;/p&gt;
@@ -2947,54 +3023,108 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Nói về cú Duo</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>noi-ve-cu-duo</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Công nghệ</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>04-10-2026</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>04-10-2026</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>data\blogs\Nói về cú Duo và DET.md</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t># Nói về cú Duo và DET</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>&lt;h1 id="noi-ve-cu-duo-va-det"&gt;Nói về cú Duo và DET&lt;/h1&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Sách self-help có thật sự hữu ích?</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>sach-self-help-co-that-su-huu-ich</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
         <is>
           <t>10-06-2026</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>12-06-2026</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>Sách Self-help có thể hiểu nôm na là cuốn sách tự phát triển bản thân. Chúng đồng hành với các độc giả thông qua việc đề cập đến các phương pháp, giải pháp để đi đến thành công, hạnh phúc hay chân - thiện - mĩ. Những cuốn sách đó thường có...</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>data\blogs\Sách self-help có thật sự hữu ích.md</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t># Sách self-help có thật sự hữu ích?
 Sách Self-help có thể hiểu nôm na là cuốn sách tự phát triển bản thân. Chúng đồng hành với các độc giả thông qua việc đề cập đến các phương pháp, giải pháp để đi đến thành công, hạnh phúc hay chân - thiện - mĩ. Những cuốn sách đó thường có đặc điểm chung là bán chạy bởi dễ đọc - dễ hiểu nếu so với những cuốn giáo trình khô khan. Tiêu biểu những cuốn điển hình mà anh em có lẽ đã quá quen thuộc là Đắc nhân tâm, Những kẻ xuất chúng, Nghĩ giàu làm giàu, 7 thói quen để thành đạt, Atomic Habit… 
@@ -3021,7 +3151,7 @@
 Một lần nữa, Hải muốn nhấn mạnh rằng: “Tri thức không chỉ phát triển nhờ sự đồng thuận tuyệt đối, mà nhờ những cuộc đối thoại tử tế. Vì vậy, mong anh em đọc bài viết như một góc nhìn để suy ngẫm, thay vì một kết luận cuối cùng. Mọi quan điểm ít nhiều đều mang dấu vết của trải nghiệm cá nhân. Mục đích của mỗi bài viết không phải là để ai đúng tuyệt đối, mà là liệu chúng ta có thể cùng nhau suy nghĩ sâu hơn sau mỗi bài viết hay không? Vì vậy, hãy đọc với tinh thần cởi mở và phản biện hoặc góp ý khi anh em có suy nghĩ khác nha!”.</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>&lt;h1 id="sach-self-help-co-that-su-huu-ich"&gt;Sách self-help có thật sự hữu ích?&lt;/h1&gt;
 &lt;p&gt;Sách Self-help có thể hiểu nôm na là cuốn sách tự phát triển bản thân. Chúng đồng hành với các độc giả thông qua việc đề cập đến các phương pháp, giải pháp để đi đến thành công, hạnh phúc hay chân - thiện - mĩ. Những cuốn sách đó thường có đặc điểm chung là bán chạy bởi dễ đọc - dễ hiểu nếu so với những cuốn giáo trình khô khan. Tiêu biểu những cuốn điển hình mà anh em có lẽ đã quá quen thuộc là Đắc nhân tâm, Những kẻ xuất chúng, Nghĩ giàu làm giàu, 7 thói quen để thành đạt, Atomic Habit… &lt;/p&gt;
@@ -3049,92 +3179,92 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Thử thay đổi cách đặt câu hỏi</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>thu-thay-doi-cach-dat-cau-hoi</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
         <is>
           <t>09-07-2026</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
         <is>
           <t>data\blogs\Thử thay đổi cách đặt câu hỏi.md</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Thử thay đổi góc nhìn</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>thu-thay-doi-goc-nhin</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
         <is>
           <t>09-07-2026</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>Một anh tài xế ở một nước phương Tây nào đó làm việc 11 tiếng mỗi ngày. Anh ta thường xuyên sử dụng đồ hộp, mì gói và nước tăng lực - thứ mà người Việt hay gọi là combo chạy thận. Anh ta có một mức thu nhập đủ để lo cho bản thân và để dành....</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>data\blogs\Thử thay đổi góc nhìn.md</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t># Thử thay đổi góc nhìn
 Một anh tài xế ở một nước phương Tây nào đó làm việc 11 tiếng mỗi ngày. Anh ta thường xuyên sử dụng đồ hộp, mì gói và nước tăng lực - thứ mà người Việt hay gọi là combo chạy thận. Anh ta có một mức thu nhập đủ để lo cho bản thân và để dành. Anh ta luôn tự hào mình làm việc chăm chỉ. Cho tới một ngày, một sự cố ập đến, anh ta bị bệnh nặng và phải nhập viện. Sau gần 3 tháng điều trị, anh ta cũng đã khỏi bệnh. Vì không có bảo hiểm, tổng chi phí cho hóa đơn dài hơn 100 trang gồm tiền giường, tiền thuốc, tiền mổ và loạt chi phí khác đã chạm ngưỡng 1 triệu đô. Và tất nhiên, số tiền anh ta dành giụm rất nhỏ khi so với chi phí điều trị. Người từng tự đắc rằng mình không bao giờ nợ ai bất kỳ điều gì trên đời này cuối cùng lại nhận món nợ 1 triệu đô theo một cách mà không ai ngờ tới - viện phí.
@@ -3142,7 +3272,7 @@
 ## Thật ra tất cả mọi thứ còn tồn tại là vì còn nợ</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>&lt;h1 id="thu-thay-oi-goc-nhin"&gt;Thử thay đổi góc nhìn&lt;/h1&gt;
 &lt;p&gt;Một anh tài xế ở một nước phương Tây nào đó làm việc 11 tiếng mỗi ngày. Anh ta thường xuyên sử dụng đồ hộp, mì gói và nước tăng lực - thứ mà người Việt hay gọi là combo chạy thận. Anh ta có một mức thu nhập đủ để lo cho bản thân và để dành. Anh ta luôn tự hào mình làm việc chăm chỉ. Cho tới một ngày, một sự cố ập đến, anh ta bị bệnh nặng và phải nhập viện. Sau gần 3 tháng điều trị, anh ta cũng đã khỏi bệnh. Vì không có bảo hiểm, tổng chi phí cho hóa đơn dài hơn 100 trang gồm tiền giường, tiền thuốc, tiền mổ và loạt chi phí khác đã chạm ngưỡng 1 triệu đô. Và tất nhiên, số tiền anh ta dành giụm rất nhỏ khi so với chi phí điều trị. Người từng tự đắc rằng mình không bao giờ nợ ai bất kỳ điều gì trên đời này cuối cùng lại nhận món nợ 1 triệu đô theo một cách mà không ai ngờ tới - viện phí.&lt;/p&gt;
@@ -3151,50 +3281,50 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Tài sản lớn nhất của một người</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>tai-san-lon-nhat-cua-mot-nguoi</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>Tôi thích tiền, bạn thích tiền. Tất cả mọi người đều thích tiền. Những ai nói rằng tôi không thích tiền đều là nói dối. Nói dối những người xung quanh và lừa dối chính bản thân mình. Để kiếm tiền, con người có thể phải đánh đổi rất nhiều th...</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>data\blogs\Tài sản lớn nhất của một người.md</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t># Tài sản lớn nhất của một người
 Tôi thích tiền, bạn thích tiền. Tất cả mọi người đều thích tiền. Những ai nói rằng tôi không thích tiền đều là nói dối. Nói dối những người xung quanh và lừa dối chính bản thân mình. Để kiếm tiền, con người có thể phải đánh đổi rất nhiều thứ. Có người chấp nhận làm ăn xa xứ. Có người bỏ thời gian 8 - 16 tiếng mỗi ngày để làm việc. Có người nâng cao giá trị bản thân để kiếm nhiều tiền hơn. 
@@ -3250,7 +3380,7 @@
 Tuy nhiên, cũng nên lưu ý rằng câu **"Tài sản lớn nhất của một người là sự uy tín"** là một nhận định mang tính giá trị, không phải chân lý tuyệt đối. Với người khác, họ có thể cho rằng sức khỏe, thời gian hay tri thức mới là tài sản lớn nhất. Điều hợp lý hơn là xem **uy tín là một trong những tài sản vô hình giá trị nhất**, đặc biệt trong kinh doanh, lãnh đạo và các mối quan hệ lâu dài.</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>&lt;h1 id="tai-san-lon-nhat-cua-mot-nguoi"&gt;Tài sản lớn nhất của một người&lt;/h1&gt;
 &lt;p&gt;Tôi thích tiền, bạn thích tiền. Tất cả mọi người đều thích tiền. Những ai nói rằng tôi không thích tiền đều là nói dối. Nói dối những người xung quanh và lừa dối chính bản thân mình. Để kiếm tiền, con người có thể phải đánh đổi rất nhiều thứ. Có người chấp nhận làm ăn xa xứ. Có người bỏ thời gian 8 - 16 tiếng mỗi ngày để làm việc. Có người nâng cao giá trị bản thân để kiếm nhiều tiền hơn. &lt;/p&gt;
@@ -3356,54 +3486,54 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Tâm lý học blogger - Tại sao Hải viết blog?</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>tam-ly-hoc-blogger---tai-sao-hai-viet-blog</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr">
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
         <is>
           <t>web, blog</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>01-06-2026</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>Hôm nay, Hải vào xem lại trận Argentina gặp Pháp vào mùa World Cup năm 2018. Đó là năm Mbappe 19 tuổi và đã khiến Messi dừng bước với 1 kiến tạo Penalty và ghi 2 bàn thắng. Tất cả những phút chạy của Mbappe đều được tường thuật trực tiếp và...</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học blogger -Tại sao Hải viết blog.md</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t># Tâm lý học blogger - Tại sao Hải lập blog riêng?
 Hôm nay, Hải vào xem lại trận Argentina gặp Pháp vào mùa World Cup năm 2018. Đó là năm Mbappe 19 tuổi và đã khiến Messi dừng bước với 1 kiến tạo Penalty và ghi 2 bàn thắng. Tất cả những phút chạy của Mbappe đều được tường thuật trực tiếp và ghi lại để bất kỳ ai có thể xem lại sau này. Tất cả người xem bóng đá đều biết Mbappe, biết khả năng chơi bóng của anh ta, biết tốc độ của anh ta. Hàng loạt câu lạc bộ lớn muốn ký hợp đồng với anh ta với mức giá không tưởng.
@@ -3439,7 +3569,7 @@
 ---</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-blogger-tai-sao-hai-lap-blog-rieng"&gt;Tâm lý học blogger - Tại sao Hải lập blog riêng?&lt;/h1&gt;
 &lt;p&gt;Hôm nay, Hải vào xem lại trận Argentina gặp Pháp vào mùa World Cup năm 2018. Đó là năm Mbappe 19 tuổi và đã khiến Messi dừng bước với 1 kiến tạo Penalty và ghi 2 bàn thắng. Tất cả những phút chạy của Mbappe đều được tường thuật trực tiếp và ghi lại để bất kỳ ai có thể xem lại sau này. Tất cả người xem bóng đá đều biết Mbappe, biết khả năng chơi bóng của anh ta, biết tốc độ của anh ta. Hàng loạt câu lạc bộ lớn muốn ký hợp đồng với anh ta với mức giá không tưởng.&lt;/p&gt;
@@ -3476,84 +3606,84 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Tâm lý học cá độ - Vì sao người không chơi là người thắng</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>tam-ly-hoc-ca-do---vi-sao-nguoi-khong-choi-la-nguoi-thang</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>02-07-2026</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr">
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học cá độ - Vì sao người không chơi là người thắng.md</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Tâm lý học của người lười nhưng tham vọng lớn</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>tam-ly-hoc-cua-nguoi-luoi-nhung-tham-vong-lon</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
         <is>
           <t>26-05-2026</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>Theo lẽ thường, người lười thường sẽ chọn sống yên ổn thay vì tham vọng còn người đã tham vọng thì không được phép lười biếng. Nhưng có 1 kiểu tâm lý nghe qua có vẻ lạ vì nó khá đặc biệt và giống như đang trêu đùa logic nhưng nó vẫn đang xu...</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học của người lười nhưng tham vọng đạt được thành tựu lớn.md</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t># Tâm lý học của người lười nhưng tham vọng lớn
 Theo lẽ thường, người lười thường sẽ chọn sống yên ổn thay vì tham vọng còn người đã tham vọng thì không được phép lười biếng. Nhưng có 1 kiểu tâm lý nghe qua có vẻ lạ vì nó khá đặc biệt và giống như đang trêu đùa logic nhưng nó vẫn đang xuất hiện trong hàng triệu triệu người mỗi ngày. Đó chính là tâm lý của người lười nhưng tham vọng lớn. 
@@ -3582,7 +3712,7 @@
 Giáo sư Jiang Xue Qin</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-cua-nguoi-luoi-nhung-tham-vong-lon"&gt;Tâm lý học của người lười nhưng tham vọng lớn&lt;/h1&gt;
 &lt;p&gt;Theo lẽ thường, người lười thường sẽ chọn sống yên ổn thay vì tham vọng còn người đã tham vọng thì không được phép lười biếng. Nhưng có 1 kiểu tâm lý nghe qua có vẻ lạ vì nó khá đặc biệt và giống như đang trêu đùa logic nhưng nó vẫn đang xuất hiện trong hàng triệu triệu người mỗi ngày. Đó chính là tâm lý của người lười nhưng tham vọng lớn. &lt;/p&gt;
@@ -3612,54 +3742,54 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Tâm lý học FOMO</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>tam-ly-hoc-fomo</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr">
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
         <is>
           <t>fomo</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>28-05-2026</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>Từ thời nguyên thủy, con người đã luôn sợ bỏ lỡ. Nếu bộ lạc săn được thức ăn mà 1 cá thể trong bầy không biết, cá thể đó có thể bị đói. Nếu 1 thành viên nào trong bầy người nguyên thủy bỏ lỡ việc di dời theo bầy vì thời tiết cực đoan, thành...</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học FOMO.md</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t># Tâm lý học FOMO
 Từ thời nguyên thủy, con người đã luôn sợ bỏ lỡ. Nếu bộ lạc săn được thức ăn mà 1 cá thể trong bầy không biết, cá thể đó có thể bị đói. Nếu 1 thành viên nào trong bầy người nguyên thủy bỏ lỡ việc di dời theo bầy vì thời tiết cực đoan, thành viên đó sẽ gặp nguy hiểm. Ngày nay, chúng ta thấy tâm lý FOMO (fear-of-missing-out) ở khắp mọi nơi: cái áo chỉ giảm giá trong ngày, drama trên mạng xã hội, sóng đầu tư tiền ảo, tin tức thời sự,... Khai thác FOMO là ngành công nghiệp kiếm rất nhiều tiền bởi con người không chỉ sợ thất bại, họ còn sợ mình đang đứng yên trong khi người khác vẫn chạy.
@@ -3682,7 +3812,7 @@
 FOMO không phải dấu hiệu của sự nhu nhược, hay sự thiếu quyết đoán. Nó là phản ứng rất bình thường của não bộ con người từ xưa tới nay. Từ thời kỳ săn bắt hái lượm tới thời kỳ drama và trào lưu trên mạng xã hội. Xóa bỏ hoàn toàn tâm lý FOMO là vô ích và tự hủy cơ chế bảo vệ bản thân mà tạo hóa ban tặng.</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-fomo"&gt;Tâm lý học FOMO&lt;/h1&gt;
 &lt;p&gt;Từ thời nguyên thủy, con người đã luôn sợ bỏ lỡ. Nếu bộ lạc săn được thức ăn mà 1 cá thể trong bầy không biết, cá thể đó có thể bị đói. Nếu 1 thành viên nào trong bầy người nguyên thủy bỏ lỡ việc di dời theo bầy vì thời tiết cực đoan, thành viên đó sẽ gặp nguy hiểm. Ngày nay, chúng ta thấy tâm lý FOMO (fear-of-missing-out) ở khắp mọi nơi: cái áo chỉ giảm giá trong ngày, drama trên mạng xã hội, sóng đầu tư tiền ảo, tin tức thời sự,... Khai thác FOMO là ngành công nghiệp kiếm rất nhiều tiền bởi con người không chỉ sợ thất bại, họ còn sợ mình đang đứng yên trong khi người khác vẫn chạy.&lt;/p&gt;
@@ -3706,49 +3836,91 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Tâm lý học không gì là bí mật</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>tam-ly-hoc-khong-gi-la-bi-mat</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>12-10-2026</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>12-10-2026</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>data\blogs\Tâm lý học không gì là bí mật.md</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Tâm lý học kinh nghiệm</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>tam-ly-hoc-kinh-nghiem</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr">
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>Anh đọc bài viết em cũng ổn.</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học kinh nghiệm.md</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>Anh đọc bài viết em cũng ổn.
 Ví dụ tâm lý học nhà thầu, em phân tích mục đích và hành động của nhiều nhóm người chơi nhưng không đưa ra được hệ phương trình vi phân để mô hình hóa sự thay đổi động lực của các người chơi trong dự án. Em cũng không đưa ra được mô hình xác suất có điều kiện trong trường hợp nào nhà thầu sẽ ưu tiên tìm đối tác giá rẻ và trong trường hợp nào họ ưu tiên sự yên tâm. 
 Hay 1 ví dụ khác</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>&lt;p&gt;Anh đọc bài viết em cũng ổn.&lt;/p&gt;
 &lt;p&gt;Ví dụ tâm lý học nhà thầu, em phân tích mục đích và hành động của nhiều nhóm người chơi nhưng không đưa ra được hệ phương trình vi phân để mô hình hóa sự thay đổi động lực của các người chơi trong dự án. Em cũng không đưa ra được mô hình xác suất có điều kiện trong trường hợp nào nhà thầu sẽ ưu tiên tìm đối tác giá rẻ và trong trường hợp nào họ ưu tiên sự yên tâm. &lt;/p&gt;
@@ -3756,50 +3928,50 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Tâm lý học Michelin Boy</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>tam-ly-hoc-michelin-boy</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>indraft</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr">
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr">
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
         <is>
           <t>07-06-2026</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>23-06-2026</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>Vì sao chúng ta không bao giờ nghe đến từ Michelin Girl.</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học Michelin Boy.md</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t># Tâm lý học Michelin Boy
 Vì sao chúng ta không bao giờ nghe đến từ Michelin Girl.
@@ -3822,7 +3994,7 @@
 [^1]: This is the footnote.</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-michelin-boy"&gt;Tâm lý học Michelin Boy&lt;/h1&gt;
 &lt;p&gt;Vì sao chúng ta không bao giờ nghe đến từ Michelin Girl.&lt;/p&gt;
@@ -3851,100 +4023,100 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Tâm lý học một view</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>tam-ly-hoc-mot-view</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr">
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học một view.md</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t># Tâm lý học một view</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-mot-view"&gt;Tâm lý học một view&lt;/h1&gt;</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Tâm lý học nghiện xem video phát triển bản thân</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>tam-ly-hoc-nghien-xem-video-phat-trien-ban-than</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr">
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
         <is>
           <t>29-05-2026</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>30-05-2026</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>Con người luôn muốn hoàn thiện mình và hướng tới chân thiện mỹ. Đó là lý do chúng ta luôn tìm cách để bản thân mình tốt lên hằng ngày. Tập thể dục, học tập, rèn luyện, học kỹ năng mới hay mở rộng vòng tròn các mối quan hệ xã hội - tất cả nh...</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học nghiện xem video phát triển bản thân.md</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t># Tâm lý học nghiện xem video phát triển bản thân
 Con người luôn muốn hoàn thiện mình và hướng tới chân thiện mỹ. Đó là lý do chúng ta luôn tìm cách để bản thân mình tốt lên hằng ngày. Tập thể dục, học tập, rèn luyện, học kỹ năng mới hay mở rộng vòng tròn các mối quan hệ xã hội - tất cả nhằm 1 mục đích là nâng cấp bản thân. Cũng từ đó, có một thứ nghiện khá mới trong thời đại mạng xã hội ngày nay, không phải nghiện game, không phải nghiện phim mà là nghiện xem video phát triển bản thân. 
@@ -3955,7 +4127,7 @@
 ##</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-nghien-xem-video-phat-trien-ban-than"&gt;Tâm lý học nghiện xem video phát triển bản thân&lt;/h1&gt;
 &lt;p&gt;Con người luôn muốn hoàn thiện mình và hướng tới chân thiện mỹ. Đó là lý do chúng ta luôn tìm cách để bản thân mình tốt lên hằng ngày. Tập thể dục, học tập, rèn luyện, học kỹ năng mới hay mở rộng vòng tròn các mối quan hệ xã hội - tất cả nhằm 1 mục đích là nâng cấp bản thân. Cũng từ đó, có một thứ nghiện khá mới trong thời đại mạng xã hội ngày nay, không phải nghiện game, không phải nghiện phim mà là nghiện xem video phát triển bản thân. &lt;/p&gt;
@@ -3967,58 +4139,58 @@
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Tâm lý học ngành bột mì</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>tam-ly-hoc-nganh-bot-mi</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>bột mì</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>28-05-2026</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>Chỉ trong 1 thời gian ngắn trước lúc Hải viết bài này, đã có rất nhiều người nhận kết quả test dương tính với bột mì. Trong số đó có cả những người nổi tiếng, có sức ảnh hưởng. Đa phần chúng ta đều thắc mắc tại sao những người đã giàu, đã c...</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học ngành bột mì.md</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t># Tâm lý học ngành bột mì
 Chỉ trong 1 thời gian ngắn trước lúc Hải viết bài này, đã có rất nhiều người nhận kết quả test dương tính với bột mì. Trong số đó có cả những người nổi tiếng, có sức ảnh hưởng. Đa phần chúng ta đều thắc mắc tại sao những người đã giàu, đã có gần như tất cả mọi thứ lại dính vào thứ tệ nạn này? Và tại sao trong rất nhiều thập kỷ, ngành công nghiệp này vẫn tồn tại bất kể luật pháp trừng phạt rất mạnh tay?
@@ -4055,7 +4227,7 @@
 Đứng trước lợi nhuận khổng lồ, nhiều cá nhân chấp nhận rủi ro đối mặt án tử để đi sản xuất, tàng trữ và vận chuyển bột mì. Và tất nhiên, phía bên kia của lợi nhuận đó chính là những cuộc đời bị phá hủy, những gia đình tan vỡ, những người trẻ đánh mất tương lai. Bản thân ngành công nghiệp bột mì còn tồn tại không phải chỉ nằm ở việc nó là chất kích thích, nó khai thác vào cảm giác cô đơn, áp lực, muốn hòa nhập, muốn thoát khỏi thực tại của mỗi người. Nó không chỉ là câu chuyện của pháp luật, nó còn là câu chuyện của giáo dục, môi trường sống và các mối quan hệ.</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-nganh-bot-mi"&gt;Tâm lý học ngành bột mì&lt;/h1&gt;
 &lt;p&gt;Chỉ trong 1 thời gian ngắn trước lúc Hải viết bài này, đã có rất nhiều người nhận kết quả test dương tính với bột mì. Trong số đó có cả những người nổi tiếng, có sức ảnh hưởng. Đa phần chúng ta đều thắc mắc tại sao những người đã giàu, đã có gần như tất cả mọi thứ lại dính vào thứ tệ nạn này? Và tại sao trong rất nhiều thập kỷ, ngành công nghiệp này vẫn tồn tại bất kể luật pháp trừng phạt rất mạnh tay?&lt;/p&gt;
@@ -4118,58 +4290,58 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Tâm lý học nhà thầu</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>tam-ly-hoc-nha-thau</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>Tâm lý</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>thầu, dự án</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>26-05-2026</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>Trước khi bắt đầu bài viết, Hải muốn lưu ý rằng đấu thầu và quản lý dự án là lĩnh vực cực kỳ rộng. Mỗi người tham gia dự án đều đứng ở một vị trí khác nhau nên sẽ nhìn thấy những vấn đề khác nhau. Một chủ đầu tư sẽ có góc nhìn khác nhà thầu...</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>data\blogs\Tâm lý học nhà thầu.md</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t># Tâm lý học nhà thầu
 Trước khi bắt đầu bài viết, Hải muốn lưu ý rằng đấu thầu và quản lý dự án là lĩnh vực cực kỳ rộng. Mỗi người tham gia dự án đều đứng ở một vị trí khác nhau nên sẽ nhìn thấy những vấn đề khác nhau. Một chủ đầu tư sẽ có góc nhìn khác nhà thầu. Một kỹ sư hiện trường sẽ có góc nhìn khác đơn vị thiết kế. Một công nhân sẽ có góc nhìn khác người quản lý dự án. Vì vậy, bài viết chỉ là một góc nhìn của Hải dưới lăng kính tâm lý học và lý thuyết trò chơi.
@@ -4214,7 +4386,7 @@
 Bài viết này chủ yếu được nhìn dưới lăng kính tâm lý học, kinh tế học và lý thuyết trò chơi. Hải hiểu rằng thực tế ngoài công trường luôn phức tạp hơn rất nhiều so với những gì có thể trình bày trong một bài blog. Nên nếu anh em đang làm trong lĩnh vực xây dựng, đấu thầu, quản lý dự án, giám sát, thiết kế hoặc từng tham gia các dự án lớn, Hải rất mong nhận được những góp ý, phản biện hoặc góc nhìn khác của anh em qua email **nguyenquyhai2002@gmail.com**.</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>&lt;h1 id="tam-ly-hoc-nha-thau"&gt;Tâm lý học nhà thầu&lt;/h1&gt;
 &lt;p&gt;Trước khi bắt đầu bài viết, Hải muốn lưu ý rằng đấu thầu và quản lý dự án là lĩnh vực cực kỳ rộng. Mỗi người tham gia dự án đều đứng ở một vị trí khác nhau nên sẽ nhìn thấy những vấn đề khác nhau. Một chủ đầu tư sẽ có góc nhìn khác nhà thầu. Một kỹ sư hiện trường sẽ có góc nhìn khác đơn vị thiết kế. Một công nhân sẽ có góc nhìn khác người quản lý dự án. Vì vậy, bài viết chỉ là một góc nhìn của Hải dưới lăng kính tâm lý học và lý thuyết trò chơi.&lt;/p&gt;
@@ -4297,197 +4469,15 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Tâm lý học phông bạt</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>tam-ly-hoc-phong-bat</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>26-05-2026</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>26-05-2026</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>data\blogs\Tâm lý học phông bạt.md</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Tâm lý học sưu tầm tài liệu nhưng không đọc</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>tam-ly-hoc-suu-tam-tai-lieu-nhung-khong-doc</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>29-05-2026</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>29-05-2026</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>data\blogs\Tâm lý học sưu tầm tài liệu nhưng không đọc.md</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Tâm lý học sợ hãi khi bắt đầu</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>tam-ly-hoc-so-hai-khi-bat-dau</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>in-draft</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Tâm lý</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Quý Hải Ng</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>15-09-2026</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>16-09-2026</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>- [ ] Bị đánh giá, săm soi. - [ ] Liên quan tới tiền bạc.</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>data\blogs\Tâm lý học sợ hãi khi bắt đầu.md</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>- [ ] Bị đánh giá, săm soi.
-- [ ] Liên quan tới tiền bạc.</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>&lt;ul class="task-list"&gt;
-&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Bị đánh giá, săm soi.&lt;/li&gt;
-&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Liên quan tới tiền bạc.&lt;/li&gt;
-&lt;/ul&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Tâm lý học trái tim em nhỏ lắm nên chỉ chứa được một người</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>tam-ly-hoc-trai-tim-em-nho-lam-nen-chi-chua-duoc-mot-nguoi</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>26-05-2026</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>08-06-2026</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học l...</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>data\blogs\Tâm lý học trái tim em nhỏ lắm nên chỉ chứa được một người.md</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học lớn? Tất nhiên là không phải chỉ là tải 1 hay 2 cuốn mà là tải rất rất nhiều, rồi lưu chúng vào thư mục trên máy tính hoặc điện thoại. Sau đó, chúng được mở ra từ 1-2 lần và không có sau đó nữa. Kể từ đó, đống tài liệu trên chỉ còn là file được lưu trữ trên máy tính mà không bao giờ được mở. Nếu anh em đã từng rơi vào tình huống như vậy thì đây là bài viết dành cho anh em.
-## Cảm xúc mới lạ
-## Tại sao chúng ta không bao giờ đọc
-##</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học lớn? Tất nhiên là không phải chỉ là tải 1 hay 2 cuốn mà là tải rất rất nhiều, rồi lưu chúng vào thư mục trên máy tính hoặc điện thoại. Sau đó, chúng được mở ra từ 1-2 lần và không có sau đó nữa. Kể từ đó, đống tài liệu trên chỉ còn là file được lưu trữ trên máy tính mà không bao giờ được mở. Nếu anh em đã từng rơi vào tình huống như vậy thì đây là bài viết dành cho anh em.&lt;/p&gt;
-&lt;h2 id="cam-xuc-moi-la"&gt;Cảm xúc mới lạ&lt;/h2&gt;
-&lt;h2 id="tai-sao-chung-ta-khong-bao-gio-oc"&gt;Tại sao chúng ta không bao giờ đọc&lt;/h2&gt;
-&lt;h2 id="_1"&gt;&lt;/h2&gt;</t>
-        </is>
-      </c>
-    </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Tâm lý học xổ số - vì sao người trúng số thường về nợ sau vài năm</t>
+          <t>Tâm lý học phông bạt</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>tam-ly-hoc-xo-so---vi-sao-nguoi-trung-so-thuong-ve-no-sau-vai-nam</t>
+          <t>tam-ly-hoc-phong-bat</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -4507,7 +4497,7 @@
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
-          <t>data\blogs\Tâm lý học xổ số - vì sao người trúng số thường về nợ sau vài năm.md</t>
+          <t>data\blogs\Tâm lý học phông bạt.md</t>
         </is>
       </c>
       <c r="K42" t="inlineStr"/>
@@ -4516,51 +4506,233 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tìm hiểu về MCP</t>
+          <t>Tâm lý học sưu tầm tài liệu nhưng không đọc</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>tim-hieu-ve-mcp</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>in-draft</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Công nghệ</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Quý Hải Ng</t>
-        </is>
-      </c>
+          <t>tam-ly-hoc-suu-tam-tai-lieu-nhung-khong-doc</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
+          <t>29-05-2026</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>29-05-2026</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>data\blogs\Tâm lý học sưu tầm tài liệu nhưng không đọc.md</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Tâm lý học sợ hãi khi bắt đầu</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>tam-ly-hoc-so-hai-khi-bat-dau</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Tâm lý</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>15-09-2026</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>16-09-2026</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>- [ ] Bị đánh giá, săm soi. - [ ] Liên quan tới tiền bạc.</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>data\blogs\Tâm lý học sợ hãi khi bắt đầu.md</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>- [ ] Bị đánh giá, săm soi.
+- [ ] Liên quan tới tiền bạc.</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>&lt;ul class="task-list"&gt;
+&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Bị đánh giá, săm soi.&lt;/li&gt;
+&lt;li class="task-list-item"&gt;&lt;input type="checkbox"/&gt; Liên quan tới tiền bạc.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Tâm lý học trái tim em nhỏ lắm nên chỉ chứa được một người</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>tam-ly-hoc-trai-tim-em-nho-lam-nen-chi-chua-duoc-mot-nguoi</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>26-05-2026</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>08-06-2026</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học l...</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>data\blogs\Tâm lý học trái tim em nhỏ lắm nên chỉ chứa được một người.md</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học lớn? Tất nhiên là không phải chỉ là tải 1 hay 2 cuốn mà là tải rất rất nhiều, rồi lưu chúng vào thư mục trên máy tính hoặc điện thoại. Sau đó, chúng được mở ra từ 1-2 lần và không có sau đó nữa. Kể từ đó, đống tài liệu trên chỉ còn là file được lưu trữ trên máy tính mà không bao giờ được mở. Nếu anh em đã từng rơi vào tình huống như vậy thì đây là bài viết dành cho anh em.
+## Cảm xúc mới lạ
+## Tại sao chúng ta không bao giờ đọc
+##</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Anh em có bao giờ tải xuống những tài liệu pdf, những cuốn sách, những giáo trình về ngoại ngữ như IELTS, HSK hay những tài liệu kinh tế, kỹ thuật từ các nhà xuất bản như O'reilly hay Springer cho tới những slides của những trường Đại học lớn? Tất nhiên là không phải chỉ là tải 1 hay 2 cuốn mà là tải rất rất nhiều, rồi lưu chúng vào thư mục trên máy tính hoặc điện thoại. Sau đó, chúng được mở ra từ 1-2 lần và không có sau đó nữa. Kể từ đó, đống tài liệu trên chỉ còn là file được lưu trữ trên máy tính mà không bao giờ được mở. Nếu anh em đã từng rơi vào tình huống như vậy thì đây là bài viết dành cho anh em.&lt;/p&gt;
+&lt;h2 id="cam-xuc-moi-la"&gt;Cảm xúc mới lạ&lt;/h2&gt;
+&lt;h2 id="tai-sao-chung-ta-khong-bao-gio-oc"&gt;Tại sao chúng ta không bao giờ đọc&lt;/h2&gt;
+&lt;h2 id="_1"&gt;&lt;/h2&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Tâm lý học xổ số - vì sao người trúng số thường về nợ sau vài năm</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>tam-ly-hoc-xo-so---vi-sao-nguoi-trung-so-thuong-ve-no-sau-vai-nam</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>26-05-2026</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>26-05-2026</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>data\blogs\Tâm lý học xổ số - vì sao người trúng số thường về nợ sau vài năm.md</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Tìm hiểu về MCP</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>tim-hieu-ve-mcp</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>in-draft</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Công nghệ</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
           <t>06-07-2026</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>15-07-2026</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>Hãy bắt đầu với 1 công cụ mà chúng ta đều biết - ChatGPT. Khi 1 người muốn nhờ ChatGPT làm 1 điều gì đó, họ sẽ gửi prompt và sau đó ChatGPT sẽ phản hồi lại người đó. Và xuyên suốt quá trình này chỉ nhận văn bản và trả về văn bản. Không có 1...</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>data\blogs\Tìm hiểu về MCP.md</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t># Tìm hiểu về MCP
 ## Tại sao chúng ta cần MCP
@@ -4571,7 +4743,7 @@
 *MCP như cổng kết nối USB. Nguồn: modelcontextprotocol.io*</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>&lt;h1 id="tim-hieu-ve-mcp"&gt;Tìm hiểu về MCP&lt;/h1&gt;
 &lt;h2 id="tai-sao-chung-ta-can-mcp"&gt;Tại sao chúng ta cần MCP&lt;/h2&gt;
@@ -4583,50 +4755,134 @@
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Tư bản không thể xuất hiện bên ngoài lưu thông</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>tu-ban-khong-the-xuat-hien-ben-ngoai-luu-thong</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Quý Hải Ng</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>12-10-2026</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>12-10-2026</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Tư bản không thể xuất hiện ở bên ngoài lưu thông. Vì vậy, muốn kiếm tiền, một người bắt buộc phải kết nối với thế này! Kết nối giúp cho một người có cơ hội tiếp cận với công việc ngay khi ai đó có dự định tìm nhân sự. Kết nối giúp làm giảm...</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>data\blogs\Tư bản không thể xuất hiện bên ngoài lưu thông.md</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t># Tư bản không thể xuất hiện bên ngoài lưu thông
+Tư bản không thể xuất hiện ở bên ngoài lưu thông. Vì vậy, muốn kiếm tiền, một người bắt buộc phải kết nối với thế này! Kết nối giúp cho một người có cơ hội tiếp cận với công việc ngay khi ai đó có dự định tìm nhân sự. Kết nối giúp làm giảm sự bất cân xứng thông tin. Kết nối giúp cho một người nhanh chóng tìm kiếm người phù hợp để giải quyết vấn đề hoặc mở rộng quy mô. Vì vậy, thành công của một người lúc còn trẻ đến từ khả năng chịu đựng sự từ chối. Và thành công của một người lúc về già nằm ở chất lượng danh bạ.  
+## Thành công của một người lúc còn trẻ đến từ khả năng chịu đựng sự từ chối
+Điều tệ hại nhất mà một người thành công sớm hay gặp phải đó là sự tự mãn. Nói thẳng ra là khi đạt được một thành tựu gì đó hoặc có được một vị trí nào đó - người đó cho rằng mình có đặc quyền "miễn trừ từ chối" và vì thế, được hưởng quyền "miễn trừ thất bại". Chúng ta có thể nhìn thấy điều đó ở bất cứ đâu. Trong chuyện tình cảm, trong các bản hợp đồng chuyển nhượng, sau một mùa giải thể thao chuyên nghiệp kết thúc và các bên tìm kiếm bến đỗ mới, sau khi đạt được một giải thưởng từ một cuộc thi hay tổ chức nào đó,... 
+Công bằng mà nói thì chẳng ai trong chúng ta thích thất bại và sự từ chối. Nếu có ai đó nói tôi thích thì chắc chắn là nói dối - nói dối một cách trắng trợn. Nhưng hãy thực sự nhìn lại và sâu chuỗi lại tất cả mọi thứ từ sâu thẳm trong tim: Bạn học được từ cái gì nhiều nhất? Ai là người thay đổi bạn nhiều nhất? Ai là người củng cố niềm tin của bạn mạnh mẽ nhất? Có phải là từ sự thất bại? Có phải là vì từ người từ chối bạn và mang lại cho bạn điều khổ đau và tuyệt vọng nhất?
+Thất bại phơi bày bức tranh toàn cảnh một cách sắc nét nhất, thất bại làm cho một người nhìn thấy hầu hết khía cạnh và sắc màu của cuộc sống - thứ mà thành công ít khi nào có thể hiển thị ra. Những năm trung học, khi các bài báo địa phương viết về Hải và bạn bè cũng như phụ huynh đọc được, Hải đã được trải nghiệm cảm giác được nhiều người quan tâm và dành nhiều lời khen trông như nào. Và đó cũng là lúc khả năng đưa ra lời đề nghị và chấp nhận lời từ chối đã bắt đầu xuống mức rất thấp. Vào năm cuối đại học, Hải nói thầy muốn tự ứng cử vào vị trí lớp phó phong trào và được cả lớp đồng ý với tỉ lệ 100% - và tất nhiên cũng là vì vị trí này chẳng có ai đứng ra cạnh tranh với Hải. 
+Nhưng đây cũng là điểm yếu lớn nhất của Hải. Chúng bộc lộ ngay khi Hải bắt đầu làm công việc bán hàng qua điện thoại - hay còn được biết với tên gọi telesale. Chắc mọi người cũng biết nếu như bán những mặt hàng có giá trị cao như ô tô, bất động sản hay bảo hiểm thì tỉ lệ từ chối sẽ là khoảng 99%. Và vì thế, đây là lĩnh vực mà Hải có thể nói là thất bại đúng nghĩa. Thất bại vì để cho cảm xúc khi bị từ chối chi phối. Thất bại khi để cho một cuộc gọi bị cúp máy ngang kéo theo cảm xúc tiêu cực cả ngày. Thất bại khi cho rằng công việc mình đang làm là không nên và không dám nhận là mình làm công việc này. Nhưng Hải không hiểu rằng bản chất của telesale là để đánh giá mức độ quan tâm của khách đối với sản phẩm cũng như khả năng tài chính của khách. Dựa vào gì? Dựa vào tone giọng, thời gian phản hồi, câu trả lời của khách và những câu follow-up phía sau được chuẩn bị cho khách. Từ đó mới xác định đúng những người phù hợp để kết nối cũng như làm cho khách nghĩ đến sale và muốn liên hệ ngay khi muốn mua sản phẩm - thứ mà không một trường học nào dạy. 
+Chúng ta đều đã, đang và sẽ từ chối rất nhiều người. Bao nhiêu người mỗi ngày chúng ta gặp mà chúng ta không chào hỏi, không bắt chuyện? Mỗi ngày chúng ta gặp đâu đó khoảng 1000 người: trên đường đến cơ quan, tại nơi làm việc, tại cửa hàng, tại công viên, tại các câu lạc bộ,... Bao nhiêu người trong số đó bạn nghĩ rằng nên chủ động làm phiền họ một chút? 500, 200, 100, 10, 1 hay không ai cả? Thực ra nếu bạn không chấp nhận rủi ro gây khó chịu một chút với người khác và có thể nhận lại sự từ chối thì sẽ không có điều gì mới tuyệt vời xảy đến với bạn. Nếu bạn dám làm phiền 100 người trong số 1000 người bạn lướt qua mỗi ngày bất kể đó là về cái gì từ nói chuyện phiếm, hỏi han, xin số điện thoại cho tới giới thiệu bản thân và công việc,... - bạn sẽ nhanh chóng trở thành bậc thầy bắt chuyện. Nếu bạn nhìn ngược lại, bạn đã từ chối bắt chuyện với 900 người (khoảng 90% người bạn gặp). Và vì thế, bạn không trông mong cả 100 người bạn làm phiền sẽ níu lại chia sẻ với thật lâu với bạn. Không, chỉ 10 người sẽ làm điều đó và 90 người sẽ từ chối bạn (90%). 
+Bạn có quyền từ chối người khác, và thực tế là bạn đang từ chối bắt chuyện với hơn 900 người trong số 1000 người bạn gặp mỗi ngày. Và vì thế, người khác cũng vậy. Việc ngại bị từ chối và không bao giờ chủ động kết nối với ai sẽ làm cửa sổ cơ hội của một người bị thu hẹp lại. Khi một người đưa ra đủ nhiều offer bất kể đó là gì và nhận lại đủ nhiều sự từ chối, họ sẽ từng bước điều chỉnh lại offer cho phù hợp và theo thời gian - tỉ lệ bị từ chối ngày càng giảm đi. Bởi vì họ ngày càng thấu hiểu và nhận định chính xác hơn những gì mà phần đa mọi người quan tâm và thực sự cần. 
+Thực ra bạn nhận được bao nhiêu email mỗi ngày thì nên gửi đi bấy nhiêu email. Người ta có nhiều lý do để không trả lời mail của bạn giữa hàng trăm email khác trong hộp thư. Không sao cả, kể cả khi không nhận lại được hồi âm, bạn vẫn có thể gửi mail follow-up nếu cần thiết. Khi người ta cảm thấy offer đưa ra là phù hợp, họ sẽ trả lời. 
+Tương tự, khi người ta đã quyết định đưa số điện thoại hoặc card cho bạn, có nghĩa là người ta cho phép bạn gọi điện làm phiền họ một chút - hoặc nhiều chút nếu như những gì bạn mang đến cho họ làm cho họ cảm thấy hay và cần phải nghe tiếp. Và lúc đó đã không còn là làm phiền nữa mà là đó là một phần giá trị mà bạn đã mang đến trong cuộc đời của người khác.
+Và một lần nữa, tư bản không thể xuất hiện bên ngoài lưu thông. Lý do mà một người luôn chịu thiệt thòi luôn đến từ sự bất cân xứng thông tin. Sự bất cân xứng thông tin sẽ chỉ luôn mang lại lợi thế cho người có được sự đối xứng về thông tin đó. Chỉ có kết nối và thực sự lắng nghe từ nhiều người mới giúp một người giải quyết bài toán đó. Bạn luôn phải mua mắc vì bạn không biết ở đâu bán rẻ hơn. Bạn phải chấp nhận đồng lương thấp vì bạn không biết ở đâu sẵn sàng trả cho bạn con số cao hơn. Bạn buộc phải nghe và tin cái câu "ở đâu cũng thế thôi" chỉ vì bạn hoàn toàn mù mờ về chỗ khác. Bạn buộc phải tin vào câu "ai mà chả thế" là bởi vì bạn chưa có cơ hội được kết nối và tiếp xúc với những người khác. Và vì thế, thành công của người trẻ đến từ khả năng dám chấp nhận bị từ chối để mở rộng kết nối!
+## Thành công của một người khi về già nằm ở chất lượng danh bạ
+Sẽ đến một lúc nào đó, khả năng thử lại hay tạo dựng một mối quan hệ mới ngày càng giảm sút. Bởi vì lúc này, người đó không còn tuổi trẻ, không còn nhiều thời gian và nguồn lực. Có lẽ lúc này, người đó chỉ muốn rằng một cuộc gọi hoặc một tin nhắn của mình sẽ khiến cho những người thân - không cần biết là đang ở đâu - không cần biết là cuộc sống mưu sinh hiện tại như nào - đều tụ họp và ăn một bữa cơm. Tiền bạc không phải là tất cả nhưng nó quả thực là công cụ hiệu quả để làm điều đó trở nên dễ dàng hơn bao giờ hết. 
+Vì vậy, có lẽ lúc này người đó chỉ muốn một cuộc gọi của mình có thể giải quyết được mọi vấn đề. Gọi cho người có khả năng giải quyết vấn đề đó, và họ bắt máy. Họ lưu danh bạ của người đó ở chế độ ưu tiên cao kể cả khi người đó đã không còn quyền lực hay khả năng như lúc còn trẻ. Họ gửi lời hỏi thăm bản thân người đó và con cháu người đó.  
+Có lẽ chỉ đến phút cuối cùng của cuộc đời một người mới có thể biết được cả cuộc đời người đó là thành công hay thất bại, là hạnh phúc hay khổ đau. Khi bạn nằm trên giường bệnh và chỉ còn một phút, bạn biết rằng thời gian của mình đã hết. Ngay lúc đó, cái tôi, bãn ngã và sự sợ hãi hoàn toàn biến mất và cũng không còn gì là bí mật gì trên đời này nữa. Tất cả những gì còn lại lúc này là tình yêu thương bao quanh bản thân vào khoảnh khắc đó. Con cái, cháu chắt, bạn bè và con cái của bạn bè - tất cả tình yêu thương bao quanh bản thân vào khoảnh khắc đó và tất cả tình yêu thương mà bản thân đã vun đắp suốt cuộc đời này. Định nghĩa của sự thành công ở một đời người nằm ở khoảnh khắc cuối cùng, rằng người đó cảm thấy mình đã đi qua một hành trình tuyệt vời hay vẫn còn nhiều tiếc nuối?</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>&lt;h1 id="tu-ban-khong-the-xuat-hien-ben-ngoai-luu-thong"&gt;Tư bản không thể xuất hiện bên ngoài lưu thông&lt;/h1&gt;
+&lt;p&gt;Tư bản không thể xuất hiện ở bên ngoài lưu thông. Vì vậy, muốn kiếm tiền, một người bắt buộc phải kết nối với thế này! Kết nối giúp cho một người có cơ hội tiếp cận với công việc ngay khi ai đó có dự định tìm nhân sự. Kết nối giúp làm giảm sự bất cân xứng thông tin. Kết nối giúp cho một người nhanh chóng tìm kiếm người phù hợp để giải quyết vấn đề hoặc mở rộng quy mô. Vì vậy, thành công của một người lúc còn trẻ đến từ khả năng chịu đựng sự từ chối. Và thành công của một người lúc về già nằm ở chất lượng danh bạ.  &lt;/p&gt;
+&lt;h2 id="thanh-cong-cua-mot-nguoi-luc-con-tre-en-tu-kha-nang-chiu-ung-su-tu-choi"&gt;Thành công của một người lúc còn trẻ đến từ khả năng chịu đựng sự từ chối&lt;/h2&gt;
+&lt;p&gt;Điều tệ hại nhất mà một người thành công sớm hay gặp phải đó là sự tự mãn. Nói thẳng ra là khi đạt được một thành tựu gì đó hoặc có được một vị trí nào đó - người đó cho rằng mình có đặc quyền "miễn trừ từ chối" và vì thế, được hưởng quyền "miễn trừ thất bại". Chúng ta có thể nhìn thấy điều đó ở bất cứ đâu. Trong chuyện tình cảm, trong các bản hợp đồng chuyển nhượng, sau một mùa giải thể thao chuyên nghiệp kết thúc và các bên tìm kiếm bến đỗ mới, sau khi đạt được một giải thưởng từ một cuộc thi hay tổ chức nào đó,... &lt;/p&gt;
+&lt;p&gt;Công bằng mà nói thì chẳng ai trong chúng ta thích thất bại và sự từ chối. Nếu có ai đó nói tôi thích thì chắc chắn là nói dối - nói dối một cách trắng trợn. Nhưng hãy thực sự nhìn lại và sâu chuỗi lại tất cả mọi thứ từ sâu thẳm trong tim: Bạn học được từ cái gì nhiều nhất? Ai là người thay đổi bạn nhiều nhất? Ai là người củng cố niềm tin của bạn mạnh mẽ nhất? Có phải là từ sự thất bại? Có phải là vì từ người từ chối bạn và mang lại cho bạn điều khổ đau và tuyệt vọng nhất?&lt;/p&gt;
+&lt;p&gt;Thất bại phơi bày bức tranh toàn cảnh một cách sắc nét nhất, thất bại làm cho một người nhìn thấy hầu hết khía cạnh và sắc màu của cuộc sống - thứ mà thành công ít khi nào có thể hiển thị ra. Những năm trung học, khi các bài báo địa phương viết về Hải và bạn bè cũng như phụ huynh đọc được, Hải đã được trải nghiệm cảm giác được nhiều người quan tâm và dành nhiều lời khen trông như nào. Và đó cũng là lúc khả năng đưa ra lời đề nghị và chấp nhận lời từ chối đã bắt đầu xuống mức rất thấp. Vào năm cuối đại học, Hải nói thầy muốn tự ứng cử vào vị trí lớp phó phong trào và được cả lớp đồng ý với tỉ lệ 100% - và tất nhiên cũng là vì vị trí này chẳng có ai đứng ra cạnh tranh với Hải. &lt;/p&gt;
+&lt;p&gt;Nhưng đây cũng là điểm yếu lớn nhất của Hải. Chúng bộc lộ ngay khi Hải bắt đầu làm công việc bán hàng qua điện thoại - hay còn được biết với tên gọi telesale. Chắc mọi người cũng biết nếu như bán những mặt hàng có giá trị cao như ô tô, bất động sản hay bảo hiểm thì tỉ lệ từ chối sẽ là khoảng 99%. Và vì thế, đây là lĩnh vực mà Hải có thể nói là thất bại đúng nghĩa. Thất bại vì để cho cảm xúc khi bị từ chối chi phối. Thất bại khi để cho một cuộc gọi bị cúp máy ngang kéo theo cảm xúc tiêu cực cả ngày. Thất bại khi cho rằng công việc mình đang làm là không nên và không dám nhận là mình làm công việc này. Nhưng Hải không hiểu rằng bản chất của telesale là để đánh giá mức độ quan tâm của khách đối với sản phẩm cũng như khả năng tài chính của khách. Dựa vào gì? Dựa vào tone giọng, thời gian phản hồi, câu trả lời của khách và những câu follow-up phía sau được chuẩn bị cho khách. Từ đó mới xác định đúng những người phù hợp để kết nối cũng như làm cho khách nghĩ đến sale và muốn liên hệ ngay khi muốn mua sản phẩm - thứ mà không một trường học nào dạy. &lt;/p&gt;
+&lt;p&gt;Chúng ta đều đã, đang và sẽ từ chối rất nhiều người. Bao nhiêu người mỗi ngày chúng ta gặp mà chúng ta không chào hỏi, không bắt chuyện? Mỗi ngày chúng ta gặp đâu đó khoảng 1000 người: trên đường đến cơ quan, tại nơi làm việc, tại cửa hàng, tại công viên, tại các câu lạc bộ,... Bao nhiêu người trong số đó bạn nghĩ rằng nên chủ động làm phiền họ một chút? 500, 200, 100, 10, 1 hay không ai cả? Thực ra nếu bạn không chấp nhận rủi ro gây khó chịu một chút với người khác và có thể nhận lại sự từ chối thì sẽ không có điều gì mới tuyệt vời xảy đến với bạn. Nếu bạn dám làm phiền 100 người trong số 1000 người bạn lướt qua mỗi ngày bất kể đó là về cái gì từ nói chuyện phiếm, hỏi han, xin số điện thoại cho tới giới thiệu bản thân và công việc,... - bạn sẽ nhanh chóng trở thành bậc thầy bắt chuyện. Nếu bạn nhìn ngược lại, bạn đã từ chối bắt chuyện với 900 người (khoảng 90% người bạn gặp). Và vì thế, bạn không trông mong cả 100 người bạn làm phiền sẽ níu lại chia sẻ với thật lâu với bạn. Không, chỉ 10 người sẽ làm điều đó và 90 người sẽ từ chối bạn (90%). &lt;/p&gt;
+&lt;p&gt;Bạn có quyền từ chối người khác, và thực tế là bạn đang từ chối bắt chuyện với hơn 900 người trong số 1000 người bạn gặp mỗi ngày. Và vì thế, người khác cũng vậy. Việc ngại bị từ chối và không bao giờ chủ động kết nối với ai sẽ làm cửa sổ cơ hội của một người bị thu hẹp lại. Khi một người đưa ra đủ nhiều offer bất kể đó là gì và nhận lại đủ nhiều sự từ chối, họ sẽ từng bước điều chỉnh lại offer cho phù hợp và theo thời gian - tỉ lệ bị từ chối ngày càng giảm đi. Bởi vì họ ngày càng thấu hiểu và nhận định chính xác hơn những gì mà phần đa mọi người quan tâm và thực sự cần. &lt;/p&gt;
+&lt;p&gt;Thực ra bạn nhận được bao nhiêu email mỗi ngày thì nên gửi đi bấy nhiêu email. Người ta có nhiều lý do để không trả lời mail của bạn giữa hàng trăm email khác trong hộp thư. Không sao cả, kể cả khi không nhận lại được hồi âm, bạn vẫn có thể gửi mail follow-up nếu cần thiết. Khi người ta cảm thấy offer đưa ra là phù hợp, họ sẽ trả lời. &lt;/p&gt;
+&lt;p&gt;Tương tự, khi người ta đã quyết định đưa số điện thoại hoặc card cho bạn, có nghĩa là người ta cho phép bạn gọi điện làm phiền họ một chút - hoặc nhiều chút nếu như những gì bạn mang đến cho họ làm cho họ cảm thấy hay và cần phải nghe tiếp. Và lúc đó đã không còn là làm phiền nữa mà là đó là một phần giá trị mà bạn đã mang đến trong cuộc đời của người khác.&lt;/p&gt;
+&lt;p&gt;Và một lần nữa, tư bản không thể xuất hiện bên ngoài lưu thông. Lý do mà một người luôn chịu thiệt thòi luôn đến từ sự bất cân xứng thông tin. Sự bất cân xứng thông tin sẽ chỉ luôn mang lại lợi thế cho người có được sự đối xứng về thông tin đó. Chỉ có kết nối và thực sự lắng nghe từ nhiều người mới giúp một người giải quyết bài toán đó. Bạn luôn phải mua mắc vì bạn không biết ở đâu bán rẻ hơn. Bạn phải chấp nhận đồng lương thấp vì bạn không biết ở đâu sẵn sàng trả cho bạn con số cao hơn. Bạn buộc phải nghe và tin cái câu "ở đâu cũng thế thôi" chỉ vì bạn hoàn toàn mù mờ về chỗ khác. Bạn buộc phải tin vào câu "ai mà chả thế" là bởi vì bạn chưa có cơ hội được kết nối và tiếp xúc với những người khác. Và vì thế, thành công của người trẻ đến từ khả năng dám chấp nhận bị từ chối để mở rộng kết nối!&lt;/p&gt;
+&lt;h2 id="thanh-cong-cua-mot-nguoi-khi-ve-gia-nam-o-chat-luong-danh-ba"&gt;Thành công của một người khi về già nằm ở chất lượng danh bạ&lt;/h2&gt;
+&lt;p&gt;Sẽ đến một lúc nào đó, khả năng thử lại hay tạo dựng một mối quan hệ mới ngày càng giảm sút. Bởi vì lúc này, người đó không còn tuổi trẻ, không còn nhiều thời gian và nguồn lực. Có lẽ lúc này, người đó chỉ muốn rằng một cuộc gọi hoặc một tin nhắn của mình sẽ khiến cho những người thân - không cần biết là đang ở đâu - không cần biết là cuộc sống mưu sinh hiện tại như nào - đều tụ họp và ăn một bữa cơm. Tiền bạc không phải là tất cả nhưng nó quả thực là công cụ hiệu quả để làm điều đó trở nên dễ dàng hơn bao giờ hết. &lt;/p&gt;
+&lt;p&gt;Vì vậy, có lẽ lúc này người đó chỉ muốn một cuộc gọi của mình có thể giải quyết được mọi vấn đề. Gọi cho người có khả năng giải quyết vấn đề đó, và họ bắt máy. Họ lưu danh bạ của người đó ở chế độ ưu tiên cao kể cả khi người đó đã không còn quyền lực hay khả năng như lúc còn trẻ. Họ gửi lời hỏi thăm bản thân người đó và con cháu người đó.  &lt;/p&gt;
+&lt;p&gt;Có lẽ chỉ đến phút cuối cùng của cuộc đời một người mới có thể biết được cả cuộc đời người đó là thành công hay thất bại, là hạnh phúc hay khổ đau. Khi bạn nằm trên giường bệnh và chỉ còn một phút, bạn biết rằng thời gian của mình đã hết. Ngay lúc đó, cái tôi, bãn ngã và sự sợ hãi hoàn toàn biến mất và cũng không còn gì là bí mật gì trên đời này nữa. Tất cả những gì còn lại lúc này là tình yêu thương bao quanh bản thân vào khoảnh khắc đó. Con cái, cháu chắt, bạn bè và con cái của bạn bè - tất cả tình yêu thương bao quanh bản thân vào khoảnh khắc đó và tất cả tình yêu thương mà bản thân đã vun đắp suốt cuộc đời này. Định nghĩa của sự thành công ở một đời người nằm ở khoảnh khắc cuối cùng, rằng người đó cảm thấy mình đã đi qua một hành trình tuyệt vời hay vẫn còn nhiều tiếc nuối?&lt;/p&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>Tư duy cắt chuỗi</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>tu-duy-cat-chuoi</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr">
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr">
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>Để có thể thích nghi với hầu hết toàn bộ nền tảng, môi trường triển khai trong ngành phần mềm và thông tin, có 1 kỹ thuật mang tên cắt chuỗi. Nó giúp chúng ta vượt qua mọi tư duy và rảo cản về môi trường triển khai, chi phí vận hành. Nó hỗ...</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>data\blogs\Tư duy cắt chuỗi.md</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t># Tư duy cắt chuỗi
 Để có thể thích nghi với hầu hết toàn bộ nền tảng, môi trường triển khai trong ngành phần mềm và thông tin, có 1 kỹ thuật mang tên cắt chuỗi. Nó giúp chúng ta vượt qua mọi tư duy và rảo cản về môi trường triển khai, chi phí vận hành. Nó hỗ trợ chúng ta có nền tảng để tự dụng lên mọi nội dung, hệ thống. Nó chính là bước khác biệt và cũng là bước khó nhất trong toàn bộ quy trình tự động.   
@@ -4641,7 +4897,7 @@
 ## Kết</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="L49" t="inlineStr">
         <is>
           <t>&lt;h1 id="tu-duy-cat-chuoi"&gt;Tư duy cắt chuỗi&lt;/h1&gt;
 &lt;p&gt;Để có thể thích nghi với hầu hết toàn bộ nền tảng, môi trường triển khai trong ngành phần mềm và thông tin, có 1 kỹ thuật mang tên cắt chuỗi. Nó giúp chúng ta vượt qua mọi tư duy và rảo cản về môi trường triển khai, chi phí vận hành. Nó hỗ trợ chúng ta có nền tảng để tự dụng lên mọi nội dung, hệ thống. Nó chính là bước khác biệt và cũng là bước khó nhất trong toàn bộ quy trình tự động.   &lt;/p&gt;
@@ -4657,84 +4913,84 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>Tư duy Excel</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>tu-duy-excel</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr">
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr">
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
         <is>
           <t>data\blogs\Tư duy Excel.md</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>Tư duy ngược và tư duy mở ngành phần mềm</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>tu-duy-nguoc-va-tu-duy-mo-nganh-phan-mem</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr">
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H51" t="inlineStr">
         <is>
           <t>08-06-2026</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>Linux - Windows - Mac</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J51" t="inlineStr">
         <is>
           <t>data\blogs\Tư duy ngược và tư duy mở ngành phần mềm.md</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t># Tư duy ngược và tư duy mở ngành phần mềm
 ## Những thứ có giá trị nhất đôi khi là rẻ nhất hoặc miễn phí
@@ -4743,7 +4999,7 @@
 ## Giải pháp triệu đô</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L51" t="inlineStr">
         <is>
           <t>&lt;h1 id="tu-duy-nguoc-va-tu-duy-mo-nganh-phan-mem"&gt;Tư duy ngược và tư duy mở ngành phần mềm&lt;/h1&gt;
 &lt;h2 id="nhung-thu-co-gia-tri-nhat-oi-khi-la-re-nhat-hoac-mien-phi"&gt;Những thứ có giá trị nhất đôi khi là rẻ nhất hoặc miễn phí&lt;/h2&gt;
@@ -4753,58 +5009,58 @@
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>Tư duy xô nước</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>tu-duy-xo-nuoc</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>Tư duy</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>xô nước, đường ống</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>15-06-2026</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H52" t="inlineStr">
         <is>
           <t>16-06-2026</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>Câu chuyện kể về một thị trấn nọ nơi những ngày đầu các hộ dân đều mang theo xô đến sông để mang nước về nhà mỗi ngày. Về sau, các gia đình chọn trả tiền để thuê những thanh niên trai tráng trong làng xách nước thay vì tự mình mang xô đến....</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>data\blogs\Tư duy xô nước.md</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t># Tư duy xô nước
 Câu chuyện kể về một thị trấn nọ nơi những ngày đầu các hộ dân đều mang theo xô đến sông để mang nước về nhà mỗi ngày. Về sau, các gia đình chọn trả tiền để thuê những thanh niên trai tráng trong làng xách nước thay vì tự mình mang xô đến.  Giai đoạn đầu, các thanh niên trong làng hứng khởi và xách xô nước vì số tiền họ kiếm được phụ thuộc vào số xô nước họ giao. Các gia đình ai ai cũng muốn gả con gái cho những thanh niên chăm chỉ sẵn sàng đi xách nước vào cả khung giờ chiều tối, nửa đêm để đáp ứng nhu cầu sử dụng nước cho nhiều gia đình. Sự thành đạt, tinh thần làm việc chăm chỉ, tương lai cầu tiến được thể hiện bằng số giờ đi xách xô nước và số xô nước họ đã mang đến từng nhà. Các thanh niên ốm yếu, gầy gò trong làng lúc này cũng đã tham gia vì công việc này ngày nào cũng có và không hết việc. Và đó cũng là việc mà các thanh thiếu niên chí khí trong làng lúc bấy giờ nên dấn thân. 
@@ -4834,7 +5090,7 @@
 Một trong những thứ có thể tồn tại lâu hơn tuổi thọ của con người đó là đường ống. Con người rồi sẽ già đi. Sức khỏe rồi sẽ suy giảm. Thời gian của mỗi người đều có giới hạn. Nhưng những gì chúng ta để lại thì không nhất thiết phải biến mất. Ai cũng có thể phải xách xô ở một giai đoạn nào đó của cuộc đời. Không có gì đáng xấu hổ khi dùng thời gian và sức lao động để kiếm sống. Vấn đề chỉ nằm ở chỗ: liệu sau mỗi ngày xách xô, chúng ta có dành ra một phần thời gian để xây đường ống hay không? Bởi vì đến một lúc nào đó, thứ quyết định giá trị của một con người không còn là họ đã đổ bao nhiêu mồ hôi, thức bao nhiêu đêm hay làm việc bao nhiêu giờ mỗi ngày, mà là những gì vẫn tiếp tục tạo ra giá trị ngay cả khi họ không còn ở đó.</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
+      <c r="L52" t="inlineStr">
         <is>
           <t>&lt;h1 id="tu-duy-xo-nuoc"&gt;Tư duy xô nước&lt;/h1&gt;
 &lt;p&gt;Câu chuyện kể về một thị trấn nọ nơi những ngày đầu các hộ dân đều mang theo xô đến sông để mang nước về nhà mỗi ngày. Về sau, các gia đình chọn trả tiền để thuê những thanh niên trai tráng trong làng xách nước thay vì tự mình mang xô đến.  Giai đoạn đầu, các thanh niên trong làng hứng khởi và xách xô nước vì số tiền họ kiếm được phụ thuộc vào số xô nước họ giao. Các gia đình ai ai cũng muốn gả con gái cho những thanh niên chăm chỉ sẵn sàng đi xách nước vào cả khung giờ chiều tối, nửa đêm để đáp ứng nhu cầu sử dụng nước cho nhiều gia đình. Sự thành đạt, tinh thần làm việc chăm chỉ, tương lai cầu tiến được thể hiện bằng số giờ đi xách xô nước và số xô nước họ đã mang đến từng nhà. Các thanh niên ốm yếu, gầy gò trong làng lúc này cũng đã tham gia vì công việc này ngày nào cũng có và không hết việc. Và đó cũng là việc mà các thanh thiếu niên chí khí trong làng lúc bấy giờ nên dấn thân. &lt;/p&gt;
@@ -4865,54 +5121,54 @@
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>Tại sao Bitcoin cưa đôi?</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>tai-sao-bitcoin-cua-doi</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>Công nghệ</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr">
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải...</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="J53" t="inlineStr">
         <is>
           <t>data\blogs\Tại sao Bitcon cưa đôi.md</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t># Tại sao Bitcoin cưa đôi?
 Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải có đáng để đọc và có đủ sức thuyết phục hay không?". Hải hoàn toàn hiểu, và cũng theo một góc độ nào đó, chính vì Hải chưa từng được hưởng lợi hay chịu thiệt hại từ Bitcoin, anh em có thể tham khảo bài viết từ một người có góc nhìn trung lập. Mục tiêu của bài viết là đưa ra thật nhiều góc nhìn vì cho tới nay vẫn có rất nhiều ý kiến trái chiều về tiền mã hóa. Có người thì bảo rằng đó là công nghệ tương lai của nhân loại, cũng có người nói đó là trò lừa bịp, lừa đảo và rửa tiền. Vì vậy, muốn biết nó thực sự là gì, chúng ta phải thảo luận về nó, phải đặt câu hỏi về nó, phải xem qua các trường hợp trước đây nó được sử dụng cho mục đích gì?
@@ -4978,7 +5234,7 @@
 [^3]: [Controlled supply - Bitcoin Wiki](https://en.bitcoin.it/wiki/Controlled_supply)</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="L53" t="inlineStr">
         <is>
           <t>&lt;h1 id="tai-sao-bitcoin-cua-oi"&gt;Tại sao Bitcoin cưa đôi?&lt;/h1&gt;
 &lt;p&gt;Trước khi bắt đầu bài viết, Hải muốn nhấn mạnh rằng Hải chưa từng tham gia đầu tư, giao dịch hay đào crypto trước đây. Tất nhiên anh em hoàn toàn có thể thắc mắc rằng: "Nếu Hải chưa từng đụng vào Bitcoin thì liệu bài viết về Bitcoin của Hải có đáng để đọc và có đủ sức thuyết phục hay không?". Hải hoàn toàn hiểu, và cũng theo một góc độ nào đó, chính vì Hải chưa từng được hưởng lợi hay chịu thiệt hại từ Bitcoin, anh em có thể tham khảo bài viết từ một người có góc nhìn trung lập. Mục tiêu của bài viết là đưa ra thật nhiều góc nhìn vì cho tới nay vẫn có rất nhiều ý kiến trái chiều về tiền mã hóa. Có người thì bảo rằng đó là công nghệ tương lai của nhân loại, cũng có người nói đó là trò lừa bịp, lừa đảo và rửa tiền. Vì vậy, muốn biết nó thực sự là gì, chúng ta phải thảo luận về nó, phải đặt câu hỏi về nó, phải xem qua các trường hợp trước đây nó được sử dụng cho mục đích gì?&lt;/p&gt;
@@ -5070,104 +5326,104 @@
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
         <is>
           <t>Tại sao lại là Blockchain</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>tai-sao-lai-la-blockchain</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>Công nghệ</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr">
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H54" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr">
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
         <is>
           <t>data\blogs\Tại sao lại là Blockchain.md</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t># Tại sao lại là Blockchain?</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="L54" t="inlineStr">
         <is>
           <t>&lt;h1 id="tai-sao-lai-la-blockchain"&gt;Tại sao lại là Blockchain?&lt;/h1&gt;</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t>Tại sao lại là start-up?</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>tai-sao-lai-la-start-up</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr">
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr">
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
         <is>
           <t>27-08-2026</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H55" t="inlineStr">
         <is>
           <t>02-09-2026</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="I55" t="inlineStr">
         <is>
           <t>&gt; "Đừng bao giờ đánh mất đi ước mơ và khát vọng của chính mình. Vì nếu bạn làm thế, bạn có lẽ vẫn sẽ tồn tại nhưng bạn đã ngừng sống mất rồi!" &gt; &gt; _- Henry David Thoreau_</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="J55" t="inlineStr">
         <is>
           <t>data\blogs\Tại sao lại là start-up.md</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="K55" t="inlineStr">
         <is>
           <t># Tại sao lại là start-up?
 &gt; "Đừng bao giờ đánh mất đi ước mơ và khát vọng của chính mình. Vì nếu bạn làm thế, bạn có lẽ vẫn sẽ tồn tại nhưng bạn đã ngừng sống mất rồi!"
@@ -5198,7 +5454,7 @@
 Xã hội thay đổi thì con người và tổ chức cũng cần đổi thay. Và bất kể sự lựa chọn của mỗi người có là gì, miễn là sống thật tốt - đều xứng đáng được trân trọng.</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr">
+      <c r="L55" t="inlineStr">
         <is>
           <t>&lt;h1 id="tai-sao-lai-la-start-up"&gt;Tại sao lại là start-up?&lt;/h1&gt;
 &lt;blockquote&gt;
@@ -5232,56 +5488,56 @@
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
+    <row r="56">
+      <c r="A56" t="inlineStr">
         <is>
           <t>Vì sao con người tự ti</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>vi-sao-con-nguoi-tu-ti</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>in-draft</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr">
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr">
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
         <is>
           <t>23-07-2026</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="H56" t="inlineStr">
         <is>
           <t>23-07-2026</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t>- [ ] họ không tự hào về bản thân họ, về môi trường họ sinh ra, về</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="J56" t="inlineStr">
         <is>
           <t>data\blogs\Vì sao con người tự ti.md</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t># Vì sao con người tự ti?
 - [ ] họ không tự hào về bản thân họ, về môi trường họ sinh ra, về</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr">
+      <c r="L56" t="inlineStr">
         <is>
           <t>&lt;h1 id="vi-sao-con-nguoi-tu-ti"&gt;Vì sao con người tự ti?&lt;/h1&gt;
 &lt;ul class="task-list"&gt;
@@ -5290,84 +5546,84 @@
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
+    <row r="57">
+      <c r="A57" t="inlineStr">
         <is>
           <t>Vì sao khởi nghiệp thất bại</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>vi-sao-khoi-nghiep-that-bai</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr">
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H57" t="inlineStr">
         <is>
           <t>20-07-2026</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr">
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
         <is>
           <t>data\blogs\Vì sao khởi nghiệp thất bại.md</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
+    <row r="58">
+      <c r="A58" t="inlineStr">
         <is>
           <t>Vì sao người giàu thích nợ?</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>vi-sao-nguoi-giau-thich-no</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr">
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
         <is>
           <t>Quý Hải Ng</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr">
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
         <is>
           <t>23-06-2026</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="H58" t="inlineStr">
         <is>
           <t>02-07-2026</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I58" t="inlineStr">
         <is>
           <t>Có 1 lần trong cuộc phỏng vấn, tổng thống thứ 45 và 47 của Hoa Kỳ - Donald Trump có chia sẻ về câu chuyện cho tiền người giàu hơn ông khoảng 900 triệu đô. Đó là một ngày khi ông cùng người đẹp dạo phố và ông Trump nói với cô gái: “Em biết n...</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="J58" t="inlineStr">
         <is>
           <t>data\blogs\Vì sao người giàu thích nợ.md</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="K58" t="inlineStr">
         <is>
           <t># Vì sao người giàu thích nợ
 Có 1 lần trong cuộc phỏng vấn, tổng thống thứ 45 và 47 của Hoa Kỳ - Donald Trump có chia sẻ về câu chuyện cho tiền người giàu hơn ông khoảng 900 triệu đô. Đó là một ngày khi ông cùng người đẹp dạo phố và ông Trump nói với cô gái: “Em biết người đàn ông đó là ai không?”. “Em biết, ông ấy là ăn xin” - cô gái đáp. Ông Trump nói tiếp: “Ngay bây giờ, ông ấy đang có nhiều hơn anh 900 triệu đô”. Và cô gái thắc mắc: “Làm sao người ăn xin có thể có nhiều tiền hơn ông được?”. Bởi vì người ăn xin tuy  không có đồng nào nhưng cũng không có nợ. Trong khi đó, ông Trump nợ 900 triệu đô. Đó là thời điểm bất động sản ở Mỹ đang ở dưới đáy chu kỳ vào những năm đầu thập niên 90. Và tất nhiên sau đó, thị trường bất động sản ở New York mà ông Trump đầu tư xây dựng đã phát triển bùng nổ.
@@ -5402,7 +5658,7 @@
 Cái gì quan trọng thì nhắc lại ba lần: “Ai sinh ra trên đời cũng chỉ có 2 bàn tay trắng và sẽ không cầm theo được bất cứ thứ gì khi rời đi”. Nhìn nhận về nợ ra sao, đó là quan điểm của mỗi người. Chúng ta chỉ biết rằng, trong lịch sử loài người, nếu không có thứ đó, sẽ mất rất lâu nữa để có hàng ngàn sa số những công trình, công nghệ được xây dựng và phát triển tới tận ngày nay. Không có thứ đó, hàng triệu triệu người sẽ phải chôn vùi giấc mơ, những điều mình muốn làm và mang theo nó sang thế giới bên kia thay vì để lại cho nhân loại.</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr">
+      <c r="L58" t="inlineStr">
         <is>
           <t>&lt;h1 id="vi-sao-nguoi-giau-thich-no"&gt;Vì sao người giàu thích nợ&lt;/h1&gt;
 &lt;p&gt;Có 1 lần trong cuộc phỏng vấn, tổng thống thứ 45 và 47 của Hoa Kỳ - Donald Trump có chia sẻ về câu chuyện cho tiền người giàu hơn ông khoảng 900 triệu đô. Đó là một ngày khi ông cùng người đẹp dạo phố và ông Trump nói với cô gái: “Em biết người đàn ông đó là ai không?”. “Em biết, ông ấy là ăn xin” - cô gái đáp. Ông Trump nói tiếp: “Ngay bây giờ, ông ấy đang có nhiều hơn anh 900 triệu đô”. Và cô gái thắc mắc: “Làm sao người ăn xin có thể có nhiều tiền hơn ông được?”. Bởi vì người ăn xin tuy  không có đồng nào nhưng cũng không có nợ. Trong khi đó, ông Trump nợ 900 triệu đô. Đó là thời điểm bất động sản ở Mỹ đang ở dưới đáy chu kỳ vào những năm đầu thập niên 90. Và tất nhiên sau đó, thị trường bất động sản ở New York mà ông Trump đầu tư xây dựng đã phát triển bùng nổ.&lt;/p&gt;
@@ -5438,50 +5694,50 @@
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
+    <row r="59">
+      <c r="A59" t="inlineStr">
         <is>
           <t>Điều mà nhà trường không bao giờ nói với anh em</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>dieu-ma-nha-truong-khong-bao-gio-noi-voi-anh-em</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>Kinh tế</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr">
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
         <is>
           <t>25-05-2026</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="H59" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I59" t="inlineStr">
         <is>
           <t>Hầu hết chúng ta được dạy rằng, phải học thật giỏi, thi vào những trường tốt nhất thì mới có cơ hội vào được 1 công ty tốt. Sau đó làm việc thật chăm chỉ, 8 tiếng mỗi ngày, 5 ngày mỗi tuần, có thể chủ động xin tăng ca để tích lũy thêm tiền...</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="J59" t="inlineStr">
         <is>
           <t>data\blogs\Điều mà nhà trường không bao giờ nói với anh em.md</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="K59" t="inlineStr">
         <is>
           <t># Điều mà nhà trường không bao giờ nói với anh em
 ## 2 kiểu tư duy về tiền
@@ -5528,7 +5784,7 @@
 Tâm lý học về tiền</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr">
+      <c r="L59" t="inlineStr">
         <is>
           <t>&lt;h1 id="ieu-ma-nha-truong-khong-bao-gio-noi-voi-anh-em"&gt;Điều mà nhà trường không bao giờ nói với anh em&lt;/h1&gt;
 &lt;h2 id="2-kieu-tu-duy-ve-tien"&gt;2 kiểu tư duy về tiền&lt;/h2&gt;

</xml_diff>

<commit_message>
Tu ban khong the xuat hien ben ngoai luu thong 2nd edited
</commit_message>
<xml_diff>
--- a/data/blog_list.xlsx
+++ b/data/blog_list.xlsx
@@ -4785,12 +4785,12 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>12-10-2026</t>
+          <t>13-10-2026</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Tư bản không thể xuất hiện ở bên ngoài lưu thông. Vì vậy, muốn kiếm tiền, một người bắt buộc phải kết nối với thế này! Kết nối giúp cho một người có cơ hội tiếp cận với công việc ngay khi ai đó có dự định tìm nhân sự. Kết nối giúp làm giảm...</t>
+          <t>Tư bản không thể xuất hiện ở bên ngoài lưu thông. Vì vậy, muốn kiếm tiền, một người bắt buộc phải kết nối với thế giới này! Kết nối giúp cho một người có cơ hội tiếp cận với công việc ngay khi ai đó có dự định tìm nhân sự. Kết nối giúp làm...</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -4801,17 +4801,17 @@
       <c r="K48" t="inlineStr">
         <is>
           <t># Tư bản không thể xuất hiện bên ngoài lưu thông
-Tư bản không thể xuất hiện ở bên ngoài lưu thông. Vì vậy, muốn kiếm tiền, một người bắt buộc phải kết nối với thế này! Kết nối giúp cho một người có cơ hội tiếp cận với công việc ngay khi ai đó có dự định tìm nhân sự. Kết nối giúp làm giảm sự bất cân xứng thông tin. Kết nối giúp cho một người nhanh chóng tìm kiếm người phù hợp để giải quyết vấn đề hoặc mở rộng quy mô. Vì vậy, thành công của một người lúc còn trẻ đến từ khả năng chịu đựng sự từ chối. Và thành công của một người lúc về già nằm ở chất lượng danh bạ.  
+Tư bản không thể xuất hiện ở bên ngoài lưu thông. Vì vậy, muốn kiếm tiền, một người bắt buộc phải kết nối với thế giới này! Kết nối giúp cho một người có cơ hội tiếp cận với công việc ngay khi ai đó có dự định tìm nhân sự. Kết nối giúp làm giảm sự bất cân xứng thông tin. Kết nối giúp cho một người nhanh chóng tìm kiếm người phù hợp để giải quyết vấn đề hoặc mở rộng quy mô. Vì vậy, thành công của một người lúc còn trẻ đến từ khả năng chịu đựng sự từ chối. Và thành công của một người lúc về già nằm ở chất lượng danh bạ.  
 ## Thành công của một người lúc còn trẻ đến từ khả năng chịu đựng sự từ chối
 Điều tệ hại nhất mà một người thành công sớm hay gặp phải đó là sự tự mãn. Nói thẳng ra là khi đạt được một thành tựu gì đó hoặc có được một vị trí nào đó - người đó cho rằng mình có đặc quyền "miễn trừ từ chối" và vì thế, được hưởng quyền "miễn trừ thất bại". Chúng ta có thể nhìn thấy điều đó ở bất cứ đâu. Trong chuyện tình cảm, trong các bản hợp đồng chuyển nhượng, sau một mùa giải thể thao chuyên nghiệp kết thúc và các bên tìm kiếm bến đỗ mới, sau khi đạt được một giải thưởng từ một cuộc thi hay tổ chức nào đó,... 
-Công bằng mà nói thì chẳng ai trong chúng ta thích thất bại và sự từ chối. Nếu có ai đó nói tôi thích thì chắc chắn là nói dối - nói dối một cách trắng trợn. Nhưng hãy thực sự nhìn lại và sâu chuỗi lại tất cả mọi thứ từ sâu thẳm trong tim: Bạn học được từ cái gì nhiều nhất? Ai là người thay đổi bạn nhiều nhất? Ai là người củng cố niềm tin của bạn mạnh mẽ nhất? Có phải là từ sự thất bại? Có phải là vì từ người từ chối bạn và mang lại cho bạn điều khổ đau và tuyệt vọng nhất?
+Công bằng mà nói thì chẳng ai trong chúng ta thích thất bại và sự từ chối. Nếu có ai đó nói tôi thích thì chắc chắn là nói dối - nói dối một cách trắng trợn. Nhưng hãy thực sự nhìn lại và sâu chuỗi lại tất cả mọi thứ từ sâu thẳm trong tim: Bạn học được từ cái gì nhiều nhất? Ai là người thay đổi bạn nhiều nhất? Ai là người củng cố niềm tin của bạn mạnh mẽ nhất? Có phải là từ sự thất bại? Có phải là từ người từ chối bạn và mang lại cho bạn điều khổ đau và tuyệt vọng nhất?
 Thất bại phơi bày bức tranh toàn cảnh một cách sắc nét nhất, thất bại làm cho một người nhìn thấy hầu hết khía cạnh và sắc màu của cuộc sống - thứ mà thành công ít khi nào có thể hiển thị ra. Những năm trung học, khi các bài báo địa phương viết về Hải và bạn bè cũng như phụ huynh đọc được, Hải đã được trải nghiệm cảm giác được nhiều người quan tâm và dành nhiều lời khen trông như nào. Và đó cũng là lúc khả năng đưa ra lời đề nghị và chấp nhận lời từ chối đã bắt đầu xuống mức rất thấp. Vào năm cuối đại học, Hải nói thầy muốn tự ứng cử vào vị trí lớp phó phong trào và được cả lớp đồng ý với tỉ lệ 100% - và tất nhiên cũng là vì vị trí này chẳng có ai đứng ra cạnh tranh với Hải. 
 Nhưng đây cũng là điểm yếu lớn nhất của Hải. Chúng bộc lộ ngay khi Hải bắt đầu làm công việc bán hàng qua điện thoại - hay còn được biết với tên gọi telesale. Chắc mọi người cũng biết nếu như bán những mặt hàng có giá trị cao như ô tô, bất động sản hay bảo hiểm thì tỉ lệ từ chối sẽ là khoảng 99%. Và vì thế, đây là lĩnh vực mà Hải có thể nói là thất bại đúng nghĩa. Thất bại vì để cho cảm xúc khi bị từ chối chi phối. Thất bại khi để cho một cuộc gọi bị cúp máy ngang kéo theo cảm xúc tiêu cực cả ngày. Thất bại khi cho rằng công việc mình đang làm là không nên và không dám nhận là mình làm công việc này. Nhưng Hải không hiểu rằng bản chất của telesale là để đánh giá mức độ quan tâm của khách đối với sản phẩm cũng như khả năng tài chính của khách. Dựa vào gì? Dựa vào tone giọng, thời gian phản hồi, câu trả lời của khách và những câu follow-up phía sau được chuẩn bị cho khách. Từ đó mới xác định đúng những người phù hợp để kết nối cũng như làm cho khách nghĩ đến sale và muốn liên hệ ngay khi muốn mua sản phẩm - thứ mà không một trường học nào dạy. 
 Chúng ta đều đã, đang và sẽ từ chối rất nhiều người. Bao nhiêu người mỗi ngày chúng ta gặp mà chúng ta không chào hỏi, không bắt chuyện? Mỗi ngày chúng ta gặp đâu đó khoảng 1000 người: trên đường đến cơ quan, tại nơi làm việc, tại cửa hàng, tại công viên, tại các câu lạc bộ,... Bao nhiêu người trong số đó bạn nghĩ rằng nên chủ động làm phiền họ một chút? 500, 200, 100, 10, 1 hay không ai cả? Thực ra nếu bạn không chấp nhận rủi ro gây khó chịu một chút với người khác và có thể nhận lại sự từ chối thì sẽ không có điều gì mới tuyệt vời xảy đến với bạn. Nếu bạn dám làm phiền 100 người trong số 1000 người bạn lướt qua mỗi ngày bất kể đó là về cái gì từ nói chuyện phiếm, hỏi han, xin số điện thoại cho tới giới thiệu bản thân và công việc,... - bạn sẽ nhanh chóng trở thành bậc thầy bắt chuyện. Nếu bạn nhìn ngược lại, bạn đã từ chối bắt chuyện với 900 người (khoảng 90% người bạn gặp). Và vì thế, bạn không trông mong cả 100 người bạn làm phiền sẽ níu lại chia sẻ với thật lâu với bạn. Không, chỉ 10 người sẽ làm điều đó và 90 người sẽ từ chối bạn (90%). 
-Bạn có quyền từ chối người khác, và thực tế là bạn đang từ chối bắt chuyện với hơn 900 người trong số 1000 người bạn gặp mỗi ngày. Và vì thế, người khác cũng vậy. Việc ngại bị từ chối và không bao giờ chủ động kết nối với ai sẽ làm cửa sổ cơ hội của một người bị thu hẹp lại. Khi một người đưa ra đủ nhiều offer bất kể đó là gì và nhận lại đủ nhiều sự từ chối, họ sẽ từng bước điều chỉnh lại offer cho phù hợp và theo thời gian - tỉ lệ bị từ chối ngày càng giảm đi. Bởi vì họ ngày càng thấu hiểu và nhận định chính xác hơn những gì mà phần đa mọi người quan tâm và thực sự cần. 
+Bạn có quyền từ chối người khác, và thực tế là bạn đang từ chối bắt chuyện với hơn 900 người trong số 1000 người bạn gặp mỗi ngày. Và vì thế, người khác cũng vậy. Việc ngại bị từ chối và không bao giờ chủ động kết nối với ai sẽ làm cửa sổ cơ hội của một người bị thu hẹp lại. Khi một người đưa ra đủ nhiều offer bất kể đó là gì và nhận lại đủ nhiều sự từ chối, họ sẽ từng bước điều chỉnh lại offer cho phù hợp và theo thời gian, tỉ lệ bị từ chối ngày càng giảm đi. Bởi vì họ ngày càng thấu hiểu và nhận định chính xác hơn những gì mà phần đa mọi người quan tâm và thực sự cần. 
 Thực ra bạn nhận được bao nhiêu email mỗi ngày thì nên gửi đi bấy nhiêu email. Người ta có nhiều lý do để không trả lời mail của bạn giữa hàng trăm email khác trong hộp thư. Không sao cả, kể cả khi không nhận lại được hồi âm, bạn vẫn có thể gửi mail follow-up nếu cần thiết. Khi người ta cảm thấy offer đưa ra là phù hợp, họ sẽ trả lời. 
-Tương tự, khi người ta đã quyết định đưa số điện thoại hoặc card cho bạn, có nghĩa là người ta cho phép bạn gọi điện làm phiền họ một chút - hoặc nhiều chút nếu như những gì bạn mang đến cho họ làm cho họ cảm thấy hay và cần phải nghe tiếp. Và lúc đó đã không còn là làm phiền nữa mà là đó là một phần giá trị mà bạn đã mang đến trong cuộc đời của người khác.
-Và một lần nữa, tư bản không thể xuất hiện bên ngoài lưu thông. Lý do mà một người luôn chịu thiệt thòi luôn đến từ sự bất cân xứng thông tin. Sự bất cân xứng thông tin sẽ chỉ luôn mang lại lợi thế cho người có được sự đối xứng về thông tin đó. Chỉ có kết nối và thực sự lắng nghe từ nhiều người mới giúp một người giải quyết bài toán đó. Bạn luôn phải mua mắc vì bạn không biết ở đâu bán rẻ hơn. Bạn phải chấp nhận đồng lương thấp vì bạn không biết ở đâu sẵn sàng trả cho bạn con số cao hơn. Bạn buộc phải nghe và tin cái câu "ở đâu cũng thế thôi" chỉ vì bạn hoàn toàn mù mờ về chỗ khác. Bạn buộc phải tin vào câu "ai mà chả thế" là bởi vì bạn chưa có cơ hội được kết nối và tiếp xúc với những người khác. Và vì thế, thành công của người trẻ đến từ khả năng dám chấp nhận bị từ chối để mở rộng kết nối!
+Tương tự, khi người ta đã quyết định đưa số điện thoại hoặc card cho bạn, có nghĩa là người ta cho phép bạn gọi điện làm phiền họ một chút - hoặc nhiều chút nếu như những gì bạn mang đến cho họ làm cho họ cảm thấy hay và cần phải nghe tiếp. Và lúc đó đã không còn là làm phiền nữa mà là đó là một phần giá trị bạn đã mang đến trong cuộc đời của người khác.
+Và một lần nữa, tư bản không thể xuất hiện bên ngoài lưu thông. Lý do mà một người chịu thiệt thòi luôn đến từ sự bất cân xứng thông tin. Sự bất cân xứng thông tin sẽ chỉ luôn mang lại lợi thế cho người có được sự đối xứng về thông tin đó. Chỉ có kết nối và thực sự lắng nghe từ nhiều người mới giúp một người giải quyết bài toán đó. Bạn luôn phải mua mắc vì bạn không biết ở đâu bán rẻ hơn. Bạn phải chấp nhận đồng lương thấp vì bạn không biết ở đâu sẵn sàng trả cho bạn con số cao hơn. Bạn buộc phải nghe và tin cái câu "ở đâu cũng thế thôi" chỉ vì bạn hoàn toàn mù mờ về chỗ khác. Bạn buộc phải tin vào câu "ai mà chả thế" là bởi vì bạn chưa có cơ hội được kết nối và tiếp xúc với những người khác. Và vì thế, thành công của người trẻ đến từ khả năng dám chấp nhận bị từ chối để mở rộng kết nối!
 ## Thành công của một người khi về già nằm ở chất lượng danh bạ
 Sẽ đến một lúc nào đó, khả năng thử lại hay tạo dựng một mối quan hệ mới ngày càng giảm sút. Bởi vì lúc này, người đó không còn tuổi trẻ, không còn nhiều thời gian và nguồn lực. Có lẽ lúc này, người đó chỉ muốn rằng một cuộc gọi hoặc một tin nhắn của mình sẽ khiến cho những người thân - không cần biết là đang ở đâu - không cần biết là cuộc sống mưu sinh hiện tại như nào - đều tụ họp và ăn một bữa cơm. Tiền bạc không phải là tất cả nhưng nó quả thực là công cụ hiệu quả để làm điều đó trở nên dễ dàng hơn bao giờ hết. 
 Vì vậy, có lẽ lúc này người đó chỉ muốn một cuộc gọi của mình có thể giải quyết được mọi vấn đề. Gọi cho người có khả năng giải quyết vấn đề đó, và họ bắt máy. Họ lưu danh bạ của người đó ở chế độ ưu tiên cao kể cả khi người đó đã không còn quyền lực hay khả năng như lúc còn trẻ. Họ gửi lời hỏi thăm bản thân người đó và con cháu người đó.  
@@ -4821,17 +4821,17 @@
       <c r="L48" t="inlineStr">
         <is>
           <t>&lt;h1 id="tu-ban-khong-the-xuat-hien-ben-ngoai-luu-thong"&gt;Tư bản không thể xuất hiện bên ngoài lưu thông&lt;/h1&gt;
-&lt;p&gt;Tư bản không thể xuất hiện ở bên ngoài lưu thông. Vì vậy, muốn kiếm tiền, một người bắt buộc phải kết nối với thế này! Kết nối giúp cho một người có cơ hội tiếp cận với công việc ngay khi ai đó có dự định tìm nhân sự. Kết nối giúp làm giảm sự bất cân xứng thông tin. Kết nối giúp cho một người nhanh chóng tìm kiếm người phù hợp để giải quyết vấn đề hoặc mở rộng quy mô. Vì vậy, thành công của một người lúc còn trẻ đến từ khả năng chịu đựng sự từ chối. Và thành công của một người lúc về già nằm ở chất lượng danh bạ.  &lt;/p&gt;
+&lt;p&gt;Tư bản không thể xuất hiện ở bên ngoài lưu thông. Vì vậy, muốn kiếm tiền, một người bắt buộc phải kết nối với thế giới này! Kết nối giúp cho một người có cơ hội tiếp cận với công việc ngay khi ai đó có dự định tìm nhân sự. Kết nối giúp làm giảm sự bất cân xứng thông tin. Kết nối giúp cho một người nhanh chóng tìm kiếm người phù hợp để giải quyết vấn đề hoặc mở rộng quy mô. Vì vậy, thành công của một người lúc còn trẻ đến từ khả năng chịu đựng sự từ chối. Và thành công của một người lúc về già nằm ở chất lượng danh bạ.  &lt;/p&gt;
 &lt;h2 id="thanh-cong-cua-mot-nguoi-luc-con-tre-en-tu-kha-nang-chiu-ung-su-tu-choi"&gt;Thành công của một người lúc còn trẻ đến từ khả năng chịu đựng sự từ chối&lt;/h2&gt;
 &lt;p&gt;Điều tệ hại nhất mà một người thành công sớm hay gặp phải đó là sự tự mãn. Nói thẳng ra là khi đạt được một thành tựu gì đó hoặc có được một vị trí nào đó - người đó cho rằng mình có đặc quyền "miễn trừ từ chối" và vì thế, được hưởng quyền "miễn trừ thất bại". Chúng ta có thể nhìn thấy điều đó ở bất cứ đâu. Trong chuyện tình cảm, trong các bản hợp đồng chuyển nhượng, sau một mùa giải thể thao chuyên nghiệp kết thúc và các bên tìm kiếm bến đỗ mới, sau khi đạt được một giải thưởng từ một cuộc thi hay tổ chức nào đó,... &lt;/p&gt;
-&lt;p&gt;Công bằng mà nói thì chẳng ai trong chúng ta thích thất bại và sự từ chối. Nếu có ai đó nói tôi thích thì chắc chắn là nói dối - nói dối một cách trắng trợn. Nhưng hãy thực sự nhìn lại và sâu chuỗi lại tất cả mọi thứ từ sâu thẳm trong tim: Bạn học được từ cái gì nhiều nhất? Ai là người thay đổi bạn nhiều nhất? Ai là người củng cố niềm tin của bạn mạnh mẽ nhất? Có phải là từ sự thất bại? Có phải là vì từ người từ chối bạn và mang lại cho bạn điều khổ đau và tuyệt vọng nhất?&lt;/p&gt;
+&lt;p&gt;Công bằng mà nói thì chẳng ai trong chúng ta thích thất bại và sự từ chối. Nếu có ai đó nói tôi thích thì chắc chắn là nói dối - nói dối một cách trắng trợn. Nhưng hãy thực sự nhìn lại và sâu chuỗi lại tất cả mọi thứ từ sâu thẳm trong tim: Bạn học được từ cái gì nhiều nhất? Ai là người thay đổi bạn nhiều nhất? Ai là người củng cố niềm tin của bạn mạnh mẽ nhất? Có phải là từ sự thất bại? Có phải là từ người từ chối bạn và mang lại cho bạn điều khổ đau và tuyệt vọng nhất?&lt;/p&gt;
 &lt;p&gt;Thất bại phơi bày bức tranh toàn cảnh một cách sắc nét nhất, thất bại làm cho một người nhìn thấy hầu hết khía cạnh và sắc màu của cuộc sống - thứ mà thành công ít khi nào có thể hiển thị ra. Những năm trung học, khi các bài báo địa phương viết về Hải và bạn bè cũng như phụ huynh đọc được, Hải đã được trải nghiệm cảm giác được nhiều người quan tâm và dành nhiều lời khen trông như nào. Và đó cũng là lúc khả năng đưa ra lời đề nghị và chấp nhận lời từ chối đã bắt đầu xuống mức rất thấp. Vào năm cuối đại học, Hải nói thầy muốn tự ứng cử vào vị trí lớp phó phong trào và được cả lớp đồng ý với tỉ lệ 100% - và tất nhiên cũng là vì vị trí này chẳng có ai đứng ra cạnh tranh với Hải. &lt;/p&gt;
 &lt;p&gt;Nhưng đây cũng là điểm yếu lớn nhất của Hải. Chúng bộc lộ ngay khi Hải bắt đầu làm công việc bán hàng qua điện thoại - hay còn được biết với tên gọi telesale. Chắc mọi người cũng biết nếu như bán những mặt hàng có giá trị cao như ô tô, bất động sản hay bảo hiểm thì tỉ lệ từ chối sẽ là khoảng 99%. Và vì thế, đây là lĩnh vực mà Hải có thể nói là thất bại đúng nghĩa. Thất bại vì để cho cảm xúc khi bị từ chối chi phối. Thất bại khi để cho một cuộc gọi bị cúp máy ngang kéo theo cảm xúc tiêu cực cả ngày. Thất bại khi cho rằng công việc mình đang làm là không nên và không dám nhận là mình làm công việc này. Nhưng Hải không hiểu rằng bản chất của telesale là để đánh giá mức độ quan tâm của khách đối với sản phẩm cũng như khả năng tài chính của khách. Dựa vào gì? Dựa vào tone giọng, thời gian phản hồi, câu trả lời của khách và những câu follow-up phía sau được chuẩn bị cho khách. Từ đó mới xác định đúng những người phù hợp để kết nối cũng như làm cho khách nghĩ đến sale và muốn liên hệ ngay khi muốn mua sản phẩm - thứ mà không một trường học nào dạy. &lt;/p&gt;
 &lt;p&gt;Chúng ta đều đã, đang và sẽ từ chối rất nhiều người. Bao nhiêu người mỗi ngày chúng ta gặp mà chúng ta không chào hỏi, không bắt chuyện? Mỗi ngày chúng ta gặp đâu đó khoảng 1000 người: trên đường đến cơ quan, tại nơi làm việc, tại cửa hàng, tại công viên, tại các câu lạc bộ,... Bao nhiêu người trong số đó bạn nghĩ rằng nên chủ động làm phiền họ một chút? 500, 200, 100, 10, 1 hay không ai cả? Thực ra nếu bạn không chấp nhận rủi ro gây khó chịu một chút với người khác và có thể nhận lại sự từ chối thì sẽ không có điều gì mới tuyệt vời xảy đến với bạn. Nếu bạn dám làm phiền 100 người trong số 1000 người bạn lướt qua mỗi ngày bất kể đó là về cái gì từ nói chuyện phiếm, hỏi han, xin số điện thoại cho tới giới thiệu bản thân và công việc,... - bạn sẽ nhanh chóng trở thành bậc thầy bắt chuyện. Nếu bạn nhìn ngược lại, bạn đã từ chối bắt chuyện với 900 người (khoảng 90% người bạn gặp). Và vì thế, bạn không trông mong cả 100 người bạn làm phiền sẽ níu lại chia sẻ với thật lâu với bạn. Không, chỉ 10 người sẽ làm điều đó và 90 người sẽ từ chối bạn (90%). &lt;/p&gt;
-&lt;p&gt;Bạn có quyền từ chối người khác, và thực tế là bạn đang từ chối bắt chuyện với hơn 900 người trong số 1000 người bạn gặp mỗi ngày. Và vì thế, người khác cũng vậy. Việc ngại bị từ chối và không bao giờ chủ động kết nối với ai sẽ làm cửa sổ cơ hội của một người bị thu hẹp lại. Khi một người đưa ra đủ nhiều offer bất kể đó là gì và nhận lại đủ nhiều sự từ chối, họ sẽ từng bước điều chỉnh lại offer cho phù hợp và theo thời gian - tỉ lệ bị từ chối ngày càng giảm đi. Bởi vì họ ngày càng thấu hiểu và nhận định chính xác hơn những gì mà phần đa mọi người quan tâm và thực sự cần. &lt;/p&gt;
+&lt;p&gt;Bạn có quyền từ chối người khác, và thực tế là bạn đang từ chối bắt chuyện với hơn 900 người trong số 1000 người bạn gặp mỗi ngày. Và vì thế, người khác cũng vậy. Việc ngại bị từ chối và không bao giờ chủ động kết nối với ai sẽ làm cửa sổ cơ hội của một người bị thu hẹp lại. Khi một người đưa ra đủ nhiều offer bất kể đó là gì và nhận lại đủ nhiều sự từ chối, họ sẽ từng bước điều chỉnh lại offer cho phù hợp và theo thời gian, tỉ lệ bị từ chối ngày càng giảm đi. Bởi vì họ ngày càng thấu hiểu và nhận định chính xác hơn những gì mà phần đa mọi người quan tâm và thực sự cần. &lt;/p&gt;
 &lt;p&gt;Thực ra bạn nhận được bao nhiêu email mỗi ngày thì nên gửi đi bấy nhiêu email. Người ta có nhiều lý do để không trả lời mail của bạn giữa hàng trăm email khác trong hộp thư. Không sao cả, kể cả khi không nhận lại được hồi âm, bạn vẫn có thể gửi mail follow-up nếu cần thiết. Khi người ta cảm thấy offer đưa ra là phù hợp, họ sẽ trả lời. &lt;/p&gt;
-&lt;p&gt;Tương tự, khi người ta đã quyết định đưa số điện thoại hoặc card cho bạn, có nghĩa là người ta cho phép bạn gọi điện làm phiền họ một chút - hoặc nhiều chút nếu như những gì bạn mang đến cho họ làm cho họ cảm thấy hay và cần phải nghe tiếp. Và lúc đó đã không còn là làm phiền nữa mà là đó là một phần giá trị mà bạn đã mang đến trong cuộc đời của người khác.&lt;/p&gt;
-&lt;p&gt;Và một lần nữa, tư bản không thể xuất hiện bên ngoài lưu thông. Lý do mà một người luôn chịu thiệt thòi luôn đến từ sự bất cân xứng thông tin. Sự bất cân xứng thông tin sẽ chỉ luôn mang lại lợi thế cho người có được sự đối xứng về thông tin đó. Chỉ có kết nối và thực sự lắng nghe từ nhiều người mới giúp một người giải quyết bài toán đó. Bạn luôn phải mua mắc vì bạn không biết ở đâu bán rẻ hơn. Bạn phải chấp nhận đồng lương thấp vì bạn không biết ở đâu sẵn sàng trả cho bạn con số cao hơn. Bạn buộc phải nghe và tin cái câu "ở đâu cũng thế thôi" chỉ vì bạn hoàn toàn mù mờ về chỗ khác. Bạn buộc phải tin vào câu "ai mà chả thế" là bởi vì bạn chưa có cơ hội được kết nối và tiếp xúc với những người khác. Và vì thế, thành công của người trẻ đến từ khả năng dám chấp nhận bị từ chối để mở rộng kết nối!&lt;/p&gt;
+&lt;p&gt;Tương tự, khi người ta đã quyết định đưa số điện thoại hoặc card cho bạn, có nghĩa là người ta cho phép bạn gọi điện làm phiền họ một chút - hoặc nhiều chút nếu như những gì bạn mang đến cho họ làm cho họ cảm thấy hay và cần phải nghe tiếp. Và lúc đó đã không còn là làm phiền nữa mà là đó là một phần giá trị bạn đã mang đến trong cuộc đời của người khác.&lt;/p&gt;
+&lt;p&gt;Và một lần nữa, tư bản không thể xuất hiện bên ngoài lưu thông. Lý do mà một người chịu thiệt thòi luôn đến từ sự bất cân xứng thông tin. Sự bất cân xứng thông tin sẽ chỉ luôn mang lại lợi thế cho người có được sự đối xứng về thông tin đó. Chỉ có kết nối và thực sự lắng nghe từ nhiều người mới giúp một người giải quyết bài toán đó. Bạn luôn phải mua mắc vì bạn không biết ở đâu bán rẻ hơn. Bạn phải chấp nhận đồng lương thấp vì bạn không biết ở đâu sẵn sàng trả cho bạn con số cao hơn. Bạn buộc phải nghe và tin cái câu "ở đâu cũng thế thôi" chỉ vì bạn hoàn toàn mù mờ về chỗ khác. Bạn buộc phải tin vào câu "ai mà chả thế" là bởi vì bạn chưa có cơ hội được kết nối và tiếp xúc với những người khác. Và vì thế, thành công của người trẻ đến từ khả năng dám chấp nhận bị từ chối để mở rộng kết nối!&lt;/p&gt;
 &lt;h2 id="thanh-cong-cua-mot-nguoi-khi-ve-gia-nam-o-chat-luong-danh-ba"&gt;Thành công của một người khi về già nằm ở chất lượng danh bạ&lt;/h2&gt;
 &lt;p&gt;Sẽ đến một lúc nào đó, khả năng thử lại hay tạo dựng một mối quan hệ mới ngày càng giảm sút. Bởi vì lúc này, người đó không còn tuổi trẻ, không còn nhiều thời gian và nguồn lực. Có lẽ lúc này, người đó chỉ muốn rằng một cuộc gọi hoặc một tin nhắn của mình sẽ khiến cho những người thân - không cần biết là đang ở đâu - không cần biết là cuộc sống mưu sinh hiện tại như nào - đều tụ họp và ăn một bữa cơm. Tiền bạc không phải là tất cả nhưng nó quả thực là công cụ hiệu quả để làm điều đó trở nên dễ dàng hơn bao giờ hết. &lt;/p&gt;
 &lt;p&gt;Vì vậy, có lẽ lúc này người đó chỉ muốn một cuộc gọi của mình có thể giải quyết được mọi vấn đề. Gọi cho người có khả năng giải quyết vấn đề đó, và họ bắt máy. Họ lưu danh bạ của người đó ở chế độ ưu tiên cao kể cả khi người đó đã không còn quyền lực hay khả năng như lúc còn trẻ. Họ gửi lời hỏi thăm bản thân người đó và con cháu người đó.  &lt;/p&gt;

</xml_diff>